<commit_message>
Add latest identity and EGO content
</commit_message>
<xml_diff>
--- a/CharacterTable.xlsx
+++ b/CharacterTable.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CharacterData" sheetId="1" r:id="Raa64c6d83e4f405f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillData" sheetId="2" r:id="Re4b8fa462af14784"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DeckData" sheetId="3" r:id="R7809c7a7fd5a402d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DeckInfo" sheetId="4" r:id="R6d32776ca29b4a5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="추천덱" sheetId="5" r:id="R5f4605b27ce64ae2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="참조" sheetId="6" r:id="R13b5b8b3480b4007"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EGOData" sheetId="7" r:id="R007a22d2fed84510"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EGOGiftData" sheetId="8" r:id="Rf7e2d8c8ece34773"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CharacterData" sheetId="1" r:id="Ra817f330410b4a46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SkillData" sheetId="2" r:id="R7e315aff346f4629"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DeckData" sheetId="3" r:id="Rc411a3894e25416c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DeckInfo" sheetId="4" r:id="R411857e8b0924813"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="추천덱" sheetId="5" r:id="Re74c132714b04c4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="참조" sheetId="6" r:id="R8dd004a6c086484f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EGOData" sheetId="7" r:id="R8f6e07d6280d476b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EGOGiftData" sheetId="8" r:id="R04c059260150484f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9088,6 +9088,55 @@
         <x:v>46289</x:v>
       </x:c>
     </x:row>
+    <x:row r="190">
+      <x:c r="A190" t="str">
+        <x:v>10315</x:v>
+      </x:c>
+      <x:c r="B190" t="str">
+        <x:v>돈키호테</x:v>
+      </x:c>
+      <x:c r="C190" t="str">
+        <x:v>오트쿠튀르::르누아르 브랜드 매니저 돈키호테</x:v>
+      </x:c>
+      <x:c r="D190" t="str">
+        <x:v>★★★</x:v>
+      </x:c>
+      <x:c r="E190" t="str">
+        <x:v>르누아르</x:v>
+      </x:c>
+      <x:c r="F190" t="str">
+        <x:v>시지프</x:v>
+      </x:c>
+      <x:c r="G190" t="str"/>
+      <x:c r="H190" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I190" t="str">
+        <x:v>시즌</x:v>
+      </x:c>
+      <x:c r="J190" t="str">
+        <x:v>충전</x:v>
+      </x:c>
+      <x:c r="K190" t="str">
+        <x:v>진동</x:v>
+      </x:c>
+      <x:c r="L190" t="str"/>
+      <x:c r="M190" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N190" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="O190" t="str">
+        <x:v>./images/identities/10315_normal.webp</x:v>
+      </x:c>
+      <x:c r="P190" t="str">
+        <x:v>./images/identities/10315_awaken.webp</x:v>
+      </x:c>
+      <x:c r="Q190" s="2" t="n">
+        <x:v>46296</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -16839,6 +16888,47 @@
         <x:v>./images/skills/10917_skill3.webp</x:v>
       </x:c>
     </x:row>
+    <x:row r="190">
+      <x:c r="A190" t="str">
+        <x:v>10315</x:v>
+      </x:c>
+      <x:c r="B190" t="str">
+        <x:v>못 박히라</x:v>
+      </x:c>
+      <x:c r="C190" t="str">
+        <x:v>오만</x:v>
+      </x:c>
+      <x:c r="D190" t="str">
+        <x:v>타격</x:v>
+      </x:c>
+      <x:c r="E190" t="str">
+        <x:v>./images/skills/10315_skill1.webp</x:v>
+      </x:c>
+      <x:c r="F190" t="str">
+        <x:v>못 생기라</x:v>
+      </x:c>
+      <x:c r="G190" t="str">
+        <x:v>질투</x:v>
+      </x:c>
+      <x:c r="H190" t="str">
+        <x:v>타격</x:v>
+      </x:c>
+      <x:c r="I190" t="str">
+        <x:v>./images/skills/10315_skill2.webp</x:v>
+      </x:c>
+      <x:c r="J190" t="str">
+        <x:v>탄생을 끊으리라!</x:v>
+      </x:c>
+      <x:c r="K190" t="str">
+        <x:v>나태</x:v>
+      </x:c>
+      <x:c r="L190" t="str">
+        <x:v>타격</x:v>
+      </x:c>
+      <x:c r="M190" t="str">
+        <x:v>./images/skills/10315_skill3.webp</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -30039,6 +30129,52 @@
       </x:c>
       <x:c r="G114" t="str">
         <x:v>./images/ego/129.webp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" t="str">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="B115" t="str">
+        <x:v>구멍</x:v>
+      </x:c>
+      <x:c r="C115" t="str">
+        <x:v>파우스트</x:v>
+      </x:c>
+      <x:c r="D115" t="str">
+        <x:v>WAW</x:v>
+      </x:c>
+      <x:c r="E115" t="str">
+        <x:v>오만</x:v>
+      </x:c>
+      <x:c r="F115" t="str">
+        <x:v>우울 x2, 오만 x4, 질투 x2</x:v>
+      </x:c>
+      <x:c r="G115" t="str">
+        <x:v>./images/ego/130.webp</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" t="str">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="B116" t="str">
+        <x:v>구멍</x:v>
+      </x:c>
+      <x:c r="C116" t="str">
+        <x:v>뫼르소</x:v>
+      </x:c>
+      <x:c r="D116" t="str">
+        <x:v>WAW</x:v>
+      </x:c>
+      <x:c r="E116" t="str">
+        <x:v>오만</x:v>
+      </x:c>
+      <x:c r="F116" t="str">
+        <x:v>나태 x2, 우울 x2, 오만 x4, 질투 x4</x:v>
+      </x:c>
+      <x:c r="G116" t="str">
+        <x:v>./images/ego/131.webp</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Lock sinner hint and add EGO skill effect clues
The sinner, grade and sin hints alone identified 105 of 115 EGOs, so
the sinner hint now unlocks only after two guesses. In its place, the
awakening skill effect is revealed line by line as a paid clue, with
the EGO name always masked and the sinner/sin masked until their hints
are opened.

Adds scripts/fetch-ego-effects.js, which fills only the 효과 column of
the EGOData sheet from limbusdeck.com, and carries the field through
build-egos.js.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CharacterTable.xlsx
+++ b/CharacterTable.xlsx
@@ -72,9 +72,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -127,14 +126,74 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
-        <a:ea typeface="Calibri Light"/>
-        <a:cs typeface="Calibri Light"/>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -186,7 +245,7 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -195,13 +254,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -235,6 +294,17 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -289,6 +359,47 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -392,7 +503,7 @@
       <c r="P2" t="str">
         <v>./images/identities/10101_awaken.png</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2">
         <v>44984</v>
       </c>
     </row>
@@ -439,7 +550,7 @@
       <c r="P3" t="str">
         <v>./images/identities/10102_awaken.png</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3">
         <v>44984</v>
       </c>
     </row>
@@ -486,7 +597,7 @@
       <c r="P4" t="str">
         <v>./images/identities/10103_awaken.png</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4">
         <v>44984</v>
       </c>
     </row>
@@ -533,7 +644,7 @@
       <c r="P5" t="str">
         <v>./images/identities/10104_awaken.png</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5">
         <v>45092</v>
       </c>
     </row>
@@ -580,7 +691,7 @@
       <c r="P6" t="str">
         <v>./images/identities/10105_awaken.png</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6">
         <v>45189</v>
       </c>
     </row>
@@ -630,7 +741,7 @@
       <c r="P7" t="str">
         <v>./images/identities/10106_awaken.png</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7">
         <v>45239</v>
       </c>
     </row>
@@ -680,7 +791,7 @@
       <c r="P8" t="str">
         <v>./images/identities/10107_awaken.png</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8">
         <v>45267</v>
       </c>
     </row>
@@ -727,7 +838,7 @@
       <c r="P9" t="str">
         <v>./images/identities/10108_awaken.png</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9">
         <v>45316</v>
       </c>
     </row>
@@ -774,7 +885,7 @@
       <c r="P10" t="str">
         <v>./images/identities/10109_awaken.png</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10">
         <v>45428</v>
       </c>
     </row>
@@ -821,7 +932,7 @@
       <c r="P11" t="str">
         <v>./images/identities/10110_awaken.png</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11">
         <v>45540</v>
       </c>
     </row>
@@ -868,7 +979,7 @@
       <c r="P12" t="str">
         <v>./images/identities/10111_awaken.png</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12">
         <v>45680</v>
       </c>
     </row>
@@ -915,7 +1026,7 @@
       <c r="P13" t="str">
         <v>./images/identities/10112_awaken.png</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13">
         <v>45708</v>
       </c>
     </row>
@@ -965,7 +1076,7 @@
       <c r="P14" t="str">
         <v>./images/identities/10113_awaken.png</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14">
         <v>45841</v>
       </c>
     </row>
@@ -1015,7 +1126,7 @@
       <c r="P15" t="str">
         <v>./images/identities/10114_awaken.png</v>
       </c>
-      <c r="Q15" s="1">
+      <c r="Q15">
         <v>45897</v>
       </c>
     </row>
@@ -1065,7 +1176,7 @@
       <c r="P16" t="str">
         <v>./images/identities/10115_awaken.png</v>
       </c>
-      <c r="Q16" s="1">
+      <c r="Q16">
         <v>46072</v>
       </c>
     </row>
@@ -1115,7 +1226,7 @@
       <c r="P17" t="str">
         <v>./images/identities/10116_awaken.png</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17">
         <v>46239</v>
       </c>
     </row>
@@ -1159,7 +1270,7 @@
       <c r="P18" t="str">
         <v>./images/identities/10201_awaken.png</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18">
         <v>44984</v>
       </c>
     </row>
@@ -1206,7 +1317,7 @@
       <c r="P19" t="str">
         <v>./images/identities/10202_awaken.png</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19">
         <v>44984</v>
       </c>
     </row>
@@ -1256,7 +1367,7 @@
       <c r="P20" t="str">
         <v>./images/identities/10203_awaken.png</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20">
         <v>44984</v>
       </c>
     </row>
@@ -1303,7 +1414,7 @@
       <c r="P21" t="str">
         <v>./images/identities/10204_awaken.png</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21">
         <v>45008</v>
       </c>
     </row>
@@ -1347,7 +1458,7 @@
       <c r="P22" t="str">
         <v>./images/identities/10205_awaken.png</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22">
         <v>45148</v>
       </c>
     </row>
@@ -1394,7 +1505,7 @@
       <c r="P23" t="str">
         <v>./images/identities/10206_awaken.png</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23">
         <v>45176</v>
       </c>
     </row>
@@ -1441,7 +1552,7 @@
       <c r="P24" t="str">
         <v>./images/identities/10207_awaken.png</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24">
         <v>45225</v>
       </c>
     </row>
@@ -1488,7 +1599,7 @@
       <c r="P25" t="str">
         <v>./images/identities/10208_awaken.png</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25">
         <v>45344</v>
       </c>
     </row>
@@ -1535,7 +1646,7 @@
       <c r="P26" t="str">
         <v>./images/identities/10209_awaken.png</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26">
         <v>45386</v>
       </c>
     </row>
@@ -1582,7 +1693,7 @@
       <c r="P27" t="str">
         <v>./images/identities/10210_awaken.png</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27">
         <v>45512</v>
       </c>
     </row>
@@ -1629,7 +1740,7 @@
       <c r="P28" t="str">
         <v>./images/identities/10211_awaken.png</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28">
         <v>45680</v>
       </c>
     </row>
@@ -1676,7 +1787,7 @@
       <c r="P29" t="str">
         <v>./images/identities/10212_awaken.png</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29">
         <v>45799</v>
       </c>
     </row>
@@ -1726,7 +1837,7 @@
       <c r="P30" t="str">
         <v>./images/identities/10213_awaken.png</v>
       </c>
-      <c r="Q30" s="1">
+      <c r="Q30">
         <v>45939</v>
       </c>
     </row>
@@ -1776,7 +1887,7 @@
       <c r="P31" t="str">
         <v>./images/identities/10214_awaken.png</v>
       </c>
-      <c r="Q31" s="1">
+      <c r="Q31">
         <v>46022</v>
       </c>
     </row>
@@ -1826,7 +1937,7 @@
       <c r="P32" t="str">
         <v>./images/identities/10215_awaken.png</v>
       </c>
-      <c r="Q32" s="1">
+      <c r="Q32">
         <v>46114</v>
       </c>
     </row>
@@ -1876,7 +1987,7 @@
       <c r="P33" t="str">
         <v>./images/identities/10216_awaken.png</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33">
         <v>46212</v>
       </c>
     </row>
@@ -1923,7 +2034,7 @@
       <c r="P34" t="str">
         <v>./images/identities/10301_awaken.png</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34">
         <v>44984</v>
       </c>
     </row>
@@ -1973,7 +2084,7 @@
       <c r="P35" t="str">
         <v>./images/identities/10302_awaken.png</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35">
         <v>44984</v>
       </c>
     </row>
@@ -2020,7 +2131,7 @@
       <c r="P36" t="str">
         <v>./images/identities/10303_awaken.png</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36">
         <v>44984</v>
       </c>
     </row>
@@ -2067,7 +2178,7 @@
       <c r="P37" t="str">
         <v>./images/identities/10304_awaken.png</v>
       </c>
-      <c r="Q37" s="1">
+      <c r="Q37">
         <v>45050</v>
       </c>
     </row>
@@ -2111,7 +2222,7 @@
       <c r="P38" t="str">
         <v>./images/identities/10305_awaken.png</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38">
         <v>45127</v>
       </c>
     </row>
@@ -2158,7 +2269,7 @@
       <c r="P39" t="str">
         <v>./images/identities/10306_awaken.png</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39">
         <v>45253</v>
       </c>
     </row>
@@ -2205,7 +2316,7 @@
       <c r="P40" t="str">
         <v>./images/identities/10307_awaken.png</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40">
         <v>45302</v>
       </c>
     </row>
@@ -2252,7 +2363,7 @@
       <c r="P41" t="str">
         <v>./images/identities/10308_awaken.png</v>
       </c>
-      <c r="Q41" s="1">
+      <c r="Q41">
         <v>45344</v>
       </c>
     </row>
@@ -2299,7 +2410,7 @@
       <c r="P42" t="str">
         <v>./images/identities/10309_awaken.png</v>
       </c>
-      <c r="Q42" s="1">
+      <c r="Q42">
         <v>45470</v>
       </c>
     </row>
@@ -2346,7 +2457,7 @@
       <c r="P43" t="str">
         <v>./images/identities/10310_awaken.png</v>
       </c>
-      <c r="Q43" s="1">
+      <c r="Q43">
         <v>45638</v>
       </c>
     </row>
@@ -2396,7 +2507,7 @@
       <c r="P44" t="str">
         <v>./images/identities/10311_awaken.png</v>
       </c>
-      <c r="Q44" s="1">
+      <c r="Q44">
         <v>45722</v>
       </c>
     </row>
@@ -2446,7 +2557,7 @@
       <c r="P45" t="str">
         <v>./images/identities/10312_awaken.png</v>
       </c>
-      <c r="Q45" s="1">
+      <c r="Q45">
         <v>45855</v>
       </c>
     </row>
@@ -2496,7 +2607,7 @@
       <c r="P46" t="str">
         <v>./images/identities/10313_awaken.png</v>
       </c>
-      <c r="Q46" s="1">
+      <c r="Q46">
         <v>45981</v>
       </c>
     </row>
@@ -2546,7 +2657,7 @@
       <c r="P47" t="str">
         <v>./images/identities/10314_awaken.png</v>
       </c>
-      <c r="Q47" s="1">
+      <c r="Q47">
         <v>46030</v>
       </c>
     </row>
@@ -2593,7 +2704,7 @@
       <c r="P48" t="str">
         <v>./images/identities/10401_awaken.png</v>
       </c>
-      <c r="Q48" s="1">
+      <c r="Q48">
         <v>44984</v>
       </c>
     </row>
@@ -2640,7 +2751,7 @@
       <c r="P49" t="str">
         <v>./images/identities/10402_awaken.png</v>
       </c>
-      <c r="Q49" s="1">
+      <c r="Q49">
         <v>44984</v>
       </c>
     </row>
@@ -2687,7 +2798,7 @@
       <c r="P50" t="str">
         <v>./images/identities/10403_awaken.png</v>
       </c>
-      <c r="Q50" s="1">
+      <c r="Q50">
         <v>44984</v>
       </c>
     </row>
@@ -2734,7 +2845,7 @@
       <c r="P51" t="str">
         <v>./images/identities/10404_awaken.png</v>
       </c>
-      <c r="Q51" s="1">
+      <c r="Q51">
         <v>45036</v>
       </c>
     </row>
@@ -2781,7 +2892,7 @@
       <c r="P52" t="str">
         <v>./images/identities/10405_awaken.png</v>
       </c>
-      <c r="Q52" s="1">
+      <c r="Q52">
         <v>45162</v>
       </c>
     </row>
@@ -2834,7 +2945,7 @@
       <c r="P53" t="str">
         <v>./images/identities/10406_awaken.png</v>
       </c>
-      <c r="Q53" s="1">
+      <c r="Q53">
         <v>45246</v>
       </c>
     </row>
@@ -2881,7 +2992,7 @@
       <c r="P54" t="str">
         <v>./images/identities/10407_awaken.png</v>
       </c>
-      <c r="Q54" s="1">
+      <c r="Q54">
         <v>45358</v>
       </c>
     </row>
@@ -2928,7 +3039,7 @@
       <c r="P55" t="str">
         <v>./images/identities/10408_awaken.png</v>
       </c>
-      <c r="Q55" s="1">
+      <c r="Q55">
         <v>45400</v>
       </c>
     </row>
@@ -2975,7 +3086,7 @@
       <c r="P56" t="str">
         <v>./images/identities/10409_awaken.png</v>
       </c>
-      <c r="Q56" s="1">
+      <c r="Q56">
         <v>45456</v>
       </c>
     </row>
@@ -3025,7 +3136,7 @@
       <c r="P57" t="str">
         <v>./images/identities/10410_awaken.png</v>
       </c>
-      <c r="Q57" s="1">
+      <c r="Q57">
         <v>45540</v>
       </c>
     </row>
@@ -3072,7 +3183,7 @@
       <c r="P58" t="str">
         <v>./images/identities/10411_awaken.png</v>
       </c>
-      <c r="Q58" s="1">
+      <c r="Q58">
         <v>45736</v>
       </c>
     </row>
@@ -3122,7 +3233,7 @@
       <c r="P59" t="str">
         <v>./images/identities/10412_awaken.png</v>
       </c>
-      <c r="Q59" s="1">
+      <c r="Q59">
         <v>45911</v>
       </c>
     </row>
@@ -3172,7 +3283,7 @@
       <c r="P60" t="str">
         <v>./images/identities/10413_awaken.png</v>
       </c>
-      <c r="Q60" s="1">
+      <c r="Q60">
         <v>45995</v>
       </c>
     </row>
@@ -3222,7 +3333,7 @@
       <c r="P61" t="str">
         <v>./images/identities/10414_awaken.png</v>
       </c>
-      <c r="Q61" s="1">
+      <c r="Q61">
         <v>46086</v>
       </c>
     </row>
@@ -3275,7 +3386,7 @@
       <c r="P62" t="str">
         <v>./images/identities/10415_awaken.png</v>
       </c>
-      <c r="Q62" s="1">
+      <c r="Q62">
         <v>46156</v>
       </c>
     </row>
@@ -3322,7 +3433,7 @@
       <c r="P63" t="str">
         <v>./images/identities/10501_awaken.png</v>
       </c>
-      <c r="Q63" s="1">
+      <c r="Q63">
         <v>44984</v>
       </c>
     </row>
@@ -3369,7 +3480,7 @@
       <c r="P64" t="str">
         <v>./images/identities/10502_awaken.png</v>
       </c>
-      <c r="Q64" s="1">
+      <c r="Q64">
         <v>44984</v>
       </c>
     </row>
@@ -3419,7 +3530,7 @@
       <c r="P65" t="str">
         <v>./images/identities/10503_awaken.png</v>
       </c>
-      <c r="Q65" s="1">
+      <c r="Q65">
         <v>44984</v>
       </c>
     </row>
@@ -3463,7 +3574,7 @@
       <c r="P66" t="str">
         <v>./images/identities/10504_awaken.png</v>
       </c>
-      <c r="Q66" s="1">
+      <c r="Q66">
         <v>44994</v>
       </c>
     </row>
@@ -3513,7 +3624,7 @@
       <c r="P67" t="str">
         <v>./images/identities/10505_awaken.png</v>
       </c>
-      <c r="Q67" s="1">
+      <c r="Q67">
         <v>45078</v>
       </c>
     </row>
@@ -3563,7 +3674,7 @@
       <c r="P68" t="str">
         <v>./images/identities/10506_awaken.png</v>
       </c>
-      <c r="Q68" s="1">
+      <c r="Q68">
         <v>45120</v>
       </c>
     </row>
@@ -3610,7 +3721,7 @@
       <c r="P69" t="str">
         <v>./images/identities/10507_awaken.png</v>
       </c>
-      <c r="Q69" s="1">
+      <c r="Q69">
         <v>45253</v>
       </c>
     </row>
@@ -3657,7 +3768,7 @@
       <c r="P70" t="str">
         <v>./images/identities/10508_awaken.png</v>
       </c>
-      <c r="Q70" s="1">
+      <c r="Q70">
         <v>45344</v>
       </c>
     </row>
@@ -3704,7 +3815,7 @@
       <c r="P71" t="str">
         <v>./images/identities/10509_awaken.png</v>
       </c>
-      <c r="Q71" s="1">
+      <c r="Q71">
         <v>45379</v>
       </c>
     </row>
@@ -3751,7 +3862,7 @@
       <c r="P72" t="str">
         <v>./images/identities/10510_awaken.png</v>
       </c>
-      <c r="Q72" s="1">
+      <c r="Q72">
         <v>45484</v>
       </c>
     </row>
@@ -3801,7 +3912,7 @@
       <c r="P73" t="str">
         <v>./images/identities/10511_awaken.png</v>
       </c>
-      <c r="Q73" s="1">
+      <c r="Q73">
         <v>45575</v>
       </c>
     </row>
@@ -3851,7 +3962,7 @@
       <c r="P74" t="str">
         <v>./images/identities/10512_awaken.png</v>
       </c>
-      <c r="Q74" s="1">
+      <c r="Q74">
         <v>45827</v>
       </c>
     </row>
@@ -3901,7 +4012,7 @@
       <c r="P75" t="str">
         <v>./images/identities/10513_awaken.png</v>
       </c>
-      <c r="Q75" s="1">
+      <c r="Q75">
         <v>45960</v>
       </c>
     </row>
@@ -3951,7 +4062,7 @@
       <c r="P76" t="str">
         <v>./images/identities/10514_awaken.png</v>
       </c>
-      <c r="Q76" s="1">
+      <c r="Q76">
         <v>46086</v>
       </c>
     </row>
@@ -4001,7 +4112,7 @@
       <c r="P77" t="str">
         <v>./images/identities/10515_awaken.png</v>
       </c>
-      <c r="Q77" s="1">
+      <c r="Q77">
         <v>46128</v>
       </c>
     </row>
@@ -4051,7 +4162,7 @@
       <c r="P78" t="str">
         <v>./images/identities/10601_awaken.png</v>
       </c>
-      <c r="Q78" s="1">
+      <c r="Q78">
         <v>44984</v>
       </c>
     </row>
@@ -4098,7 +4209,7 @@
       <c r="P79" t="str">
         <v>./images/identities/10602_awaken.png</v>
       </c>
-      <c r="Q79" s="1">
+      <c r="Q79">
         <v>44984</v>
       </c>
     </row>
@@ -4145,7 +4256,7 @@
       <c r="P80" t="str">
         <v>./images/identities/10603_awaken.png</v>
       </c>
-      <c r="Q80" s="1">
+      <c r="Q80">
         <v>44984</v>
       </c>
     </row>
@@ -4192,7 +4303,7 @@
       <c r="P81" t="str">
         <v>./images/identities/10604_awaken.png</v>
       </c>
-      <c r="Q81" s="1">
+      <c r="Q81">
         <v>45022</v>
       </c>
     </row>
@@ -4239,7 +4350,7 @@
       <c r="P82" t="str">
         <v>./images/identities/10605_awaken.png</v>
       </c>
-      <c r="Q82" s="1">
+      <c r="Q82">
         <v>45106</v>
       </c>
     </row>
@@ -4289,7 +4400,7 @@
       <c r="P83" t="str">
         <v>./images/identities/10606_awaken.png</v>
       </c>
-      <c r="Q83" s="1">
+      <c r="Q83">
         <v>45162</v>
       </c>
     </row>
@@ -4336,7 +4447,7 @@
       <c r="P84" t="str">
         <v>./images/identities/10607_awaken.png</v>
       </c>
-      <c r="Q84" s="1">
+      <c r="Q84">
         <v>45225</v>
       </c>
     </row>
@@ -4383,7 +4494,7 @@
       <c r="P85" t="str">
         <v>./images/identities/10608_awaken.png</v>
       </c>
-      <c r="Q85" s="1">
+      <c r="Q85">
         <v>45316</v>
       </c>
     </row>
@@ -4430,7 +4541,7 @@
       <c r="P86" t="str">
         <v>./images/identities/10609_awaken.png</v>
       </c>
-      <c r="Q86" s="1">
+      <c r="Q86">
         <v>45456</v>
       </c>
     </row>
@@ -4477,7 +4588,7 @@
       <c r="P87" t="str">
         <v>./images/identities/10610_awaken.png</v>
       </c>
-      <c r="Q87" s="1">
+      <c r="Q87">
         <v>45582</v>
       </c>
     </row>
@@ -4524,7 +4635,7 @@
       <c r="P88" t="str">
         <v>./images/identities/10611_awaken.png</v>
       </c>
-      <c r="Q88" s="1">
+      <c r="Q88">
         <v>45666</v>
       </c>
     </row>
@@ -4574,7 +4685,7 @@
       <c r="P89" t="str">
         <v>./images/identities/10612_awaken.png</v>
       </c>
-      <c r="Q89" s="1">
+      <c r="Q89">
         <v>45777</v>
       </c>
     </row>
@@ -4624,7 +4735,7 @@
       <c r="P90" t="str">
         <v>./images/identities/10613_awaken.png</v>
       </c>
-      <c r="Q90" s="1">
+      <c r="Q90">
         <v>45883</v>
       </c>
     </row>
@@ -4674,7 +4785,7 @@
       <c r="P91" t="str">
         <v>./images/identities/10614_awaken.png</v>
       </c>
-      <c r="Q91" s="1">
+      <c r="Q91">
         <v>46114</v>
       </c>
     </row>
@@ -4724,7 +4835,7 @@
       <c r="P92" t="str">
         <v>./images/identities/10615_awaken.png</v>
       </c>
-      <c r="Q92" s="1">
+      <c r="Q92">
         <v>46184</v>
       </c>
     </row>
@@ -4774,7 +4885,7 @@
       <c r="P93" t="str">
         <v>./images/identities/10616_awaken.png</v>
       </c>
-      <c r="Q93" s="1">
+      <c r="Q93">
         <v>46254</v>
       </c>
     </row>
@@ -4821,7 +4932,7 @@
       <c r="P94" t="str">
         <v>./images/identities/10701_awaken.png</v>
       </c>
-      <c r="Q94" s="1">
+      <c r="Q94">
         <v>44984</v>
       </c>
     </row>
@@ -4868,7 +4979,7 @@
       <c r="P95" t="str">
         <v>./images/identities/10702_awaken.png</v>
       </c>
-      <c r="Q95" s="1">
+      <c r="Q95">
         <v>44984</v>
       </c>
     </row>
@@ -4921,7 +5032,7 @@
       <c r="P96" t="str">
         <v>./images/identities/10703_awaken.png</v>
       </c>
-      <c r="Q96" s="1">
+      <c r="Q96">
         <v>44984</v>
       </c>
     </row>
@@ -4968,7 +5079,7 @@
       <c r="P97" t="str">
         <v>./images/identities/10704_awaken.png</v>
       </c>
-      <c r="Q97" s="1">
+      <c r="Q97">
         <v>45008</v>
       </c>
     </row>
@@ -5021,7 +5132,7 @@
       <c r="P98" t="str">
         <v>./images/identities/10705_awaken.png</v>
       </c>
-      <c r="Q98" s="1">
+      <c r="Q98">
         <v>45085</v>
       </c>
     </row>
@@ -5068,7 +5179,7 @@
       <c r="P99" t="str">
         <v>./images/identities/10706_awaken.png</v>
       </c>
-      <c r="Q99" s="1">
+      <c r="Q99">
         <v>45176</v>
       </c>
     </row>
@@ -5118,7 +5229,7 @@
       <c r="P100" t="str">
         <v>./images/identities/10707_awaken.png</v>
       </c>
-      <c r="Q100" s="1">
+      <c r="Q100">
         <v>45267</v>
       </c>
     </row>
@@ -5165,7 +5276,7 @@
       <c r="P101" t="str">
         <v>./images/identities/10708_awaken.png</v>
       </c>
-      <c r="Q101" s="1">
+      <c r="Q101">
         <v>45372</v>
       </c>
     </row>
@@ -5212,7 +5323,7 @@
       <c r="P102" t="str">
         <v>./images/identities/10709_awaken.png</v>
       </c>
-      <c r="Q102" s="1">
+      <c r="Q102">
         <v>45512</v>
       </c>
     </row>
@@ -5259,7 +5370,7 @@
       <c r="P103" t="str">
         <v>./images/identities/10710_awaken.png</v>
       </c>
-      <c r="Q103" s="1">
+      <c r="Q103">
         <v>45526</v>
       </c>
     </row>
@@ -5306,7 +5417,7 @@
       <c r="P104" t="str">
         <v>./images/identities/10711_awaken.png</v>
       </c>
-      <c r="Q104" s="1">
+      <c r="Q104">
         <v>45666</v>
       </c>
     </row>
@@ -5353,7 +5464,7 @@
       <c r="P105" t="str">
         <v>./images/identities/10712_awaken.png</v>
       </c>
-      <c r="Q105" s="1">
+      <c r="Q105">
         <v>45694</v>
       </c>
     </row>
@@ -5403,7 +5514,7 @@
       <c r="P106" t="str">
         <v>./images/identities/10713_awaken.png</v>
       </c>
-      <c r="Q106" s="1">
+      <c r="Q106">
         <v>45953</v>
       </c>
     </row>
@@ -5453,7 +5564,7 @@
       <c r="P107" t="str">
         <v>./images/identities/10714_awaken.png</v>
       </c>
-      <c r="Q107" s="1">
+      <c r="Q107">
         <v>45981</v>
       </c>
     </row>
@@ -5503,7 +5614,7 @@
       <c r="P108" t="str">
         <v>./images/identities/10715_awaken.png</v>
       </c>
-      <c r="Q108" s="1">
+      <c r="Q108">
         <v>46142</v>
       </c>
     </row>
@@ -5553,7 +5664,7 @@
       <c r="P109" t="str">
         <v>./images/identities/10716_awaken.png</v>
       </c>
-      <c r="Q109" s="1">
+      <c r="Q109">
         <v>46198</v>
       </c>
     </row>
@@ -5600,7 +5711,7 @@
       <c r="P110" t="str">
         <v>./images/identities/10801_awaken.png</v>
       </c>
-      <c r="Q110" s="1">
+      <c r="Q110">
         <v>44984</v>
       </c>
     </row>
@@ -5650,7 +5761,7 @@
       <c r="P111" t="str">
         <v>./images/identities/10802_awaken.png</v>
       </c>
-      <c r="Q111" s="1">
+      <c r="Q111">
         <v>44984</v>
       </c>
     </row>
@@ -5697,7 +5808,7 @@
       <c r="P112" t="str">
         <v>./images/identities/10803_awaken.png</v>
       </c>
-      <c r="Q112" s="1">
+      <c r="Q112">
         <v>44984</v>
       </c>
     </row>
@@ -5747,7 +5858,7 @@
       <c r="P113" t="str">
         <v>./images/identities/10804_awaken.png</v>
       </c>
-      <c r="Q113" s="1">
+      <c r="Q113">
         <v>44984</v>
       </c>
     </row>
@@ -5797,7 +5908,7 @@
       <c r="P114" t="str">
         <v>./images/identities/10805_awaken.png</v>
       </c>
-      <c r="Q114" s="1">
+      <c r="Q114">
         <v>45092</v>
       </c>
     </row>
@@ -5844,7 +5955,7 @@
       <c r="P115" t="str">
         <v>./images/identities/10806_awaken.png</v>
       </c>
-      <c r="Q115" s="1">
+      <c r="Q115">
         <v>45113</v>
       </c>
     </row>
@@ -5894,7 +6005,7 @@
       <c r="P116" t="str">
         <v>./images/identities/10807_awaken.png</v>
       </c>
-      <c r="Q116" s="1">
+      <c r="Q116">
         <v>45134</v>
       </c>
     </row>
@@ -5947,7 +6058,7 @@
       <c r="P117" t="str">
         <v>./images/identities/10808_awaken.png</v>
       </c>
-      <c r="Q117" s="1">
+      <c r="Q117">
         <v>45330</v>
       </c>
     </row>
@@ -5997,7 +6108,7 @@
       <c r="P118" t="str">
         <v>./images/identities/10809_awaken.png</v>
       </c>
-      <c r="Q118" s="1">
+      <c r="Q118">
         <v>45400</v>
       </c>
     </row>
@@ -6044,7 +6155,7 @@
       <c r="P119" t="str">
         <v>./images/identities/10810_awaken.png</v>
       </c>
-      <c r="Q119" s="1">
+      <c r="Q119">
         <v>45568</v>
       </c>
     </row>
@@ -6091,7 +6202,7 @@
       <c r="P120" t="str">
         <v>./images/identities/10811_awaken.png</v>
       </c>
-      <c r="Q120" s="1">
+      <c r="Q120">
         <v>45694</v>
       </c>
     </row>
@@ -6141,7 +6252,7 @@
       <c r="P121" t="str">
         <v>./images/identities/10812_awaken.png</v>
       </c>
-      <c r="Q121" s="1">
+      <c r="Q121">
         <v>45813</v>
       </c>
     </row>
@@ -6191,7 +6302,7 @@
       <c r="P122" t="str">
         <v>./images/identities/10813_awaken.png</v>
       </c>
-      <c r="Q122" s="1">
+      <c r="Q122">
         <v>45967</v>
       </c>
     </row>
@@ -6241,7 +6352,7 @@
       <c r="P123" t="str">
         <v>./images/identities/10814_awaken.png</v>
       </c>
-      <c r="Q123" s="1">
+      <c r="Q123">
         <v>46044</v>
       </c>
     </row>
@@ -6291,7 +6402,7 @@
       <c r="P124" t="str">
         <v>./images/identities/10815_awaken.png</v>
       </c>
-      <c r="Q124" s="1">
+      <c r="Q124">
         <v>46184</v>
       </c>
     </row>
@@ -6338,7 +6449,7 @@
       <c r="P125" t="str">
         <v>./images/identities/10901_awaken.png</v>
       </c>
-      <c r="Q125" s="1">
+      <c r="Q125">
         <v>44984</v>
       </c>
     </row>
@@ -6388,7 +6499,7 @@
       <c r="P126" t="str">
         <v>./images/identities/10902_awaken.png</v>
       </c>
-      <c r="Q126" s="1">
+      <c r="Q126">
         <v>44984</v>
       </c>
     </row>
@@ -6432,7 +6543,7 @@
       <c r="P127" t="str">
         <v>./images/identities/10903_awaken.png</v>
       </c>
-      <c r="Q127" s="1">
+      <c r="Q127">
         <v>44984</v>
       </c>
     </row>
@@ -6479,7 +6590,7 @@
       <c r="P128" t="str">
         <v>./images/identities/10904_awaken.png</v>
       </c>
-      <c r="Q128" s="1">
+      <c r="Q128">
         <v>44994</v>
       </c>
     </row>
@@ -6529,7 +6640,7 @@
       <c r="P129" t="str">
         <v>./images/identities/10905_awaken.png</v>
       </c>
-      <c r="Q129" s="1">
+      <c r="Q129">
         <v>45078</v>
       </c>
     </row>
@@ -6576,7 +6687,7 @@
       <c r="P130" t="str">
         <v>./images/identities/10906_awaken.png</v>
       </c>
-      <c r="Q130" s="1">
+      <c r="Q130">
         <v>45120</v>
       </c>
     </row>
@@ -6623,7 +6734,7 @@
       <c r="P131" t="str">
         <v>./images/identities/10907_awaken.png</v>
       </c>
-      <c r="Q131" s="1">
+      <c r="Q131">
         <v>45190</v>
       </c>
     </row>
@@ -6670,7 +6781,7 @@
       <c r="P132" t="str">
         <v>./images/identities/10908_awaken.png</v>
       </c>
-      <c r="Q132" s="1">
+      <c r="Q132">
         <v>45358</v>
       </c>
     </row>
@@ -6717,7 +6828,7 @@
       <c r="P133" t="str">
         <v>./images/identities/10909_awaken.png</v>
       </c>
-      <c r="Q133" s="1">
+      <c r="Q133">
         <v>45470</v>
       </c>
     </row>
@@ -6764,7 +6875,7 @@
       <c r="P134" t="str">
         <v>./images/identities/10910_awaken.png</v>
       </c>
-      <c r="Q134" s="1">
+      <c r="Q134">
         <v>45554</v>
       </c>
     </row>
@@ -6814,7 +6925,7 @@
       <c r="P135" t="str">
         <v>./images/identities/10911_awaken.png</v>
       </c>
-      <c r="Q135" s="1">
+      <c r="Q135">
         <v>45610</v>
       </c>
     </row>
@@ -6864,7 +6975,7 @@
       <c r="P136" t="str">
         <v>./images/identities/10912_awaken.png</v>
       </c>
-      <c r="Q136" s="1">
+      <c r="Q136">
         <v>45792</v>
       </c>
     </row>
@@ -6914,7 +7025,7 @@
       <c r="P137" t="str">
         <v>./images/identities/10913_awaken.png</v>
       </c>
-      <c r="Q137" s="1">
+      <c r="Q137">
         <v>45855</v>
       </c>
     </row>
@@ -6964,7 +7075,7 @@
       <c r="P138" t="str">
         <v>./images/identities/10914_awaken.png</v>
       </c>
-      <c r="Q138" s="1">
+      <c r="Q138">
         <v>46009</v>
       </c>
     </row>
@@ -7014,7 +7125,7 @@
       <c r="P139" t="str">
         <v>./images/identities/10915_awaken.png</v>
       </c>
-      <c r="Q139" s="1">
+      <c r="Q139">
         <v>46128</v>
       </c>
     </row>
@@ -7064,7 +7175,7 @@
       <c r="P140" t="str">
         <v>./images/identities/10916_awaken.png</v>
       </c>
-      <c r="Q140" s="1">
+      <c r="Q140">
         <v>46198</v>
       </c>
     </row>
@@ -7111,7 +7222,7 @@
       <c r="P141" t="str">
         <v>./images/identities/11001_awaken.png</v>
       </c>
-      <c r="Q141" s="1">
+      <c r="Q141">
         <v>44984</v>
       </c>
     </row>
@@ -7161,7 +7272,7 @@
       <c r="P142" t="str">
         <v>./images/identities/11002_awaken.png</v>
       </c>
-      <c r="Q142" s="1">
+      <c r="Q142">
         <v>44984</v>
       </c>
     </row>
@@ -7208,7 +7319,7 @@
       <c r="P143" t="str">
         <v>./images/identities/11003_awaken.png</v>
       </c>
-      <c r="Q143" s="1">
+      <c r="Q143">
         <v>44984</v>
       </c>
     </row>
@@ -7258,7 +7369,7 @@
       <c r="P144" t="str">
         <v>./images/identities/11004_awaken.png</v>
       </c>
-      <c r="Q144" s="1">
+      <c r="Q144">
         <v>44984</v>
       </c>
     </row>
@@ -7308,7 +7419,7 @@
       <c r="P145" t="str">
         <v>./images/identities/11005_awaken.png</v>
       </c>
-      <c r="Q145" s="1">
+      <c r="Q145">
         <v>45050</v>
       </c>
     </row>
@@ -7355,7 +7466,7 @@
       <c r="P146" t="str">
         <v>./images/identities/11006_awaken.png</v>
       </c>
-      <c r="Q146" s="1">
+      <c r="Q146">
         <v>45106</v>
       </c>
     </row>
@@ -7402,7 +7513,7 @@
       <c r="P147" t="str">
         <v>./images/identities/11007_awaken.png</v>
       </c>
-      <c r="Q147" s="1">
+      <c r="Q147">
         <v>45134</v>
       </c>
     </row>
@@ -7449,7 +7560,7 @@
       <c r="P148" t="str">
         <v>./images/identities/11008_awaken.png</v>
       </c>
-      <c r="Q148" s="1">
+      <c r="Q148">
         <v>45281</v>
       </c>
     </row>
@@ -7496,7 +7607,7 @@
       <c r="P149" t="str">
         <v>./images/identities/11009_awaken.png</v>
       </c>
-      <c r="Q149" s="1">
+      <c r="Q149">
         <v>45414</v>
       </c>
     </row>
@@ -7543,7 +7654,7 @@
       <c r="P150" t="str">
         <v>./images/identities/11010_awaken.png</v>
       </c>
-      <c r="Q150" s="1">
+      <c r="Q150">
         <v>45575</v>
       </c>
     </row>
@@ -7590,7 +7701,7 @@
       <c r="P151" t="str">
         <v>./images/identities/11011_awaken.png</v>
       </c>
-      <c r="Q151" s="1">
+      <c r="Q151">
         <v>45624</v>
       </c>
     </row>
@@ -7637,7 +7748,7 @@
       <c r="P152" t="str">
         <v>./images/identities/11012_awaken.png</v>
       </c>
-      <c r="Q152" s="1">
+      <c r="Q152">
         <v>45750</v>
       </c>
     </row>
@@ -7687,7 +7798,7 @@
       <c r="P153" t="str">
         <v>./images/identities/11013_awaken.png</v>
       </c>
-      <c r="Q153" s="1">
+      <c r="Q153">
         <v>45827</v>
       </c>
     </row>
@@ -7737,7 +7848,7 @@
       <c r="P154" t="str">
         <v>./images/identities/11014_awaken.png</v>
       </c>
-      <c r="Q154" s="1">
+      <c r="Q154">
         <v>45897</v>
       </c>
     </row>
@@ -7787,7 +7898,7 @@
       <c r="P155" t="str">
         <v>./images/identities/11015_awaken.png</v>
       </c>
-      <c r="Q155" s="1">
+      <c r="Q155">
         <v>46058</v>
       </c>
     </row>
@@ -7834,7 +7945,7 @@
       <c r="P156" t="str">
         <v>./images/identities/11101_awaken.png</v>
       </c>
-      <c r="Q156" s="1">
+      <c r="Q156">
         <v>44984</v>
       </c>
     </row>
@@ -7881,7 +7992,7 @@
       <c r="P157" t="str">
         <v>./images/identities/11102_awaken.png</v>
       </c>
-      <c r="Q157" s="1">
+      <c r="Q157">
         <v>44984</v>
       </c>
     </row>
@@ -7928,7 +8039,7 @@
       <c r="P158" t="str">
         <v>./images/identities/11103_awaken.png</v>
       </c>
-      <c r="Q158" s="1">
+      <c r="Q158">
         <v>44984</v>
       </c>
     </row>
@@ -7975,7 +8086,7 @@
       <c r="P159" t="str">
         <v>./images/identities/11104_awaken.png</v>
       </c>
-      <c r="Q159" s="1">
+      <c r="Q159">
         <v>45022</v>
       </c>
     </row>
@@ -8022,7 +8133,7 @@
       <c r="P160" t="str">
         <v>./images/identities/11105_awaken.png</v>
       </c>
-      <c r="Q160" s="1">
+      <c r="Q160">
         <v>45203</v>
       </c>
     </row>
@@ -8069,7 +8180,7 @@
       <c r="P161" t="str">
         <v>./images/identities/11106_awaken.png</v>
       </c>
-      <c r="Q161" s="1">
+      <c r="Q161">
         <v>45281</v>
       </c>
     </row>
@@ -8116,7 +8227,7 @@
       <c r="P162" t="str">
         <v>./images/identities/11107_awaken.png</v>
       </c>
-      <c r="Q162" s="1">
+      <c r="Q162">
         <v>45302</v>
       </c>
     </row>
@@ -8163,7 +8274,7 @@
       <c r="P163" t="str">
         <v>./images/identities/11108_awaken.png</v>
       </c>
-      <c r="Q163" s="1">
+      <c r="Q163">
         <v>45379</v>
       </c>
     </row>
@@ -8210,7 +8321,7 @@
       <c r="P164" t="str">
         <v>./images/identities/11109_awaken.png</v>
       </c>
-      <c r="Q164" s="1">
+      <c r="Q164">
         <v>45428</v>
       </c>
     </row>
@@ -8260,7 +8371,7 @@
       <c r="P165" t="str">
         <v>./images/identities/11110_awaken.png</v>
       </c>
-      <c r="Q165" s="1">
+      <c r="Q165">
         <v>45498</v>
       </c>
     </row>
@@ -8307,7 +8418,7 @@
       <c r="P166" t="str">
         <v>./images/identities/11111_awaken.png</v>
       </c>
-      <c r="Q166" s="1">
+      <c r="Q166">
         <v>45582</v>
       </c>
     </row>
@@ -8354,7 +8465,7 @@
       <c r="P167" t="str">
         <v>./images/identities/11112_awaken.png</v>
       </c>
-      <c r="Q167" s="1">
+      <c r="Q167">
         <v>45736</v>
       </c>
     </row>
@@ -8401,7 +8512,7 @@
       <c r="P168" t="str">
         <v>./images/identities/11113_awaken.png</v>
       </c>
-      <c r="Q168" s="1">
+      <c r="Q168">
         <v>45869</v>
       </c>
     </row>
@@ -8451,7 +8562,7 @@
       <c r="P169" t="str">
         <v>./images/identities/11114_awaken.png</v>
       </c>
-      <c r="Q169" s="1">
+      <c r="Q169">
         <v>46022</v>
       </c>
     </row>
@@ -8501,7 +8612,7 @@
       <c r="P170" t="str">
         <v>./images/identities/11115_awaken.png</v>
       </c>
-      <c r="Q170" s="1">
+      <c r="Q170">
         <v>46170</v>
       </c>
     </row>
@@ -8548,7 +8659,7 @@
       <c r="P171" t="str">
         <v>./images/identities/11201_awaken.png</v>
       </c>
-      <c r="Q171" s="1">
+      <c r="Q171">
         <v>44984</v>
       </c>
     </row>
@@ -8595,7 +8706,7 @@
       <c r="P172" t="str">
         <v>./images/identities/11202_awaken.png</v>
       </c>
-      <c r="Q172" s="1">
+      <c r="Q172">
         <v>44984</v>
       </c>
     </row>
@@ -8642,7 +8753,7 @@
       <c r="P173" t="str">
         <v>./images/identities/11203_awaken.png</v>
       </c>
-      <c r="Q173" s="1">
+      <c r="Q173">
         <v>44984</v>
       </c>
     </row>
@@ -8689,7 +8800,7 @@
       <c r="P174" t="str">
         <v>./images/identities/11204_awaken.png</v>
       </c>
-      <c r="Q174" s="1">
+      <c r="Q174">
         <v>45036</v>
       </c>
     </row>
@@ -8742,7 +8853,7 @@
       <c r="P175" t="str">
         <v>./images/identities/11205_awaken.png</v>
       </c>
-      <c r="Q175" s="1">
+      <c r="Q175">
         <v>45085</v>
       </c>
     </row>
@@ -8786,7 +8897,7 @@
       <c r="P176" t="str">
         <v>./images/identities/11206_awaken.png</v>
       </c>
-      <c r="Q176" s="1">
+      <c r="Q176">
         <v>45148</v>
       </c>
     </row>
@@ -8836,7 +8947,7 @@
       <c r="P177" t="str">
         <v>./images/identities/11207_awaken.png</v>
       </c>
-      <c r="Q177" s="1">
+      <c r="Q177">
         <v>45246</v>
       </c>
     </row>
@@ -8883,7 +8994,7 @@
       <c r="P178" t="str">
         <v>./images/identities/11208_awaken.png</v>
       </c>
-      <c r="Q178" s="1">
+      <c r="Q178">
         <v>45344</v>
       </c>
     </row>
@@ -8930,7 +9041,7 @@
       <c r="P179" t="str">
         <v>./images/identities/11209_awaken.png</v>
       </c>
-      <c r="Q179" s="1">
+      <c r="Q179">
         <v>45386</v>
       </c>
     </row>
@@ -8980,7 +9091,7 @@
       <c r="P180" t="str">
         <v>./images/identities/11210_awaken.png</v>
       </c>
-      <c r="Q180" s="1">
+      <c r="Q180">
         <v>45596</v>
       </c>
     </row>
@@ -9027,7 +9138,7 @@
       <c r="P181" t="str">
         <v>./images/identities/11211_awaken.png</v>
       </c>
-      <c r="Q181" s="1">
+      <c r="Q181">
         <v>45722</v>
       </c>
     </row>
@@ -9077,7 +9188,7 @@
       <c r="P182" t="str">
         <v>./images/identities/11212_awaken.png</v>
       </c>
-      <c r="Q182" s="1">
+      <c r="Q182">
         <v>45792</v>
       </c>
     </row>
@@ -9127,7 +9238,7 @@
       <c r="P183" t="str">
         <v>./images/identities/11213_awaken.png</v>
       </c>
-      <c r="Q183" s="1">
+      <c r="Q183">
         <v>45967</v>
       </c>
     </row>
@@ -9177,7 +9288,7 @@
       <c r="P184" t="str">
         <v>./images/identities/11214_awaken.png</v>
       </c>
-      <c r="Q184" s="1">
+      <c r="Q184">
         <v>46058</v>
       </c>
     </row>
@@ -9227,7 +9338,7 @@
       <c r="P185" t="str">
         <v>./images/identities/11215_awaken.png</v>
       </c>
-      <c r="Q185" s="1">
+      <c r="Q185">
         <v>46100</v>
       </c>
     </row>
@@ -9277,7 +9388,7 @@
       <c r="P186" t="str">
         <v>./images/identities/11216_awaken.png</v>
       </c>
-      <c r="Q186" s="1">
+      <c r="Q186">
         <v>46212</v>
       </c>
     </row>
@@ -9324,10 +9435,10 @@
       <c r="O187" t="str">
         <v>./images/identities/10416_normal.png</v>
       </c>
-      <c r="P187" s="1" t="str">
+      <c r="P187" t="str">
         <v>./images/identities/10416_awaken.png</v>
       </c>
-      <c r="Q187" s="1">
+      <c r="Q187">
         <v>46282</v>
       </c>
     </row>
@@ -9374,10 +9485,10 @@
       <c r="O188" t="str">
         <v>./images/identities/10816_normal.png</v>
       </c>
-      <c r="P188" s="1" t="str">
+      <c r="P188" t="str">
         <v>./images/identities/10816_awaken.png</v>
       </c>
-      <c r="Q188" s="1">
+      <c r="Q188">
         <v>46282</v>
       </c>
     </row>
@@ -9427,7 +9538,7 @@
       <c r="P189" t="str">
         <v>./images/identities/10917_awaken.webp</v>
       </c>
-      <c r="Q189" s="1">
+      <c r="Q189">
         <v>46289</v>
       </c>
     </row>
@@ -9480,7 +9591,7 @@
       <c r="P190" t="str">
         <v>./images/identities/10315_awaken.webp</v>
       </c>
-      <c r="Q190" s="1">
+      <c r="Q190">
         <v>46296</v>
       </c>
     </row>
@@ -9533,7 +9644,7 @@
       <c r="P191" t="str">
         <v>./images/identities/11016_awaken.webp</v>
       </c>
-      <c r="Q191" s="1">
+      <c r="Q191">
         <v>46310</v>
       </c>
     </row>
@@ -27978,7 +28089,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G116"/>
+  <dimension ref="A1:H116"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -28000,10 +28111,13 @@
         <v>자원</v>
       </c>
       <c r="G1" t="str">
+        <v>효과</v>
+      </c>
+      <c r="H1" t="str">
         <v>아이콘</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2">
         <v>127</v>
       </c>
@@ -28022,11 +28136,19 @@
       <c r="F2" t="str">
         <v>질투 x5</v>
       </c>
-      <c r="G2" t="str">
+      <c r="G2" t="str" xml:space="preserve">
+        <v xml:space="preserve">[합 승리 후 공격 종료 시] 현재 체력 비율이 가장 낮은 아군 (2 + 질투 공명 수 / 2)명의 체력을 각자의 최대 체력 6%만큼 회복하고 정신력 5 회복 (최대 4명)
+[합 패배] (질투 공명 수 × 5)만큼 보호막 얻음 (최대 30)
+[합 패배] 메인 타겟에게 가하는 피해량 +200%
+코인 1: 파괴 불가 코인
+코인 1: [합 승리 후 적중시] 다음 턴에 위력 감소 1 부여 (대상 별 턴당 1회)
+코인 1: [적중시] 출혈 4 부여</v>
+      </c>
+      <c r="H2" t="str">
         <v>./images/ego/127.png</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" xml:space="preserve">
       <c r="A3">
         <v>126</v>
       </c>
@@ -28045,11 +28167,43 @@
       <c r="F3" t="str">
         <v>나태 x1, 우울 x4, 오만 x2</v>
       </c>
-      <c r="G3" t="str">
+      <c r="G3" t="str" xml:space="preserve">
+        <v xml:space="preserve">광역 난사
+이 스킬의 효과로 무작위 나비 부여시 앞면이 나올 확률로 죽은나비를 부여. 부여하지 않은 경우, 산나비를 부여. (나비 1당 개별 판정)
+메인 타겟의 침잠과 모든 나비의 합 4당, 합 위력 +1 (최대 4)
+로보토미 E.G.O::엄숙한 애도 이상이면,
+-
+[공격 시작 전] (우울 공명 수 + 1)만큼 무작위 산나비·죽은나비를 얻음 (최대 7)
+-
+[공격 종료시] 재장전
+코인 1: 파괴 불가 코인
+코인 1: [적중시] 무작위 나비 1 부여
+코인 1: [적중시] 침잠 횟수 1 증가
+코인 2: 파괴 불가 코인
+코인 2: [적중시] 무작위 나비 2 부여
+코인 2: [적중시] 침잠 횟수 1 증가
+코인 3: 파괴 불가 코인
+코인 3: [적중시] 무작위 나비 2 부여
+코인 3: [적중시] 침잠 횟수 1 증가
+코인 4: 파괴 불가 코인
+코인 4: [적중시] 무작위 나비 3 부여
+코인 4: [적중시] 침잠 횟수 1 증가
+코인 4: [적중시] 이번 턴과 다음 턴에 우울 취약 1, 우울 내성 약화 1 부여
+코인 5: 파괴 불가 코인
+코인 5: 보유한 산나비·죽은나비 전부 소모
+코인 5: [적중시] 침잠 3 부여
+코인 5: [적중시] 진동 3 부여
+코인 5: [적중시] 나비(산나비) 2 부여
+코인 5: [적중시] 나비(죽은나비) 2 부여
+코인 5: [적중시] 진동 폭발. 진동 횟수 1 감소
+코인 5: [적중시] 대상의 모든 나비만큼 우울 피해
+코인 5: [적중시] 이 코인 최종 피해량의 (이 코인에서 소모한 산나비·죽은나비 × 2)%만큼 우울 피해</v>
+      </c>
+      <c r="H3" t="str">
         <v>./images/ego/126.webp</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" xml:space="preserve">
       <c r="A4">
         <v>125</v>
       </c>
@@ -28068,11 +28222,24 @@
       <c r="F4" t="str">
         <v>분노 x1, 오만 x4, 질투 x1</v>
       </c>
-      <c r="G4" t="str">
+      <c r="G4" t="str" xml:space="preserve">
+        <v xml:space="preserve">전투에서 처음 사용 시 정신력 소모량 15 감소
+- 검계 우두머리 뫼르소면, 필요한 E.G.O 자원이 분노 1, 오만 1, 질투 1 감소
+자신의 호흡 4당, 합 위력 +1, 피해량 +6% (각각 최대 8, 30%)
+이번 전투에서 추모주를 얻었으면, 메인 타겟에게 가하는 피해량 +100%
+- 검계 우두머리 뫼르소면, 해당 효과가 피해량 +200%로 적용
+[공격 시작 전] (최대 공명 수/2)만큼 공격 가중치 증가 (최대 2, 소수점 버림)
+[공격 시작 전] 편성 순서가 가장 빠른 아군 (3 + 최대 공명 수)명의 호흡 횟수 4 증가
+[공격 종료시] 자신을 제외한 정신력이 가장 낮은 검계 소속 인격 4명의 정신력 10 회복
+[공격 종료시] 다음 턴에 추모주 4 얻음
+코인 1: [적중시] 출혈 4 부여
+코인 2: [적중시] 출혈 횟수 2 증가</v>
+      </c>
+      <c r="H4" t="str">
         <v>./images/ego/125.webp</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" xml:space="preserve">
       <c r="A5">
         <v>124</v>
       </c>
@@ -28091,11 +28258,20 @@
       <c r="F5" t="str">
         <v>분노 x2, 색욕 x3</v>
       </c>
-      <c r="G5" t="str">
+      <c r="G5" t="str" xml:space="preserve">
+        <v xml:space="preserve">[사용시] 모든 대상의 화상과 출혈의 합 6당 합 위력 +1 (최대 2)
+[공격 종료시] 현재 체력 비율이 가장 낮은 아군 2명의 체력을 최대 체력의 10%만큼 회복하고 주홍 나방 2 부여 (최소 체력 회복량: 1)
+- (색욕 공명 수 - 1)만큼 회복 대상 수 증가 (최대 2명)
+- 회복 대상이 색욕 속성 스킬을 장착했으면, 정신력 6 회복
+코인 1: [적중시] 화상 3 부여
+코인 1: [적중시] 출혈 3 부여
+코인 1: [이 코인 공격 종료 시] 적중한 대상에게 다음 턴에 분노 취약 1, 색욕 취약 1 부여</v>
+      </c>
+      <c r="H5" t="str">
         <v>./images/ego/124.webp</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" xml:space="preserve">
       <c r="A6">
         <v>123</v>
       </c>
@@ -28114,11 +28290,20 @@
       <c r="F6" t="str">
         <v>분노 x3, 나태 x2, 오만 x2</v>
       </c>
-      <c r="G6" t="str">
+      <c r="G6" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 모든 공격 대상과 자신의 화상 위력의 합 10당 최종 위력 +1 (최대 2)
+[공격 종료시] 화상 10 얻음, 자신의 화상 횟수 1 증가
+[공격 종료시] 자신의 화상이 15 이상이면, 다음 턴에 분노 피해량 증가 1 얻음 (턴당 1회)
+코인 1: [적중시] 화상 1 부여
+코인 1: [적중시] (분노 공명 수 / 2)만큼 화상 부여 (최대 3, 소수점 버림)
+코인 2: [적중시] (분노 공명 수 / 3)만큼 화상 횟수 증가 (최대 2, 소수점 버림)
+코인 2: [이 코인 공격 종료시] 자신의 화상이 15 이상이면, 모든 공격 대상에게 잔불 1 부여 (턴당 1회, 집중 전투인 경우 부위로 취급)</v>
+      </c>
+      <c r="H6" t="str">
         <v>./images/ego/123.webp</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" xml:space="preserve">
       <c r="A7">
         <v>122</v>
       </c>
@@ -28137,11 +28322,27 @@
       <c r="F7" t="str">
         <v>분노 x3, 색욕 x2, 나태 x1, 오만 x1, 질투 x1</v>
       </c>
-      <c r="G7" t="str">
+      <c r="G7" t="str" xml:space="preserve">
+        <v xml:space="preserve">메인 타겟의 출혈과 화상의 합 2당, 합 위력 +1 (최대 10)
+자신의 잃은 체력 비율만큼 피해량 증가 (최대 20%)
+서브 타겟에게 가하는 피해량 -50%
+[대상 처치시] 모든 아군이 다음 턴에 리듬 2 얻음 (스킬 당 1회)
+[공격 종료시] 자신을 제외한 정신력이 가장 낮은 아군 (1 + 최대 공명 수)명의 정신력 12 회복 (최대 4명)
+[공격 종료시] 2턴 동안 전투 종료 시 정신력 8 감소
+코인 1: [적중시] 출혈 2 부여
+코인 2: [적중시] 화상 2 부여
+코인 3: [앞면 적중시] 자신의 체력이 10% 이상이면, 4 ~ 8 만큼 체력 피해 입음 (코인당 1회)
+코인 3: - 이후 이 코인 재사용 (스킬당 최대 4회)
+코인 3: - 이 효과로 흐트러짐 상태가 되거나 체력이 1 미만으로 감소하지 않음
+코인 3: [적중시] 화상 1 부여
+코인 3: [적중시] 출혈 1 부여
+코인 3: [적중시] 무작위 아군 1명이 다음 턴에 리듬 1 ~ 3 얻음 (코인당 1회)</v>
+      </c>
+      <c r="H7" t="str">
         <v>./images/ego/122.webp</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" xml:space="preserve">
       <c r="A8">
         <v>121</v>
       </c>
@@ -28160,11 +28361,29 @@
       <c r="F8" t="str">
         <v>분노 x4, 색욕 x4, 오만 x4</v>
       </c>
-      <c r="G8" t="str">
+      <c r="G8" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 최대 공명 수만큼 호흡 얻음 (최대 7)
+[공격 시작 전] 자신의 호흡 횟수 3 증가
+[공격 종료시] 나생 [羅生] 1 얻음
+[공격 종료시] 3턴 동안 턴 종료 시 자신의 정신력 10 감소
+코인 1: 파괴 불가 코인
+코인 1: [적중시] 화상 2 부여
+코인 1: [적중시] 다음 턴에 속박 1 부여
+코인 2: 파괴 불가 코인
+코인 2: [적중시] 출혈 2 부여
+코인 2: [크리티컬 적중 시] 마지막 코인 위력 +5 (스킬 당 1회)
+코인 3: 파괴 불가 코인
+코인 3: 크리티컬 피해량 +30%
+코인 3: [코인 시작 시] (모든 대상의 화상 + 출혈 위력) 10당 피해량 +1% (최대 50%)
+코인 3: [코인 시작 시] (모든 대상의 화상 + 출혈 횟수) 10당 코인 위력 +1 (최대 5)
+코인 3: [코인 시작 시] 자신의 나생 [羅生] 을 모두 소모하고, 소모한 수치 5당 피해량 +1% (최대 198%)
+코인 3: - 공격 대상이 1명이면, 이 효과가 2배로 적용됨 (집중 전투인 경우, 본체를 기준으로 판정)</v>
+      </c>
+      <c r="H8" t="str">
         <v>./images/ego/121.webp</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" xml:space="preserve">
       <c r="A9">
         <v>120</v>
       </c>
@@ -28183,11 +28402,26 @@
       <c r="F9" t="str">
         <v>분노 x4, 우울 x2, 오만 x2, 질투 x4</v>
       </c>
-      <c r="G9" t="str">
+      <c r="G9" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 메인 대상의 화상과 침잠의 합이 10 이상이면, 코인 위력 +1
+[공격 시작 전] 최대 공명 수만큼 호흡 얻음 (최대 7)
+- 해당 공명이 완전 공명이면, (최대 공명 수) / 3만큼 추가로 호흡 횟수 증가 (최대 2, 소수점 버림)
+코인 1: 파괴 불가 코인
+코인 1: [적중시] 화상 2 부여
+코인 1: [적중시] 침잠 횟수 3 증가
+코인 2: 파괴 불가 코인
+코인 2: [파괴되지 않고 적중시] 이번 턴과 다음 턴에 깨어진 세계 1 부여
+코인 3: 파괴 불가 코인
+코인 3: [적중시] 대상의 (침잠/3)만큼 화상 부여 (최대 5, 소수점 버림)
+코인 3: [크리티컬 적중 시] 화상 횟수 1 증가
+코인 4: 파괴 불가 코인
+코인 4: [파괴되지 않고 적중시] 화상 1회 발동. 화상 횟수 1 감소</v>
+      </c>
+      <c r="H9" t="str">
         <v>./images/ego/120.webp</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" xml:space="preserve">
       <c r="A10">
         <v>119</v>
       </c>
@@ -28206,11 +28440,23 @@
       <c r="F10" t="str">
         <v>분노 x2, 탐식 x1, 질투 x3</v>
       </c>
-      <c r="G10" t="str">
+      <c r="G10" t="str" xml:space="preserve">
+        <v xml:space="preserve">메인 타겟의 화상 6당 코인 위력 +1 (최대 3)
+[공격 시작 전] (최대 공명 수 + 1)만큼 자신의 충전 횟수 증가 (최대 7)
+- 질투 공명이 4 이상이면, 대신 자신의 충전 횟수 7 증가
+[공격 시작 전] 자신의 충전 횟수를 모두 소모. 소모한 충전 횟수 1당, 피해량 +3% (최대 45%)
+- 충전 횟수를 5 이상 소모했다면, 기본 위력 +1
+코인 1: [적중시] 화상 2 부여
+코인 2: [적중시] 화상 2 부여
+코인 3: [적중시] 다음 턴에 속박 1 부여
+코인 3: [적중시] 주민등록 마이크로 칩 2 부여
+코인 3: [적중시] 자신의 충전 횟수 1~3 증가</v>
+      </c>
+      <c r="H10" t="str">
         <v>./images/ego/119.png</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" xml:space="preserve">
       <c r="A11">
         <v>118</v>
       </c>
@@ -28229,11 +28475,23 @@
       <c r="F11" t="str">
         <v>색욕 x1, 질투 x3</v>
       </c>
-      <c r="G11" t="str">
+      <c r="G11" t="str" xml:space="preserve">
+        <v xml:space="preserve">일방 공격 시 이 스킬의
+[파괴되지 않고 적중시] 효과가 발동하지 않음
+[합 승리시] 질투 공명 수만큼 질투 E.G.O 자원을 소모하고 소모한 자원 1당, 제일 적은 E.G.O 자원을 1씩 나누어 얻음 (최대 소모량 6)
+[합 패배] 최종 위력이 4 감소하는 대신 (질투 공명 수 × 5)만큼 보호막을 얻음 (최대 30)
+코인 1: 파괴 불가 코인
+코인 1: [파괴되지 않고 적중시] 현재 체력 비율이 가장 낮은 아군 2명의 체력을 각자 최대 체력의 10%만큼 회복 (스킬 당 1회)
+코인 1: - 자신을 제외한 질투 속성인 기본 공격 스킬을 보유하지 않은 아군은 회복 대상이 되지 않음
+코인 1: [적중시] 바늘 2 부여
+코인 1: [적중시] 저주 1 부여
+코인 1: [적중시] 못 1 부여</v>
+      </c>
+      <c r="H11" t="str">
         <v>./images/ego/118.webp</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" xml:space="preserve">
       <c r="A12">
         <v>117</v>
       </c>
@@ -28252,11 +28510,20 @@
       <c r="F12" t="str">
         <v>분노 x2, 나태 x3, 오만 x2</v>
       </c>
-      <c r="G12" t="str">
+      <c r="G12" t="str" xml:space="preserve">
+        <v xml:space="preserve">[합 불가능]
+전투에서 처음 사용시 필요한 E.G.O 자원이 분노 1, 나태 2, 오만 1 감소
+칼집 속 사람이 1 이상이면, 눈부시지 않은 영광 - 광휘(光輝)로 발동됨
+이 스킬은 적에게 적중하지 않고, 수비 스킬을 발동시키지 않으며, 외부 효과로 재사용이 불가능함
+[공격 종료시] 칼집 속 사람 1 얻음
+[공격 종료시] 정신력 25 회복
+[공격 종료시] 다음 턴에 공격 레벨 증가 2, 피해량 증가 1 얻음</v>
+      </c>
+      <c r="H12" t="str">
         <v>./images/ego/117.webp</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" xml:space="preserve">
       <c r="A13">
         <v>116</v>
       </c>
@@ -28275,11 +28542,22 @@
       <c r="F13" t="str">
         <v>나태 x1, 탐식 x5, 오만 x2</v>
       </c>
-      <c r="G13" t="str">
+      <c r="G13" t="str" xml:space="preserve">
+        <v xml:space="preserve">메인 타겟에게 화상 또는 파열이 있으면, 최종 위력 +3
+[공격 시작 전] 메인 타겟의 파열 위력과 파열 횟수의 합 1당 피해량 +1% (최대 25%)
+경화막이 있으면, 이 효과와 최댓값이 2배로 증가
+[공격 종료시] 경화막 10 얻음
+[공격 종료시] 자신과 현재 체력 비율이 가장 낮은 아군 1명의 체력을 자신의 최대 체력의 30%만큼 회복
+- 자신이 최대 체력일 경우, 대신 아군 2명의 체력 회복
+[공격 종료시] 자신을 포함하여 현재 정신력이 가장 낮은 아군 2명의 정신력 15 회복
+코인 1: [적중시] 파열 3 부여
+코인 1: [적중시] 화상 3 부여</v>
+      </c>
+      <c r="H13" t="str">
         <v>./images/ego/116.webp</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" xml:space="preserve">
       <c r="A14">
         <v>115</v>
       </c>
@@ -28298,11 +28576,23 @@
       <c r="F14" t="str">
         <v>나태 x1, 우울 x2, 오만 x4</v>
       </c>
-      <c r="G14" t="str">
+      <c r="G14" t="str" xml:space="preserve">
+        <v xml:space="preserve">[사용시] 호흡 4 얻음
+[공격 시작 전] 호흡 위력과 호흡 횟수의 합 5당, 최종 위력 +1 (최대 3)
+[공격 시작 전] 시엔징, 상급 시엔징이 없으면, 이 스킬에서 소모한 E.G.O 자원과 정신력을 절반만큼 돌려받음 (소수점 버림. 이 효과는 각성 스킬 사용 시 침식되는 경우에도 적용됨)
+[공격 시작 전] 시엔징이 있으면, 공격 가중치 +1, 피해량 +25%
+[공격 시작 전] 상급 시엔징이 있으면, 공격 가중치 +2, 피해량 +45%
+[공격 종료시] 시엔징 5 얻음
+- 시엔징 또는 상급 시엔징이 있으면, 전부 소모하고 상급 시엔징 5 얻음
+코인 2: 시엔징이 있으면, 크리티컬 피해량 +(호흡 위력)% (최대 20%)
+코인 2: 상급 시엔징이 있으면, 크리티컬 피해량 +(호흡 위력과 호흡 횟수의 합)% (최대 40%)
+코인 2: [적중시] 침잠 3 부여</v>
+      </c>
+      <c r="H14" t="str">
         <v>./images/ego/115.webp</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" xml:space="preserve">
       <c r="A15">
         <v>114</v>
       </c>
@@ -28321,11 +28611,27 @@
       <c r="F15" t="str">
         <v>우울 x4, 오만 x2</v>
       </c>
-      <c r="G15" t="str">
+      <c r="G15" t="str" xml:space="preserve">
+        <v xml:space="preserve">공격 대상이 1명이면, 코인 위력 +2, 피해량 +100% (집중 전투인 경우, 본체를 기준으로 판정)
+[사용시] 메인 타겟의 침잠 4 당 합 위력 +1 (최대 2)
+[공격 시작 전] 메인 타겟의 우울 내성이 1을 초과하면, 초과하는 값 0.1 당 피해량 +5% (최대 20%)
+[공격 시작 전] 우울 공명이 2 이상이면, 우울 공명 1 당 피해량 +10% (최대 40%)
+[공격 종료시] 공격 대상이 1명 이상 사망했으면, 무작위 적 일정 2명에게 (각 대상의 침잠 위력 / 2)만큼 우울 피해를 줌 (최대 15. 공격 대상이고, 침잠 위력을 많이 보유한 순으로 적용)
+코인 1: 파괴 불가 코인
+코인 1: [적중시] 침잠 3 부여
+코인 1: [적중시] 진동 3 부여
+코인 2: 파괴 불가 코인
+코인 2: [파괴되지 않고 적중시] 다음 턴에 속박 2 부여
+코인 3: 파괴 불가 코인
+코인 3: [적중시] 공격 대상 중 흐트러지거나 부위 파괴 또는 사망한 대상이 있으면, 공격 대상이 아닌 무작위 적 1명에게 침잠 2 부여 (턴당 1회, 집중 전투인 경우, 부위를 대상 1명으로 취급)
+코인 3: 공격 대상이 1명이면, 대신 3명에게 부여
+코인 3: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소</v>
+      </c>
+      <c r="H15" t="str">
         <v>./images/ego/114.webp</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" xml:space="preserve">
       <c r="A16">
         <v>103</v>
       </c>
@@ -28344,11 +28650,28 @@
       <c r="F16" t="str">
         <v>분노 x2, 색욕 x2, 나태 x6, 질투 x1</v>
       </c>
-      <c r="G16" t="str">
+      <c r="G16" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 메인 타겟의 (진동 위력 + 진동 횟수)가 30 이상이면 가중치 +1
+- 100 이상이면, 대신 가중치 +3
+[공격 시작 전] 최대 공명 수 2 당, 공격하는 모든 대상에게 진동 1 부여 (최대 3)
+[공격 종료시] 3턴 동안 턴 종료 시 정신력 10 감소
+[공격 종료시] 자신의 최대 체력의 (축적된 과거 × 2)% 만큼 체력 회복
+[공격 종료시] 홀수 턴에 (나태 공명 수)가 홀수거나, 짝수 턴에 (나태 공명 수)가 짝수면 정신력 10 회복
+코인 1: [적중시] 진동 횟수 2 증가
+코인 1: [적중시] (나태 공명 수 / 2)만큼 진동 횟수 증가 (최대 3)
+코인 1: [적중시] 메인 타겟이면, 대상의 현재 진동으로 진폭 얽힘
+코인 2: [적중시] 진동 4 부여
+코인 3: [코인 시작 시] 메인 타겟의 진동 위력 1당, 이 코인의 피해량 +1% (최대 50%)
+코인 4: [코인 시작 시] 메인 타겟의 (진동 위력 + 진동 횟수) 1당, 이 코인의 피해량 +1% (최대 100%)
+코인 4: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소
+코인 4: [적중시] 이 코인의 효과로 인한 피해량 증가량이 50% 이상이면, 진동 폭발 1회.
+코인 4: [적중시] 이 코인의 효과로 인한 피해량 증가량이 100% 이상이면, 진동 폭발 2회. 진동 횟수 2 감소</v>
+      </c>
+      <c r="H16" t="str">
         <v>./images/ego/103.webp</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" xml:space="preserve">
       <c r="A17">
         <v>102</v>
       </c>
@@ -28367,11 +28690,25 @@
       <c r="F17" t="str">
         <v>분노 x2, 우울 x2, 오만 x2, 질투 x6</v>
       </c>
-      <c r="G17" t="str">
+      <c r="G17" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 자신을 제외한 무작위 아군 1 + (질투 공명 수 / 2)명에게 마법소녀의 영창 1 부여 (최대 4명)
+- 자신에게 마법소녀 등장!이 있으면, 대신하여 무작위 아군 1 + (질투 공명 수 / 2)명에게 마법소녀의 영창 2 부여 (최대 4명)
+[공격 시작 전] (충전 - 1)만큼 공격 가중치 증가 (최대 5)
+- 자신에게 마법소녀 등장!이 있으면, 대신하여 충전만큼 공격 가중치 증가 (최대 5)
+[공격 종료시] 자신의 충전 횟수를 전부 소모하여 체력 비율이 가장 낮은 아군 2 + (질투 공명 수 / 2)명의 체력을 (소모한 충전 횟수)%만큼 회복 (최대 5명, 최대 10%)
+[공격 종료시] 로보토미 E.G.O::사랑과 증오의 이름으로 돈키호테이면, 매지컬 아르카나 1 얻음
+코인 1: 파괴 불가 코인
+코인 1: [적중시] 자신의 충전 횟수 2 증가 (턴 당 최대 10)
+코인 2: 파괴 불가 코인
+코인 2: [적중시] 다음 턴에 메인 타겟에게 악당 표식 부여
+코인 2: [적중시] 파열을 (충전 - 1)만큼 부여 (최대 4)
+코인 2: - 자신에게 마법소녀 등장!이 있으면, 파열 횟수 1 증가</v>
+      </c>
+      <c r="H17" t="str">
         <v>./images/ego/102.webp</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" xml:space="preserve">
       <c r="A18">
         <v>101</v>
       </c>
@@ -28390,11 +28727,18 @@
       <c r="F18" t="str">
         <v>탐식 x5, 우울 x1, 질투 x1</v>
       </c>
-      <c r="G18" t="str">
+      <c r="G18" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [합 불가능]
+코인 1: 대상 수비 스킬 무시
+코인 1: 이 스킬은 적에게 적중하지 않음
+코인 1: [공격 종료시] 매화첨 [埋花櫼] 얻음이 스킬의 최종 위력만큼 자신이 고정 피해를 받음
+코인 1: - 이 피해로 흐트러지거나 체력이 1 미만으로 감소하지 않음</v>
+      </c>
+      <c r="H18" t="str">
         <v>./images/ego/101.webp</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" xml:space="preserve">
       <c r="A19">
         <v>100</v>
       </c>
@@ -28413,11 +28757,24 @@
       <c r="F19" t="str">
         <v>색욕 x2, 탐식 x6, 오만 x2</v>
       </c>
-      <c r="G19" t="str">
+      <c r="G19" t="str" xml:space="preserve">
+        <v xml:space="preserve">자신의 매화침 [埋花針] 6 당 코인 위력 +1 (최대 3)
+[전투 시작시] 불허 [不許] 얻음
+[공격 시작 전] 탐식 공명 수만큼 매화침 [埋花針] 얻음 (최대 5)
+[공격 시작 전] (자신의 매화침 [埋花針] × 2)만큼 체력 피해 받음
+- 이 효과로 체력이 흐트러짐 구간 이하가 되면 흐트러지지 않고, 자신의 현재 체력보다 높은 흐트러짐 구간 제거
+[공격 종료시] 3턴 동안 턴 종료 시 정신력 10 감소
+코인 1: [적중시] 파열 횟수 1 증가
+코인 2: 자신의 잃은 체력 2%당 피해량 +1% (최대 40%)
+코인 2: [적중시] 파열 3 부여
+코인 2: [적중시] 자신의 현재 체력이 최대 체력의 30% 미만이거나, 매화침 [埋花針] 수치가 20이면 이 코인 재사용 (스킬 당 1회)
+코인 2: [재사용 적중시] 자신의 모든 체력을 소모하여 이 코인의 피해량 +20% (턴 당 1회)</v>
+      </c>
+      <c r="H19" t="str">
         <v>./images/ego/100.webp</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" xml:space="preserve">
       <c r="A20">
         <v>99</v>
       </c>
@@ -28436,11 +28793,17 @@
       <c r="F20" t="str">
         <v>나태 x2, 오만 x2</v>
       </c>
-      <c r="G20" t="str">
+      <c r="G20" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 종료시] 자신과 메인 타겟의 부정적인 효과 수의 합만큼 지네 독 부여 (최대 10)
+코인 1: [적중시] 침잠 2 부여
+코인 2: [적중시] 파열 2 부여
+코인 2: [적중시] 탐식 혹은 우울 공명이 4 이상이면, 해당 공명 수만큼 지네 독을 부여 (최대 5)</v>
+      </c>
+      <c r="H20" t="str">
         <v>./images/ego/99.webp</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" xml:space="preserve">
       <c r="A21">
         <v>98</v>
       </c>
@@ -28459,11 +28822,17 @@
       <c r="F21" t="str">
         <v>색욕 x1, 탐식 x5, 우울 x2, 오만 x1</v>
       </c>
-      <c r="G21" t="str">
+      <c r="G21" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 얽혀버린 저주 부적을 4 + (탐식 공명 수)만큼 부여함 (최대 10)
+코인 2: 얽혀버린 저주 부적 당 피해량 +5% (최대 50%)
+코인 2: [적중시] 파열을 (대상의 얽혀버린 저주 부적 / 2)만큼 부여 (최대 4, 소수점 버림)
+코인 2: [적중시] 파열 횟수를 (대상의 얽혀버린 저주 부적 / 4)만큼 부여 (최대 2, 소수점 버림)</v>
+      </c>
+      <c r="H21" t="str">
         <v>./images/ego/98.webp</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" xml:space="preserve">
       <c r="A22">
         <v>97</v>
       </c>
@@ -28482,11 +28851,18 @@
       <c r="F22" t="str">
         <v>분노 x7, 오만 x3</v>
       </c>
-      <c r="G22" t="str">
+      <c r="G22" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] (최대 공명 수 / 2)만큼 공격 가중치 증가 (최대 3, 소수점 버림)
+[공격 종료시] 현재 체력 비율이 가장 낮은 아군 (1 + 최대 공명 수)명의 체력을 최대 체력의 20%만큼 회복 (최대 3명)
+[공격 종료시] 3턴 동안 턴 종료 시 정신력 10 감소
+코인 1: [적중시] 화상 8 부여
+코인 1: [적중시] 메인 타겟이면, 다음 턴에 달궈진 새장 (1 + (분노 공명 수 / 3))만큼 부여 (최대 3, 소수점 버림)</v>
+      </c>
+      <c r="H22" t="str">
         <v>./images/ego/97.webp</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" xml:space="preserve">
       <c r="A23">
         <v>96</v>
       </c>
@@ -28505,11 +28881,16 @@
       <c r="F23" t="str">
         <v>나태 x1, 우울 x1, 오만 x5</v>
       </c>
-      <c r="G23" t="str">
+      <c r="G23" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 모든 아군에게 호흡 위력을 (최대 공명 수)만큼 부여 (최대 부여량 : 6)
+- 오만 공명 3 이상이면, 부여 대상의 호흡 횟수 1 증가, 부여 대상에게 다음 턴에 가쁜 날숨 1 부여
+코인 1: [적중시] 자신의 호흡 횟수 1 증가크리티컬 피해량 +(호흡 위력과 호흡 횟수의 합)% (최대 40%)</v>
+      </c>
+      <c r="H23" t="str">
         <v>./images/ego/96.webp</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" xml:space="preserve">
       <c r="A24">
         <v>95</v>
       </c>
@@ -28528,11 +28909,20 @@
       <c r="F24" t="str">
         <v>분노 x1, 색욕 x1, 오만 x5</v>
       </c>
-      <c r="G24" t="str">
+      <c r="G24" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 최대 공명 수만큼 호흡 얻음 (최대 6)
+- 호흡이 15 이상이면, 대신 최종 위력 + (최대 공명 수) (최대 6)
+[공격 시작 전] (최대 공명 수/2)만큼 호흡 횟수 증가 (최대 3)
+- 호흡 횟수가 5 이상이면, 대신 코인 위력 + (최대 공명 수/2) (최대 3)
+[대상 처치 시] 다음 턴에 깊은 들숨 2 얻음 (턴 당 최대 6)
+코인 2: 크리티컬 피해량 +(호흡 위력과 호흡 횟수의 합)% (최대 40%)
+코인 2: [적중시] 깊은 들숨 4 얻음 (턴 당 1회)</v>
+      </c>
+      <c r="H24" t="str">
         <v>./images/ego/95.webp</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" xml:space="preserve">
       <c r="A25">
         <v>94</v>
       </c>
@@ -28551,11 +28941,27 @@
       <c r="F25" t="str">
         <v>분노 x2, 색욕 x2, 오만 x4</v>
       </c>
-      <c r="G25" t="str">
+      <c r="G25" t="str" xml:space="preserve">
+        <v xml:space="preserve">대상의 화상 수치 3 당 피해량 +3% (최대 30%)
+[공격 시작 전] 마탄이 0이면, 마탄 1 얻음
+- 마탄 수치에 따라 발사할 탄환이 정해짐
+· 첫번째 마탄
+· 두번째 마탄
+· 세번째 마탄
+· 네번째 마탄
+· 다섯번째 마탄
+· 여섯번째 마탄
+· 일곱번째 마탄
+[공격 종료시] 최대 공명 수만큼 마탄을 얻음 (최소 1, 최대 4)
+[공격 종료시] 메인 타겟이 사망하면, 화상이 있는 모든 적에게 흑염 4 부여
+코인 1: [적중시] 마탄만큼 화상 부여
+코인 1: [적중시] 마탄만큼 흑염 부여 (턴 당 대상 1명마다 최대 1회 부여)</v>
+      </c>
+      <c r="H25" t="str">
         <v>./images/ego/94.webp</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" xml:space="preserve">
       <c r="A26">
         <v>93</v>
       </c>
@@ -28574,11 +28980,20 @@
       <c r="F26" t="str">
         <v>나태 x2, 탐식 x2, 우울 x2, 오만 x2</v>
       </c>
-      <c r="G26" t="str">
+      <c r="G26" t="str" xml:space="preserve">
+        <v xml:space="preserve">대상의 정신력이 0 미만이면, 0 미만의 정신력 1 당 피해량 +1% (최대 45%)
+[공격 종료시] 자신의 체력이 최대치면, 턴 종료 시 정신력을 15 회복하고 다음 턴에 공격 위력 증가 1 얻음
+코인 1: [적중시] 진동 5 부여
+코인 1: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소
+코인 2: [적중시] 자신이 잃은 체력의 (3 + 최대 공명 수)%만큼 회복 (스킬 당 최대 30%)
+코인 2: [적중시] 침잠 4 부여
+코인 2: [적중시] 대상이 흐트러짐, 사기 저하, 패닉 상태면 다음 턴에 공격 위력 감소 1, 가장 높은 공명 속성의 취약을 1 부여</v>
+      </c>
+      <c r="H26" t="str">
         <v>./images/ego/93.webp</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" xml:space="preserve">
       <c r="A27">
         <v>92</v>
       </c>
@@ -28597,11 +29012,20 @@
       <c r="F27" t="str">
         <v>나태 x4, 탐식 x1, 오만 x2</v>
       </c>
-      <c r="G27" t="str">
+      <c r="G27" t="str" xml:space="preserve">
+        <v xml:space="preserve">대상의 정신력이 0 미만이면, 0 미만의 정신력 1 당 피해량 +1% (최대 45%)
+[공격 시작 전] (최대 공명 수 + 5)만큼 자신의 진동 횟수 증가 (최대 10)
+[공격 종료시] 공격 대상 중 흐트러짐, 사기 저하, 패닉 상태인 적이 있으면, 정신력 10 회복
+코인 1: [적중시] 진동 횟수 5 증가
+코인 1: [적중시] 대상이 흐트러짐, 사기 저하, 패닉 상태가 아니면, 침잠 5 부여
+코인 1: [적중시] 대상이 흐트러짐, 사기 저하, 패닉 상태가 아니면, 진동 폭발 2회. 대상의 진동 횟수 2 감소
+코인 2: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소</v>
+      </c>
+      <c r="H27" t="str">
         <v>./images/ego/92.webp</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" xml:space="preserve">
       <c r="A28">
         <v>91</v>
       </c>
@@ -28620,11 +29044,21 @@
       <c r="F28" t="str">
         <v>나태 x2, 우울 x1, 오만 x2, 질투 x2</v>
       </c>
-      <c r="G28" t="str">
+      <c r="G28" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] (4 + 최대 공명 수)만큼 자신의 진동 횟수 증가 (최대 8, 턴 당 최대 20)
+- 해당 공명이 나태 공명인 경우, 자신의 진동을 진동 - 태엽감기로 진폭 변환
+코인 1: [적중시] 진동 횟수 1 증가
+코인 1: [앞면 적중시] 진동 5 부여
+코인 1: [뒷면 적중시] 진동 횟수 3 증가
+코인 2: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소.
+코인 2: - 진동 폭발 시 이번 턴에 나태 취약 1 부여
+코인 2: - 최대 공명이 나태 공명 3 이상이면, 다음 턴에도 나태 취약 1 부여</v>
+      </c>
+      <c r="H28" t="str">
         <v>./images/ego/91.webp</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" xml:space="preserve">
       <c r="A29">
         <v>90</v>
       </c>
@@ -28643,11 +29077,27 @@
       <c r="F29" t="str">
         <v>분노 x2, 오만 x6</v>
       </c>
-      <c r="G29" t="str">
+      <c r="G29" t="str" xml:space="preserve">
+        <v xml:space="preserve">체력이 가장 낮은 대상 우선 공격 (아군 우선 지정)
+[공격 시작 전] (최대 공명 수 + 1)만큼 찢어진 추억을 얻음 (최대 7)
+- 해당 공명이 오만 공명이면, 효과를 대신하여 (최대 공명 수 × 2)만큼 찢어진 추억을 얻음 (최대 7)
+[공격 시작 전] 찢어진 추억당 호흡 1 얻음 (최대 7)
+[공격 종료시] 찢어진 추억 전부 소모
+코인 1: 이 코인에는 메인 타겟만 피해를 입음.
+코인 1: 메인 타겟이 아군이면, 찢어진 추억당 피해량 +15% (최대 105%)
+코인 1: [아군 처치 시] 자신과 무작위 아군 2명에게 호흡 3 부여
+코인 1: [아군 처치 시] 처치한 아군의 스킬 1, 2 속성의 E.G.O 자원 +1
+코인 1: [아군 처치 실패시] 호흡 3 얻음
+코인 2: 이 코인에는 서브 타겟만 피해를 입음.
+코인 2: - 첫 번째 코인에서 아군을 처치하지 못했으면, 서브 타겟 중 무작위 1명이 피해를 입음
+코인 2: 찢어진 추억당 크리티컬 피해량 +9% (최대 63%)
+코인 2: [크리티컬 적중 시] 출혈 3 부여</v>
+      </c>
+      <c r="H29" t="str">
         <v>./images/ego/90.webp</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" xml:space="preserve">
       <c r="A30">
         <v>89</v>
       </c>
@@ -28666,11 +29116,27 @@
       <c r="F30" t="str">
         <v>색욕 x5, 탐식 x3, 오만 x2, 질투 x2</v>
       </c>
-      <c r="G30" t="str">
+      <c r="G30" t="str" xml:space="preserve">
+        <v xml:space="preserve">이 스킬을 사용하는 동안은 체력이 1 미만으로 되지 않음.
+대상의 출혈 10 당 코인 위력 +1 (최대 2)
+자신의 누적 소모 혈찬이 100 당, 합 위력 +1 (최대 5)
+[공격 시작 전] 혈찬이 100 미만이면, 적중시마다 출혈 1 부여
+[공격 종료시] 3턴 동안 턴 종료 시 정신력 10 감소
+코인 1: 파괴 불가 코인
+코인 1: 공용 누적 소모 혈찬 1 당, 피해량 +0.1% (최대 10%)
+코인 2: 파괴 불가 코인
+코인 2: 공용 누적 소모 혈찬 100 이상이면, 1 당 피해량 +0.1% (최대 20%)
+코인 3: 파괴 불가 코인
+코인 3: 공용 누적 소모 혈찬 200 이상이면, 1 당 피해량 +0.1% (최대 30%)
+코인 4: 파괴 불가 코인
+코인 4: 공용 누적 소모 혈찬 300 이상이면, 1 당 피해량 +0.1% (최대 50%)
+코인 4: [합 승리 후 적중] 최대 색욕 완전 공명 수에 비례해서 목마른 장미 부여 (최대 4)</v>
+      </c>
+      <c r="H30" t="str">
         <v>./images/ego/89.webp</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" xml:space="preserve">
       <c r="A31">
         <v>88</v>
       </c>
@@ -28689,11 +29155,25 @@
       <c r="F31" t="str">
         <v>색욕 x4, 오만 x3, 질투 x4</v>
       </c>
-      <c r="G31" t="str">
+      <c r="G31" t="str" xml:space="preserve">
+        <v xml:space="preserve">대상의 출혈 6 당 코인 위력 +1 (최대 2)
+[공격 종료시] 3턴 동안 턴 종료 시 정신력 10 감소
+코인 1: [적중시] 출혈 2 부여
+코인 1: [적중시] 최대 공명이 4 이상이면, 대상의 출혈 1회 발동 (출혈 횟수 1 감소)
+코인 2: [적중시] 출혈 2 부여
+코인 2: [적중시] 최대 공명이 4 이상이면, 대상의 출혈 1회 발동 (출혈 횟수 1 감소)
+코인 3: 파괴 불가 코인
+코인 3: [합 승리 후 적중] 장미 쐐기 횟수 2 증가
+코인 3: [적중시] 장미 쐐기 횟수 2 증가
+코인 4: 파괴 불가 코인
+코인 4: [합 승리 후 적중] 대상의 출혈 1 + (최대 공명 수 / 2)회 발동 (최대 3회. 발동한 횟수만큼 출혈 횟수 감소)
+코인 4: [적 처치시] 적의 남은 체력을 초과하여 피해를 준 경우, 초과한 피해량을 고정 피해로 적 전체에 나눠서 가함. (최소 1)</v>
+      </c>
+      <c r="H31" t="str">
         <v>./images/ego/88.webp</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" xml:space="preserve">
       <c r="A32">
         <v>87</v>
       </c>
@@ -28712,11 +29192,19 @@
       <c r="F32" t="str">
         <v>색욕 x2, 오만 x1, 질투 x4</v>
       </c>
-      <c r="G32" t="str">
+      <c r="G32" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 종료시] 자신과 현재 체력 비율이 가장 낮은 아군 2명의 체력을 자신의 최대 체력의 15%만큼 회복
+- 회복받는 대상이 보유한 부정적인 효과 종류 1개당 최대 체력의 2.5%만큼 회복량이 증가 (최대 10%)
+- 이 스킬을 포함하여 질투 공명이 4 이상이면, 회복 대상 수 +1
+코인 1: [적중시] 출혈 4 부여
+코인 2: [적중시] 저주 3 부여
+코인 2: [앞면 적중시] 못 3 부여</v>
+      </c>
+      <c r="H32" t="str">
         <v>./images/ego/87.webp</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" xml:space="preserve">
       <c r="A33">
         <v>86</v>
       </c>
@@ -28735,11 +29223,21 @@
       <c r="F33" t="str">
         <v>색욕 x2, 오만 x2, 질투 x2</v>
       </c>
-      <c r="G33" t="str">
+      <c r="G33" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 이 스킬을 포함하여 공명 수 3 당 공격 가중치 +1 (최대 2)
+[공격 종료시] 대상에게 저주가 있다면 즉시 해당 효과를 2번 발동시키고 저주 2 감소
+코인 1: [앞면 적중시] 출혈 2 부여
+코인 2: [적중시] 저주 2 부여
+코인 2: - 저주와 못을 제외한 대상의 부정적인 효과 2개당 저주 1 추가로 부여 (최대 2)
+코인 2: [적중시] 못 3 부여
+코인 2: [적중시] 대상의 저주가 4 이상이면, 합 위력 감소 1 부여 (턴 당 1회)
+코인 2: [앞면 적중시] 다음 턴에 속박 2 부여 (턴 당 1회)</v>
+      </c>
+      <c r="H33" t="str">
         <v>./images/ego/86.webp</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" xml:space="preserve">
       <c r="A34">
         <v>85</v>
       </c>
@@ -28758,11 +29256,21 @@
       <c r="F34" t="str">
         <v>색욕 x1, 탐식 x4, 오만 x1</v>
       </c>
-      <c r="G34" t="str">
+      <c r="G34" t="str" xml:space="preserve">
+        <v xml:space="preserve">대상과 자신의 속도의 합이 6 이상이면, 코인 위력 +1
+대상의 파열 7 당 코인 위력 +1 (최대 2)
+[공격 시작 전] 다음 턴에 신속 2 얻음
+코인 2: [적중시] 올가미 2 부여
+코인 3: [적중시] 다음 턴에 체력 회복 감소 2 부여
+코인 3: [적중시] 탐식 공명 수 2 당, 파열 횟수 1 증가 (최대 3)
+코인 4: [적중시] 자신의 속도만큼 출혈을 무작위로 공격 대상에게 나누어 부여 (최대 7)
+코인 4: [적중시] 자신의 속도만큼 파열을 무작위로 공격 대상에게 나누어 부여 (최대 7)</v>
+      </c>
+      <c r="H34" t="str">
         <v>./images/ego/85.webp</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" xml:space="preserve">
       <c r="A35">
         <v>84</v>
       </c>
@@ -28781,11 +29289,21 @@
       <c r="F35" t="str">
         <v>색욕 x1, 탐식 x3, 질투 x2</v>
       </c>
-      <c r="G35" t="str">
+      <c r="G35" t="str" xml:space="preserve">
+        <v xml:space="preserve">자신과 대상의 속도의 합이 6 이상이면, 코인 위력 +1
+대상의 파열 7 당 코인 위력 +1 (최대 2)
+[공격 시작 전] 다음 턴에 신속 2 얻음
+[공격 시작 전] 최대 공명이 4 이상이면, 공격 가중치 +1
+- 해당 공명이 탐식 공명이면, 공격 가중치 +1
+코인 1: [적중시] 파열 횟수 2 증가
+코인 2: [적중시] 파열 2 부여
+코인 3: [적중시] 파열 2 부여</v>
+      </c>
+      <c r="H35" t="str">
         <v>./images/ego/84.webp</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" xml:space="preserve">
       <c r="A36">
         <v>83</v>
       </c>
@@ -28804,11 +29322,21 @@
       <c r="F36" t="str">
         <v>색욕 x2, 나태 x1, 우울 x3</v>
       </c>
-      <c r="G36" t="str">
+      <c r="G36" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 최대 공명이 4 이상이면, 공격 가중치 +1
+- 해당 공명이 우울 공명이면, 공격 가중치 +1
+[공격 종료시] 현재 체력 비율이 가장 낮은 아군 2명이 최대 체력의 (10 + (메인 공격 대상의 침잠과 침잠 횟수의 합) / 3)%만큼 체력 회복 (최대 20% 회복)
+- 최대 공명이 우울 공명 4 이상이면, 회복량이 최대 체력의 10%만큼 증가
+코인 1: [적중시] 침잠 횟수 3 증가
+코인 1: [적중시] 저주 2 부여
+코인 1: [적중시] 우울 공명 4 이상이면, 우울 취약 1 부여
+코인 1: [적중시] 초청받지 않은 자 2 부여</v>
+      </c>
+      <c r="H36" t="str">
         <v>./images/ego/83.webp</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" xml:space="preserve">
       <c r="A37">
         <v>82</v>
       </c>
@@ -28827,11 +29355,24 @@
       <c r="F37" t="str">
         <v>색욕 x1, 나태 x2, 우울 x2, 질투 x2</v>
       </c>
-      <c r="G37" t="str">
+      <c r="G37" t="str" xml:space="preserve">
+        <v xml:space="preserve">이 스킬의 코인을 굴릴 때, 공격 대상 중에 하나를 무작위로 선택해 공격
+- 첫 코인은 반드시 메인 공격 대상에게 적중함
+- 모든 적중시 효과, 해당 코인의 피해는 위 효과에서 선택된 공격 대상에게만 적용됨
+이 스킬의 효과로 나비 부여시 앞면이 나올 확률로 죽은나비를 부여
+부여하지 않은 경우, 산나비를 부여 (나비 1 당 개별 판정)
+[공격 종료시] (적중한 3코인 수 × 3)만큼 정신력 회복
+코인 1: [적중시] 무작위 나비 1 부여
+코인 2: [적중시] 무작위 나비 1 부여
+코인 3: [적중시] 무작위 나비 1 ~ 2 부여
+코인 3: [적중시] 정신력 2 ~ 6 감소
+코인 3: [적중시] 자신의 정신력이 0 이상이면, 이 코인 재사용 (스킬 당 최대 5회)</v>
+      </c>
+      <c r="H37" t="str">
         <v>./images/ego/82.webp</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" xml:space="preserve">
       <c r="A38">
         <v>81</v>
       </c>
@@ -28850,11 +29391,19 @@
       <c r="F38" t="str">
         <v>분노 x1, 우울 x3, 오만 x1, 질투 x4</v>
       </c>
-      <c r="G38" t="str">
+      <c r="G38" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] (최대 공명 수 - 2)만큼 공격 가중치 증가 (최대 2)
+[공격 시작 전] 보유한 충전 횟수가 10 미만일 때, 최대 체력의 10%만큼 체력을 소모하여 충전 횟수를 10 얻음 (이 피해로 체력이 0이 되지 않음, 소수점 버림)
+[공격 시작 전] 충전 횟수를 최대 40 소모하여 소모한 충전 횟수당 피해량 +1% (최대 30%)
+코인 1: [적중시] (충전 - 1)만큼 차원 균열 부여 (최대 2)
+코인 1: [적중시] 충전만큼 다음 턴에 신속 1, 부하 1 얻음 (한 스킬당 최대 3)
+코인 1: [적 처치시] 충전 횟수 2 증가</v>
+      </c>
+      <c r="H38" t="str">
         <v>./images/ego/81.webp</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" xml:space="preserve">
       <c r="A39">
         <v>80</v>
       </c>
@@ -28873,11 +29422,22 @@
       <c r="F39" t="str">
         <v>분노 x1, 오만 x3, 질투 x2</v>
       </c>
-      <c r="G39" t="str">
+      <c r="G39" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] (최대 공명 수 + 1)만큼 찢어진 추억을 얻음 (최대 7)
+- 해당 공명이 완전 공명이면 찢어진 추억을 (최대 공명 수 + 2)만큼 얻음
+[공격 시작 전] 찢어진 추억 당 호흡 1 얻음 (최대 7)
+[공격 시작 전] 자신의 호흡 횟수 1 증가
+[공격 종료시] 찢어진 추억 전부 소모
+코인 2: 찢어진 추억 당 크리티컬 피해량 +15% (최대 105%)
+코인 2: [적중시] 출혈 5 부여
+코인 2: [크리티컬 적중 시] 침잠 3 부여
+코인 2: [크리티컬 처치 시] 자신에게 탄환 효과가 있다면, 탄환 1 얻음 (전투 당 3회)</v>
+      </c>
+      <c r="H39" t="str">
         <v>./images/ego/80.webp</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" xml:space="preserve">
       <c r="A40">
         <v>79</v>
       </c>
@@ -28896,11 +29456,18 @@
       <c r="F40" t="str">
         <v>분노 x3, 색욕 x4, 오만 x4, 질투 x3</v>
       </c>
-      <c r="G40" t="str">
+      <c r="G40" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 최대 공명 수만큼 공격 가중치 증가 (최대 6)
+[공격 시작 전] 이번 턴과 다음 턴에 (최대 공명 수 + 1)만큼 경멸의 시선 얻음 (최대 7)
+[공격 종료시] 이 스킬을 포함하여 색욕 공명을 했다면, 자신이 보유한 기본 공격 스킬과 동일한 속성의 E.G.O 자원 +1
+[공격 종료시] 2턴 동안 턴 종료 시 자신의 정신력 10 감소
+코인 1: [공격 종료시] 출혈 15를 공격 대상에게 균등하게 나눠서 부여</v>
+      </c>
+      <c r="H40" t="str">
         <v>./images/ego/79.webp</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" xml:space="preserve">
       <c r="A41">
         <v>78</v>
       </c>
@@ -28919,11 +29486,19 @@
       <c r="F41" t="str">
         <v>분노 x1, 색욕 x1, 나태 x4, 오만 x4</v>
       </c>
-      <c r="G41" t="str">
+      <c r="G41" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] (오만 또는 나태 공명 중 가장 높은 공명 수 - 2)만큼 공격 가중치 증가 (최대 2)
+진동 폭발 시 흐트러짐 손상 100% 증가
+[공격 종료시] 3턴 동안 턴 종료 시 정신력 8 감소
+코인 1: [적중시] 진동 6 부여
+코인 1: [적중시] 진동 - 균열로 진폭 변환
+코인 1: [적중시] 진동 폭발</v>
+      </c>
+      <c r="H41" t="str">
         <v>./images/ego/78.webp</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" xml:space="preserve">
       <c r="A42">
         <v>77</v>
       </c>
@@ -28942,11 +29517,19 @@
       <c r="F42" t="str">
         <v>색욕 x2, 우울 x4, 오만 x2, 질투 x3</v>
       </c>
-      <c r="G42" t="str">
+      <c r="G42" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 종료시] 3턴 동안 턴 종료 시 정신력 10 감소
+[공격 종료시] 다음 턴에 속박 20, 묶인 왕의 앞으로 1, 공격 위력 증가 2 얻음
+코인 1: [적중시] 다음 턴에 속박 1 부여
+코인 1: [적중시] 침잠 4 부여
+코인 1: [적중시] 진동 4 부여
+코인 1: [적중시] 진동 폭발</v>
+      </c>
+      <c r="H42" t="str">
         <v>./images/ego/77.webp</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" xml:space="preserve">
       <c r="A43">
         <v>76</v>
       </c>
@@ -28965,11 +29548,19 @@
       <c r="F43" t="str">
         <v>분노 x1, 질투 x4</v>
       </c>
-      <c r="G43" t="str">
+      <c r="G43" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 자신의 충전 횟수 12 증가
+[공격 종료시] 자신을 제외하고 충전 횟수가 가장 낮은 아군 1명의 충전 횟수 8 증가
+- (최대 질투 공명 수 - 2)만큼 부여 대상 수 증가 (최대 5)
+- 최대 질투 공명 수가 4 이상이면, 자신과 부여 대상에게 질투 피해량 증가 1 부여
+- 최대 질투 공명 수가 6 이상이면, 자신과 부여 대상에게 질투 피해량 증가 1 부여
+코인 1: [적중시] 파열 3 부여</v>
+      </c>
+      <c r="H43" t="str">
         <v>./images/ego/76.webp</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" xml:space="preserve">
       <c r="A44">
         <v>75</v>
       </c>
@@ -28988,11 +29579,17 @@
       <c r="F44" t="str">
         <v>오만 x2, 질투 x4</v>
       </c>
-      <c r="G44" t="str">
+      <c r="G44" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] (질투 공명 수 - 2)만큼 공격 가중치 증가 (최대 3)
+[공격 시작 전] (질투 공명 수 - 3) × 10%만큼 피해량이 증가 (최대 30%)
+[공격 시작 전] 자신의 충전 횟수가 20 이상이면, 충전 횟수를 20 소모하여 피해량 +40%
+코인 1: [적 처치 시] 자신의 충전 횟수 2 증가</v>
+      </c>
+      <c r="H44" t="str">
         <v>./images/ego/75.webp</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" xml:space="preserve">
       <c r="A45">
         <v>74</v>
       </c>
@@ -29011,11 +29608,16 @@
       <c r="F45" t="str">
         <v>색욕 x2, 우울 x4</v>
       </c>
-      <c r="G45" t="str">
+      <c r="G45" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 종료시] 자신과 자신을 제외한 정신력이 가장 낮은 아군 2명의 정신력 15 회복
+- 대상이 사망하지 않았다면, 대상의 침잠 횟수를 3 소모하고, 대상의 침잠 위력만큼 회복 대상의 정신력 추가 회복 (최대 회복량 : 20)
+- 대상이 사망했다면, 무작위 적 3명에게 침잠 3, 저주 1 부여 (집중 전투인 경우, 무작위 부위에 부여)</v>
+      </c>
+      <c r="H45" t="str">
         <v>./images/ego/74.webp</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" xml:space="preserve">
       <c r="A46">
         <v>73</v>
       </c>
@@ -29034,11 +29636,15 @@
       <c r="F46" t="str">
         <v>나태 x3, 우울 x3</v>
       </c>
-      <c r="G46" t="str">
+      <c r="G46" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 종료시] 침잠 6 + (우울 공명 수 × 1.5)을 무작위로 공격 대상에게 나눠서 부여
+코인 1: [적중시] 대상에게 침잠이 6 이상이면 다음 턴에 속박 2 부여</v>
+      </c>
+      <c r="H46" t="str">
         <v>./images/ego/73.webp</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" xml:space="preserve">
       <c r="A47">
         <v>66</v>
       </c>
@@ -29057,11 +29663,24 @@
       <c r="F47" t="str">
         <v>색욕 x2, 나태 x4, 우울 x2, 오만 x3</v>
       </c>
-      <c r="G47" t="str">
+      <c r="G47" t="str" xml:space="preserve">
+        <v xml:space="preserve">대상의 속도가 자신보다 느릴 때, 피해량 +(대상과의 속도 차이 × 5)% (최대 50%)
+[공격 시작 전] 최대 공명 수가 3 이상일 경우, (최대 공명 수 × 2)만큼 진동 위력 부여 (최대 10)
+- 최대 공명이 나태 완전 공명일 경우, 부여한 진동 위력 값만큼 진동 횟수 부여 (최대 10)
+[공격 종료 시] 3턴 동안 턴 종료 시 정신력 10 감소
+코인 1: [적중시] 진동 10, 진동 횟수 10 부여
+코인 1: [적중시] 진동 - 영속으로 진폭 얽힘
+코인 1: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소
+코인 2: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소
+코인 3: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소
+코인 4: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소
+코인 4: [적중시] 다음 턴에 대상의 속도 최댓값 절반으로 감소</v>
+      </c>
+      <c r="H47" t="str">
         <v>./images/ego/66.webp</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" xml:space="preserve">
       <c r="A48">
         <v>65</v>
       </c>
@@ -29080,11 +29699,17 @@
       <c r="F48" t="str">
         <v>색욕 x1, 나태 x2, 우울 x3</v>
       </c>
-      <c r="G48" t="str">
+      <c r="G48" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] (최대 공명 수 - 2)만큼 공격 가중치 증가 (최대 2)
+코인 1: [공격 종료시] 자신과 현재 체력이 가장 적은 아군 1 + (최대 공명 수 - 2)명에게 자신의 최대 체력 20%만큼 보호막을 부여하고 울음 방울 2 부여 (자신 제외 최대 부여 대상 수 : 3)
+코인 1: - 대상에게 이미 울음 방울이 있으면, 울음 방울 수치를 2로 변경
+코인 1: - 최대 우울 완전 공명 수가 4 이상이면, 이 스킬의 울음 방울 수치가 3로 부여, 적용됨</v>
+      </c>
+      <c r="H48" t="str">
         <v>./images/ego/65.webp</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" xml:space="preserve">
       <c r="A49">
         <v>64</v>
       </c>
@@ -29103,11 +29728,22 @@
       <c r="F49" t="str">
         <v>분노 x1, 색욕 x3, 오만 x3, 질투 x3</v>
       </c>
-      <c r="G49" t="str">
+      <c r="G49" t="str" xml:space="preserve">
+        <v xml:space="preserve">대상의 출혈 2당 코인 위력 +1 (최대 13)
+[전투 시작시] 이 스킬의 메인 타겟은 이번 턴 동안 출혈 횟수가 감소하지 않음.
+[공격 종료시] 3턴 동안 턴 종료 시 정신력 10 감소.
+코인 1: [적중시] (대상의 출혈 위력 x 1.5)만큼 색욕 속성 피해를 줌.
+코인 1: - 색욕 공명이 4 이상이면, x1.8로 계산.
+코인 1: - 최대 색욕 완전 공명 수가 4 이상이면, x2로 계산.
+코인 1: (계산 시 반영되는 출혈 위력은 99를 초과할 수 없음.)
+코인 1: [적 처치 시] 이 스킬의 피해 또는 코인 효과로 적의 남은 체력을 초과하여 피해를 준 경우, 초과한 피해량을 고정 피해로 적 전체에 나눠서 가함.
+코인 1: (집중 전투인 경우, 본체의 체력을 기준으로 계산)</v>
+      </c>
+      <c r="H49" t="str">
         <v>./images/ego/64.webp</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" xml:space="preserve">
       <c r="A50">
         <v>63</v>
       </c>
@@ -29126,11 +29762,18 @@
       <c r="F50" t="str">
         <v>나태 x3, 우울 x3, 오만 x2</v>
       </c>
-      <c r="G50" t="str">
+      <c r="G50" t="str" xml:space="preserve">
+        <v xml:space="preserve">대상에게 진동이 있으면, 피해량 +(5 + 대상의 진동 위력과 진동 횟수의 합 / 2)% (최대 30%)
+- 최대 공명 수가 4 이상이면, 대신 피해량 +(7.5 + 대상의 진동 위력과 진동 횟수의 합 / 1.5)% (최대 40%)
+코인 1: [적중시] 진동 3, 진동 횟수 3 부여
+코인 1: [적중시] 진동 - 반향으로 진폭 변환
+코인 1: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소</v>
+      </c>
+      <c r="H50" t="str">
         <v>./images/ego/63.webp</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" xml:space="preserve">
       <c r="A51">
         <v>62</v>
       </c>
@@ -29149,11 +29792,20 @@
       <c r="F51" t="str">
         <v>색욕 x1, 탐식 x3, 오만 x2</v>
       </c>
-      <c r="G51" t="str">
+      <c r="G51" t="str" xml:space="preserve">
+        <v xml:space="preserve">이 스킬의 효과로 자신의 체력을 초과하여 회복한 경우, 초과한 회복량만큼 체력 비율이 가장 낮은 아군 1명의 체력을 대신 회복
+코인 1: [적중시] 자신의 체력을 최대 체력의 20% 만큼 회복
+코인 2: [앞면 적중시] 정신력 1 ~ 2 감소
+코인 2: [앞면 적중시] 이 코인 재사용 (스킬당 최대 5회)
+코인 2: [적중시] 자신의 체력을 피해량의 8 ~ 12%만큼 회복
+코인 2: [적중시] 탐식 취약 1 부여
+코인 2: [적중시] 출혈 1 ~ 4 부여</v>
+      </c>
+      <c r="H51" t="str">
         <v>./images/ego/62.webp</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" xml:space="preserve">
       <c r="A52">
         <v>61</v>
       </c>
@@ -29172,11 +29824,20 @@
       <c r="F52" t="str">
         <v>분노 x2, 색욕 x2, 나태 x2, 탐식 x2, 우울 x2, 오만 x2, 질투 x2</v>
       </c>
-      <c r="G52" t="str">
+      <c r="G52" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] (가장 높은 공명 수 - 2)만큼 공격 가중치 증가 (최대 3)
+[사용시] 아군 4 + (가장 높은 공명 수)명에게 해당 공명 속성의 피해량 증가와 위력 증가를 1 부여
+- 해당 공명이 4 이상이면, 해당 속성 피해량 증가를 1 추가 부여
+- 해당 공명이 5 이상이면, 해당 속성 위력 증가를 1 추가 부여
+- 해당 공명이 완전 공명 6 이상이면, 다음 턴에도 동일한 효과 부여
+코인 1: [공격 종료 시] 체력 비율이 가장 낮은 아군 4명의 체력을 최대 체력의 22%만큼 회복
+코인 1: - (가장 높은 공명 수 - 2)만큼 회복 대상 증가 (최대 3)</v>
+      </c>
+      <c r="H52" t="str">
         <v>./images/ego/61.webp</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" xml:space="preserve">
       <c r="A53">
         <v>60</v>
       </c>
@@ -29195,11 +29856,16 @@
       <c r="F53" t="str">
         <v>분노 x2, 나태 x2, 오만 x1</v>
       </c>
-      <c r="G53" t="str">
+      <c r="G53" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 출혈 횟수 4 증가
+코인 1: [적중시] 진동 5 부여
+코인 1: [앞면 적중시] 마비 2 부여</v>
+      </c>
+      <c r="H53" t="str">
         <v>./images/ego/60.webp</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" xml:space="preserve">
       <c r="A54">
         <v>59</v>
       </c>
@@ -29218,11 +29884,15 @@
       <c r="F54" t="str">
         <v>나태 x4, 탐식 x2, 우울 x2, 오만 x2</v>
       </c>
-      <c r="G54" t="str">
+      <c r="G54" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 이번 턴, 다음 턴 동안 모든 아군에게 나태 위력 증가 1, 나태 피해량 증가 2, 보호 3 부여
+코인 1: [앞면 적중시] 자신의 정신력 15 회복</v>
+      </c>
+      <c r="H54" t="str">
         <v>./images/ego/59.webp</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" xml:space="preserve">
       <c r="A55">
         <v>58</v>
       </c>
@@ -29241,11 +29911,17 @@
       <c r="F55" t="str">
         <v>나태 x3, 탐식 x3</v>
       </c>
-      <c r="G55" t="str">
+      <c r="G55" t="str" xml:space="preserve">
+        <v xml:space="preserve">가장 뒤에 있는 적 공격 (일반 전투 한정)
+[공격 시작 전] 충전 횟수를 소모하고 소모한 만큼 피해량이 증가함 (최대 75%)
+코인 1: [적중시] 충전 횟수를 소모한 경우, 차원 균열 5 부여.
+코인 1: [적중시] 피해량의 (대상의 파열x10)%만큼 오만 추가 피해를 주고, 파열 횟수 5 소모 (최대 100%)</v>
+      </c>
+      <c r="H55" t="str">
         <v>./images/ego/58.webp</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" xml:space="preserve">
       <c r="A56">
         <v>57</v>
       </c>
@@ -29264,11 +29940,18 @@
       <c r="F56" t="str">
         <v>분노 x5, 나태 x1, 탐식 x1</v>
       </c>
-      <c r="G56" t="str">
+      <c r="G56" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 모든 공격 대상의 화상의 합
+- 6당, 최종 위력 +1 (최대 4)
+- 1당, 피해량 +1% (최대 30%)
+코인 1: [적중시] 화상 4 부여
+코인 1: [앞면 적중시] 화상 6 부여</v>
+      </c>
+      <c r="H56" t="str">
         <v>./images/ego/57.webp</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" xml:space="preserve">
       <c r="A57">
         <v>56</v>
       </c>
@@ -29287,11 +29970,16 @@
       <c r="F57" t="str">
         <v>나태 x4, 우울 x1</v>
       </c>
-      <c r="G57" t="str">
+      <c r="G57" t="str" xml:space="preserve">
+        <v xml:space="preserve">가장 뒤에 있는 대상 공격 (일반 전투 한정)
+코인 1: [적중시] 나태 취약 2 부여
+코인 1: [앞면 적중시] 마비 3 부여</v>
+      </c>
+      <c r="H57" t="str">
         <v>./images/ego/56.webp</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" xml:space="preserve">
       <c r="A58">
         <v>55</v>
       </c>
@@ -29310,11 +29998,16 @@
       <c r="F58" t="str">
         <v>분노 x1, 나태 x3</v>
       </c>
-      <c r="G58" t="str">
+      <c r="G58" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 공격 위력 감소 2 부여
+코인 1: [적중시] 모든 아군에게 다음 턴에 신속 3 부여
+코인 1: [적중시] 다음 턴에 속박 2 부여</v>
+      </c>
+      <c r="H58" t="str">
         <v>./images/ego/55.webp</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" xml:space="preserve">
       <c r="A59">
         <v>54</v>
       </c>
@@ -29333,11 +30026,18 @@
       <c r="F59" t="str">
         <v>분노 x2, 색욕 x5, 질투 x1</v>
       </c>
-      <c r="G59" t="str">
+      <c r="G59" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] (색욕 공명 수)가 4 이상이면, 공격 가중치 +1
+[공격 시작 전] (최대 색욕 완전 공명 수)가 4 이상이면, 추가로 공격 가중치 +1
+코인 1: [적중시] 대상에게 화상이 없으면 화상 4 부여
+코인 1: [적중시] 화상 4 부여
+코인 1: [뒷면 적중시] 대상의 화상이 10 이상이면 다음 턴에 공격 위력 감소 1, 수비 위력 감소 1 부여</v>
+      </c>
+      <c r="H59" t="str">
         <v>./images/ego/54.webp</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" xml:space="preserve">
       <c r="A60">
         <v>53</v>
       </c>
@@ -29356,11 +30056,16 @@
       <c r="F60" t="str">
         <v>색욕 x1, 탐식 x4, 오만 x2</v>
       </c>
-      <c r="G60" t="str">
+      <c r="G60" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 자신의 체력이 50% 미만이면, 공격 가중치 +2
+코인 1: [적중시] 파열 3 부여
+코인 1: [적중시] 현재 체력 비율이 가장 낮은 아군 2명의 체력을 최대 체력의 15%만큼 회복</v>
+      </c>
+      <c r="H60" t="str">
         <v>./images/ego/53.webp</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" xml:space="preserve">
       <c r="A61">
         <v>52</v>
       </c>
@@ -29379,11 +30084,26 @@
       <c r="F61" t="str">
         <v>분노 x3, 색욕 x2, 탐식 x1</v>
       </c>
-      <c r="G61" t="str">
+      <c r="G61" t="str" xml:space="preserve">
+        <v xml:space="preserve">[피아식별불가]
+현재 체력이 가장 낮은 대상 공격
+스킬 사용 시 필요한 탐식 E.G.O 자원이 0으로 변경됨
+대상이 아군인 경우, 피해량이 항상 0으로 고정되고 수비 스킬을 발동하지 않음 (합 가능 수비 포함)
+[합 패배] 기본 위력 -8
+[공격 종료시] 이 스킬이 아군에게 적중했으면, 자신의 정신력을 이 스킬의 타겟으로 지정된 아군의 수만큼 회복
+[공격 종료시] 자신의 최대 체력의 (5 x 이 스킬의 타겟으로 지정된 아군 수)% 만큼 자신의 체력 회복 (최소 5%, 최대 20%)
+[공격 종료시] 다음 턴에 E.G.O 자원 획득량 + 1, 신속 2 얻음
+코인 1: 파괴 불가 코인
+코인 1: [적중시] 대상이 아군인 경우,
+코인 1: - 자신의 최대 체력의 (5 x 이 스킬의 타겟으로 지정된 아군 수)%만큼 대상의 체력 회복 (최대 20%)
+코인 1: - 다음 턴에 E.G.O 자원 획득량 + 1, 신속 2 부여
+코인 1: [뒷면 적중시] 화상 7 부여</v>
+      </c>
+      <c r="H61" t="str">
         <v>./images/ego/52.webp</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" xml:space="preserve">
       <c r="A62">
         <v>51</v>
       </c>
@@ -29402,11 +30122,16 @@
       <c r="F62" t="str">
         <v>분노 x3, 색욕 x2</v>
       </c>
-      <c r="G62" t="str">
+      <c r="G62" t="str" xml:space="preserve">
+        <v xml:space="preserve">대상의 체력이 25%미만일 때 피해량 +40%
+코인 1: [적 처치 시] 다음 턴에 공격 위력 증가 1 얻음
+코인 1: [적 처치 시] 아군 전체가 각자 최대 체력의 15%만큼 체력 회복</v>
+      </c>
+      <c r="H62" t="str">
         <v>./images/ego/51.webp</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" xml:space="preserve">
       <c r="A63">
         <v>50</v>
       </c>
@@ -29425,11 +30150,16 @@
       <c r="F63" t="str">
         <v>분노 x1, 탐식 x3</v>
       </c>
-      <c r="G63" t="str">
+      <c r="G63" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [앞면 적중시] 파열 12 부여
+코인 1: [앞면 적중시] 정신력 10 감소. 다음 턴에 공격 위력 증가 1을 얻음
+코인 1: [뒷면 적중시] 정신력 10 회복. 다음 턴에 보호 1을 얻음</v>
+      </c>
+      <c r="H63" t="str">
         <v>./images/ego/50.webp</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" xml:space="preserve">
       <c r="A64">
         <v>49</v>
       </c>
@@ -29448,11 +30178,17 @@
       <c r="F64" t="str">
         <v>우울 x2, 오만 x2, 질투 x2</v>
       </c>
-      <c r="G64" t="str">
+      <c r="G64" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 호흡 4 얻음
+[공격 종료시] 이 스킬이 적중한 대상 중 사망한 캐릭터 수만큼 호흡 2를 얻음
+코인 1: [적중시] 충전 횟수 2 증가
+코인 1: [크리티컬 적중 시] 자신의 충전 횟수 2 증가</v>
+      </c>
+      <c r="H64" t="str">
         <v>./images/ego/49.webp</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" xml:space="preserve">
       <c r="A65">
         <v>48</v>
       </c>
@@ -29471,11 +30207,20 @@
       <c r="F65" t="str">
         <v>탐식 x2, 오만 x2, 질투 x2</v>
       </c>
-      <c r="G65" t="str">
+      <c r="G65" t="str" xml:space="preserve">
+        <v xml:space="preserve">대상의 현재 체력이 최대 체력의 25% 미만이면, 피해량 +40%
+[공격 시작 전] 최대 공명수가 4 이상이면, 공격 가중치 +1
+[공격 종료시] 다음 턴에 자신을 포함한 무작위 아군 2+ (최대 공명 수)명에게 E.G.O 자원 획득량 + 1 부여 (최대 7명)
+[공격 종료시] 공격 대상 중 흐트러짐이나 패닉 상태인 대상이 있으면, 가장 적게 보유한 E.G.O 자원 1개를 얻음. 자신의 정신력 3 회복
+코인 1: [적중시] 진동 4 부여
+코인 1: [적중시] 침잠 6 부여
+코인 1: [적 처치 시] 현재 보유 중인 E.G.O 자원 중 무작위 속성 1개의 E.G.O 자원을 3개 얻음. 모든 아군의 정신력 3 회복</v>
+      </c>
+      <c r="H65" t="str">
         <v>./images/ego/48.webp</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" xml:space="preserve">
       <c r="A66">
         <v>47</v>
       </c>
@@ -29494,11 +30239,16 @@
       <c r="F66" t="str">
         <v>분노 x2, 색욕 x2, 질투 x3</v>
       </c>
-      <c r="G66" t="str">
+      <c r="G66" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 다음 턴에 속박 3 부여
+코인 1: [적중시] 대상에게 속박이 3 이상 있을 때 다음 턴에 더하기 코인 약화 1 부여
+코인 1: [적중시] 대상의 속도가 자신보다 느릴 때 다음 턴에 참격 취약 2 부여</v>
+      </c>
+      <c r="H66" t="str">
         <v>./images/ego/47.webp</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" xml:space="preserve">
       <c r="A67">
         <v>46</v>
       </c>
@@ -29517,11 +30267,16 @@
       <c r="F67" t="str">
         <v>색욕 x2, 탐식 x2, 질투 x1</v>
       </c>
-      <c r="G67" t="str">
+      <c r="G67" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 다음 턴에 속박 3 부여
+코인 1: [적중시] 대상에게 속박이 3 이상 있을 때 다음 턴에 더하기 코인 약화 1 부여
+코인 1: [적중시] 대상의 속도가 자신보다 느릴 때 다음 턴에 참격 취약 2 부여</v>
+      </c>
+      <c r="H67" t="str">
         <v>./images/ego/46.webp</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" xml:space="preserve">
       <c r="A68">
         <v>45</v>
       </c>
@@ -29540,11 +30295,18 @@
       <c r="F68" t="str">
         <v>분노 x4, 오만 x2</v>
       </c>
-      <c r="G68" t="str">
+      <c r="G68" t="str" xml:space="preserve">
+        <v xml:space="preserve">대상에게 화상이 있으면 스킬 위력 +2
+[공격 시작 전] 모든 공격 대상의 화상 위력의 합 1당 5%만큼 피해량 증가 (최대 100%)
+[적 처치 시] 다음 턴에 공격 위력 증가 2 얻음
+코인 1: [적중시] 이 코인 최종 피해량의 (대상의 화상 위력 × 2)%만큼 분노 피해 (최대 20%)
+코인 1: [적중시] 화상 4 부여</v>
+      </c>
+      <c r="H68" t="str">
         <v>./images/ego/45.webp</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" xml:space="preserve">
       <c r="A69">
         <v>44</v>
       </c>
@@ -29563,11 +30325,16 @@
       <c r="F69" t="str">
         <v>분노 x2, 색욕 x2</v>
       </c>
-      <c r="G69" t="str">
+      <c r="G69" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 화상 6 부여
+코인 1: [적중시] 다음 턴에 취약 1 부여
+코인 1: [앞면 적중시] 다음 턴에 취약 1 부여</v>
+      </c>
+      <c r="H69" t="str">
         <v>./images/ego/44.webp</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" xml:space="preserve">
       <c r="A70">
         <v>43</v>
       </c>
@@ -29586,11 +30353,16 @@
       <c r="F70" t="str">
         <v>나태 x4, 오만 x3</v>
       </c>
-      <c r="G70" t="str">
+      <c r="G70" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 다음 턴에 나태 취약 1 부여
+코인 1: [공격 종료시] 자신을 제외하고 현재 체력 비율이 가장 낮은 아군 2명의 체력을 자신의 최대 체력의 30%만큼 회복
+코인 1: [앞면 공격 종료 시] 대상이 흐트러지거나 사망한 경우, 체력을 회복시킨 캐릭터들에게 자신의 최대 체력의 15%만큼 보호막 부여</v>
+      </c>
+      <c r="H70" t="str">
         <v>./images/ego/43.webp</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" xml:space="preserve">
       <c r="A71">
         <v>42</v>
       </c>
@@ -29609,11 +30381,17 @@
       <c r="F71" t="str">
         <v>나태 x2, 우울 x2, 오만 x2</v>
       </c>
-      <c r="G71" t="str">
+      <c r="G71" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 메인 공격 대상의 체력이 최대 체력의 50% 이상이면, 공격 가중치 +1, 최대 체력의 75% 이상이면, 추가로 공격 가중치 +1
+코인 1: [적중시] 진동 3, 진동 횟수 7 부여
+코인 1: [앞면 적중시] 다음 턴에 속박 2 부여
+코인 1: [적중시] 진동 폭발</v>
+      </c>
+      <c r="H71" t="str">
         <v>./images/ego/42.webp</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" xml:space="preserve">
       <c r="A72">
         <v>41</v>
       </c>
@@ -29632,11 +30410,17 @@
       <c r="F72" t="str">
         <v>우울 x5, 질투 x3</v>
       </c>
-      <c r="G72" t="str">
+      <c r="G72" t="str" xml:space="preserve">
+        <v xml:space="preserve">대상의 체력이 50%이상이면, 피해량 +30%
+코인 1: [적중시] 진동 폭발
+코인 1: [적중시] 침잠 5 부여
+코인 1: [적중시] 침잠 횟수 5 증가</v>
+      </c>
+      <c r="H72" t="str">
         <v>./images/ego/41.webp</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" xml:space="preserve">
       <c r="A73">
         <v>40</v>
       </c>
@@ -29655,11 +30439,18 @@
       <c r="F73" t="str">
         <v>분노 x3, 오만 x2, 질투 x1</v>
       </c>
-      <c r="G73" t="str">
+      <c r="G73" t="str" xml:space="preserve">
+        <v xml:space="preserve">최대 공명 수 1당, 피해량 +5% (최대 30%)
+[공격 종료시] 다음 턴에 분노 위력 증가 1, 분노 피해량 증가 1 얻음
+코인 1: 파괴 불가 코인
+코인 1: [파괴되지 않고 적중시] 화상 6 부여
+코인 1: [적중시] 다음 턴에 분노 취약 3 부여</v>
+      </c>
+      <c r="H73" t="str">
         <v>./images/ego/40.webp</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" xml:space="preserve">
       <c r="A74">
         <v>39</v>
       </c>
@@ -29678,11 +30469,17 @@
       <c r="F74" t="str">
         <v>우울 x1, 오만 x3</v>
       </c>
-      <c r="G74" t="str">
+      <c r="G74" t="str" xml:space="preserve">
+        <v xml:space="preserve">대상의 체력이 50%이상이면, 피해량 +30%
+코인 1: [적중시] 출혈 4 부여
+코인 1: [적중시] 다음 턴에 정신력 회복 효율 +2
+코인 1: [적중시] 다음 턴에 정신력 감소 효율 -2</v>
+      </c>
+      <c r="H74" t="str">
         <v>./images/ego/39.webp</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" xml:space="preserve">
       <c r="A75">
         <v>38</v>
       </c>
@@ -29701,11 +30498,16 @@
       <c r="F75" t="str">
         <v>색욕 x2, 나태 x1, 오만 x3, 질투 x2</v>
       </c>
-      <c r="G75" t="str">
+      <c r="G75" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 진동 폭발
+코인 1: [공격 종료시] 현재 정신력이 가장 낮은 아군 4명에게 가장 높은 공명 속성의 피해량 증가를 1 부여
+코인 1: [공격 종료시] 현재 정신력이 가장 낮은 아군 4명의 정신력 20 회복</v>
+      </c>
+      <c r="H75" t="str">
         <v>./images/ego/38.webp</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" xml:space="preserve">
       <c r="A76">
         <v>37</v>
       </c>
@@ -29724,11 +30526,17 @@
       <c r="F76" t="str">
         <v>나태 x2, 탐식 x2, 우울 x1</v>
       </c>
-      <c r="G76" t="str">
+      <c r="G76" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 호흡 횟수 7 증가
+코인 1: [적중시] 침잠 6 부여
+코인 1: [적중시] 다음 턴에 속박 3 부여
+코인 1: [크리티컬 적중 시] 진동 폭발. 침잠 횟수 3 증가</v>
+      </c>
+      <c r="H76" t="str">
         <v>./images/ego/37.webp</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" xml:space="preserve">
       <c r="A77">
         <v>36</v>
       </c>
@@ -29747,11 +30555,16 @@
       <c r="F77" t="str">
         <v>색욕 x2, 탐식 x3, 우울 x1, 오만 x4</v>
       </c>
-      <c r="G77" t="str">
+      <c r="G77" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 파열 2 부여
+코인 1: [앞면 적중시] 출혈 2 부여
+코인 1: [적중시] 탐식 취약 2 부여</v>
+      </c>
+      <c r="H77" t="str">
         <v>./images/ego/36.webp</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" xml:space="preserve">
       <c r="A78">
         <v>35</v>
       </c>
@@ -29770,11 +30583,16 @@
       <c r="F78" t="str">
         <v>색욕 x2, 나태 x2, 오만 x2</v>
       </c>
-      <c r="G78" t="str">
+      <c r="G78" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 종료시] 정신력 18 회복
+[공격 종료시] 본인 제외 무작위 아군 2명에게 공격 위력 증가 1 부여
+코인 1: [적중시] 색욕 취약 2 부여</v>
+      </c>
+      <c r="H78" t="str">
         <v>./images/ego/35.webp</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" xml:space="preserve">
       <c r="A79">
         <v>34</v>
       </c>
@@ -29793,11 +30611,16 @@
       <c r="F79" t="str">
         <v>나태 x2, 오만 x2</v>
       </c>
-      <c r="G79" t="str">
+      <c r="G79" t="str" xml:space="preserve">
+        <v xml:space="preserve">대상의 체력이 50%미만일 때 피해량+30%
+코인 1: [적중시] 파열 4 부여
+코인 1: [적 처치 시] 무작위 아군 1명에게 피해량 증가 1 부여</v>
+      </c>
+      <c r="H79" t="str">
         <v>./images/ego/34.webp</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" xml:space="preserve">
       <c r="A80">
         <v>33</v>
       </c>
@@ -29816,11 +30639,17 @@
       <c r="F80" t="str">
         <v>분노 x3, 오만 x2</v>
       </c>
-      <c r="G80" t="str">
+      <c r="G80" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 자신에게 부여된 해제 가능한 부정적인 효과 중 무작위 2개 제거
+코인 1: [적중시] 진동 횟수 3 증가, (분노 완전 공명의 수)/3만큼 추가 증가
+코인 1: [적중시] 진동 폭발
+코인 1: 진동 폭발 시 대상에게 흐트러짐 구간이 없는 경우, 최종 흐트러짐 손상의 (12 + 3×(분노 완전 공명 수))%만큼 분노 피해를 줌</v>
+      </c>
+      <c r="H80" t="str">
         <v>./images/ego/33.webp</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" xml:space="preserve">
       <c r="A81">
         <v>32</v>
       </c>
@@ -29839,11 +30668,18 @@
       <c r="F81" t="str">
         <v>분노 x2, 색욕 x1, 나태 x2</v>
       </c>
-      <c r="G81" t="str">
+      <c r="G81" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 종료시] 다음 턴에 신속 2, 분노 위력 증가 1, 타격 위력 증가 1 얻음
+코인 1: [적중시] 화상 10 부여
+코인 1: [적중시] 대상의 화상 수치만큼 진동 부여
+코인 1: [적중시] 무작위 적 5명에게 화상 3 부여
+코인 1: [적중시] 진동 폭발. 진동 폭발 시 진동 횟수 2 감소, 진동 폭발로 대상이 흐트러진 경우 무작위 적 5명의 화상 횟수 3 증가</v>
+      </c>
+      <c r="H81" t="str">
         <v>./images/ego/32.webp</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" xml:space="preserve">
       <c r="A82">
         <v>31</v>
       </c>
@@ -29862,11 +30698,16 @@
       <c r="F82" t="str">
         <v>나태 x2, 오만 x1, 질투 x2</v>
       </c>
-      <c r="G82" t="str">
+      <c r="G82" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 종료시] 보호 3 얻음
+[공격 종료시] 다음 턴에 시술 1 얻음
+코인 1: [앞면 적중시] 마비 3 부여</v>
+      </c>
+      <c r="H82" t="str">
         <v>./images/ego/31.webp</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" xml:space="preserve">
       <c r="A83">
         <v>30</v>
       </c>
@@ -29885,11 +30726,15 @@
       <c r="F83" t="str">
         <v>나태 x4, 우울 x1, 오만 x2</v>
       </c>
-      <c r="G83" t="str">
+      <c r="G83" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 종료시] 자신을 제외하고 현재 체력이 가장 낮은 아군 2명 최대 체력의 30%만큼 체력을 회복, 다음 턴에 보호 2 부여
+코인 1: [적중시] 진동 폭발</v>
+      </c>
+      <c r="H83" t="str">
         <v>./images/ego/30.webp</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" xml:space="preserve">
       <c r="A84">
         <v>29</v>
       </c>
@@ -29908,11 +30753,18 @@
       <c r="F84" t="str">
         <v>나태 x1, 우울 x1, 질투 x2</v>
       </c>
-      <c r="G84" t="str">
+      <c r="G84" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 다음 턴에 속박 5 부여
+코인 1: [적중시] 다음 턴에 속박 3 얻음
+코인 1: [적중시] 다음 턴에 공격 위력 감소 4 부여
+코인 1: [적중시] 다음 턴에 공격 위력 감소 3 얻음
+코인 1: [적중시] 다음 턴에 보호 2 얻음</v>
+      </c>
+      <c r="H84" t="str">
         <v>./images/ego/29.webp</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" xml:space="preserve">
       <c r="A85">
         <v>28</v>
       </c>
@@ -29931,11 +30783,17 @@
       <c r="F85" t="str">
         <v>분노 x2, 우울 x3, 오만 x3, 질투 x3</v>
       </c>
-      <c r="G85" t="str">
+      <c r="G85" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 종료시] 정신력이 가장 낮은 아군 4명의 정신력 25 회복
+코인 1: [적중시] 자신의 충전 횟수 6 증가
+코인 1: [적중시] 무작위 아군 1명에게 호흡 횟수 2 부여
+코인 1: [공격 종료시] 정신력이 가장 높은 아군 4명에게 관통 위력 증가 2, 피해량 증가 2 부여</v>
+      </c>
+      <c r="H85" t="str">
         <v>./images/ego/28.webp</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" xml:space="preserve">
       <c r="A86">
         <v>27</v>
       </c>
@@ -29954,11 +30812,16 @@
       <c r="F86" t="str">
         <v>분노 x2, 색욕 x2, 나태 x1</v>
       </c>
-      <c r="G86" t="str">
+      <c r="G86" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 종료시] 다음 턴에 모든 아군에게 분노 피해량 증가 1 부여
+코인 1: [적중시] 화상 4 부여
+코인 1: [적중시] 대상에게 정신력 15 피해</v>
+      </c>
+      <c r="H86" t="str">
         <v>./images/ego/27.webp</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" xml:space="preserve">
       <c r="A87">
         <v>26</v>
       </c>
@@ -29977,11 +30840,17 @@
       <c r="F87" t="str">
         <v>분노 x1, 색욕 x4</v>
       </c>
-      <c r="G87" t="str">
+      <c r="G87" t="str" xml:space="preserve">
+        <v xml:space="preserve">가장 뒤에 있는 대상 공격 (일반 전투 한정)
+코인 1: [적중시] 공격 레벨 감소 10 부여
+코인 1: [적중시] 마비 3 부여
+코인 1: [적중시] 다음 턴에 속박 3 부여</v>
+      </c>
+      <c r="H87" t="str">
         <v>./images/ego/26.webp</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" xml:space="preserve">
       <c r="A88">
         <v>25</v>
       </c>
@@ -30000,11 +30869,17 @@
       <c r="F88" t="str">
         <v>분노 x4, 색욕 x2, 질투 x1</v>
       </c>
-      <c r="G88" t="str">
+      <c r="G88" t="str" xml:space="preserve">
+        <v xml:space="preserve">가장 뒤에 있는 대상 공격 (일반 전투 한정)
+코인 1: [앞면 적중시] 피해량의 40%만큼 흐트러짐 손상 입힘
+코인 1: [적중시] 분노 공명 수만큼 화상 부여
+코인 1: [앞면 공격 종료 시] 무작위 적 3명에게 화상 5 부여</v>
+      </c>
+      <c r="H88" t="str">
         <v>./images/ego/25.webp</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" xml:space="preserve">
       <c r="A89">
         <v>24</v>
       </c>
@@ -30023,11 +30898,17 @@
       <c r="F89" t="str">
         <v>분노 x2, 우울 x2</v>
       </c>
-      <c r="G89" t="str">
+      <c r="G89" t="str" xml:space="preserve">
+        <v xml:space="preserve">가장 뒤에 있는 대상 공격 (일반 전투 한정)
+코인 1: [적중시] 다음 턴에 속박 6 부여
+코인 1: [적중시] 진동 3 부여
+코인 1: [적중시] 진동 폭발</v>
+      </c>
+      <c r="H89" t="str">
         <v>./images/ego/24.webp</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" xml:space="preserve">
       <c r="A90">
         <v>23</v>
       </c>
@@ -30046,11 +30927,18 @@
       <c r="F90" t="str">
         <v>탐식 x6, 우울 x1</v>
       </c>
-      <c r="G90" t="str">
+      <c r="G90" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 자신의 체력이 최대 체력의 50% 미만이면, 공격 가중치 +1
+최대 체력의 25% 미만이면, 추가로 공격 가중치 +1
+코인 1: [적중시] (탐식 공명 수/2)만큼 파열 부여
+코인 1: [적중시] 다음 턴에 탐식 취약 2 부여
+코인 1: [적중시] 다음 턴에 속박 2 부여</v>
+      </c>
+      <c r="H90" t="str">
         <v>./images/ego/23.webp</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" xml:space="preserve">
       <c r="A91">
         <v>22</v>
       </c>
@@ -30069,11 +30957,16 @@
       <c r="F91" t="str">
         <v>탐식 x3, 우울 x2, 질투 x2</v>
       </c>
-      <c r="G91" t="str">
+      <c r="G91" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [앞면 공격 종료 시] 체력 비율이 가장 낮은 아군 2명의 체력 15 회복
+코인 1: [뒷면 공격 종료 시] 정신력이 가장 낮은 아군 2명의 정신력 15 회복
+코인 1: [크리티컬 공격 종료 시] 체력 비율이 가장 낮은 아군 1명의 체력 8 회복, 정신력이 가장 낮은 아군 1명의 정신력 8 회복</v>
+      </c>
+      <c r="H91" t="str">
         <v>./images/ego/22.webp</v>
       </c>
     </row>
-    <row r="92">
+    <row r="92" xml:space="preserve">
       <c r="A92">
         <v>21</v>
       </c>
@@ -30092,11 +30985,16 @@
       <c r="F92" t="str">
         <v>탐식 x3, 오만 x3</v>
       </c>
-      <c r="G92" t="str">
+      <c r="G92" t="str" xml:space="preserve">
+        <v xml:space="preserve">가장 뒤에 있는 적 공격 (일반 전투 한정)
+[공격 시작 전] 충전 횟수 5 증가. 다음 턴에 신속 2를 얻음
+코인 1: [적중시] 취약 1, 차원 균열 4 부여</v>
+      </c>
+      <c r="H92" t="str">
         <v>./images/ego/21.webp</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" xml:space="preserve">
       <c r="A93">
         <v>20</v>
       </c>
@@ -30115,11 +31013,15 @@
       <c r="F93" t="str">
         <v>색욕 x4, 질투 x2</v>
       </c>
-      <c r="G93" t="str">
+      <c r="G93" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 수비 위력 감소 2 부여
+코인 1: [적중시] 방어 레벨 감소 5 부여</v>
+      </c>
+      <c r="H93" t="str">
         <v>./images/ego/20.webp</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" xml:space="preserve">
       <c r="A94">
         <v>19</v>
       </c>
@@ -30138,11 +31040,16 @@
       <c r="F94" t="str">
         <v>색욕 x1, 우울 x5</v>
       </c>
-      <c r="G94" t="str">
+      <c r="G94" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 종료시] 정신력 15 회복
+코인 1: [적중시] 침잠 5 부여
+코인 1: [공격 종료시] 다음 턴에 모든 아군의 정신력 감소 효율 -2, E.G.O 사용시 정신력 감소량 -2</v>
+      </c>
+      <c r="H94" t="str">
         <v>./images/ego/19.webp</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" xml:space="preserve">
       <c r="A95">
         <v>18</v>
       </c>
@@ -30161,11 +31068,15 @@
       <c r="F95" t="str">
         <v>탐식 x3, 질투 x2</v>
       </c>
-      <c r="G95" t="str">
+      <c r="G95" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 다음 턴에 화상, 출혈, 진동, 파열, 침잠 중 무작위 1개 효과의 위력을 (2 + (최대 탐식 완전 공명의 수))회 부여 (최대 7)
+코인 1: [적 처치 시] 무작위 아군 2명에게 다음 턴에 호흡 횟수 2, 충전 횟수 2, 신속 2, 공격 레벨 증가 2, 방어 레벨 증가 2 중 무작위 1개 효과를 부여</v>
+      </c>
+      <c r="H95" t="str">
         <v>./images/ego/18.webp</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" xml:space="preserve">
       <c r="A96">
         <v>17</v>
       </c>
@@ -30184,11 +31095,16 @@
       <c r="F96" t="str">
         <v>분노 x2, 색욕 x2, 나태 x2, 우울 x2</v>
       </c>
-      <c r="G96" t="str">
+      <c r="G96" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 자신의 정신력이 15 이상이면 공격 가중치 +2
+코인 1: [적중시] 다음 턴에 공격 위력 감소 2 부여
+코인 1: [공격 종료 시] 자신을 제외하고 정신력이 가장 낮은 아군 4명의 정신력 25 회복</v>
+      </c>
+      <c r="H96" t="str">
         <v>./images/ego/17.webp</v>
       </c>
     </row>
-    <row r="97">
+    <row r="97" xml:space="preserve">
       <c r="A97">
         <v>16</v>
       </c>
@@ -30207,11 +31123,16 @@
       <c r="F97" t="str">
         <v>우울 x3, 질투 x2</v>
       </c>
-      <c r="G97" t="str">
+      <c r="G97" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 자신의 잃은 체력의 10%당 충전 횟수 1 증가 (최대 7)
+다음 턴에 신속 2를 얻음
+코인 1: [적중시] 마비 3, 우울 취약 1 부여</v>
+      </c>
+      <c r="H97" t="str">
         <v>./images/ego/16.webp</v>
       </c>
     </row>
-    <row r="98">
+    <row r="98" xml:space="preserve">
       <c r="A98">
         <v>15</v>
       </c>
@@ -30230,11 +31151,16 @@
       <c r="F98" t="str">
         <v>분노 x3, 색욕 x2, 질투 x3</v>
       </c>
-      <c r="G98" t="str">
+      <c r="G98" t="str" xml:space="preserve">
+        <v xml:space="preserve">[사용시] 질투 공명 수만큼 자신의 충전 횟수 증가
+충전 횟수 5를 소모할 때마다 스킬 위력 +3 (최대 12)
+코인 1: [뒷면 적중시] 자신의 충전 횟수 5 증가</v>
+      </c>
+      <c r="H98" t="str">
         <v>./images/ego/15.webp</v>
       </c>
     </row>
-    <row r="99">
+    <row r="99" xml:space="preserve">
       <c r="A99">
         <v>14</v>
       </c>
@@ -30253,11 +31179,16 @@
       <c r="F99" t="str">
         <v>색욕 x2, 질투 x2</v>
       </c>
-      <c r="G99" t="str">
+      <c r="G99" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 다음 턴에 공격 위력 증가 1 얻음
+코인 1: [적중시] 다음 턴에 신속 3 얻음
+코인 1: [적 처치 시] 다음 턴에 공격 위력 증가 2 얻음</v>
+      </c>
+      <c r="H99" t="str">
         <v>./images/ego/14.webp</v>
       </c>
     </row>
-    <row r="100">
+    <row r="100" xml:space="preserve">
       <c r="A100">
         <v>13</v>
       </c>
@@ -30276,11 +31207,15 @@
       <c r="F100" t="str">
         <v>우울 x3, 질투 x3</v>
       </c>
-      <c r="G100" t="str">
+      <c r="G100" t="str" xml:space="preserve">
+        <v xml:space="preserve">[공격 시작 전] 자신의 충전 횟수 10 증가
+코인 1: [적중시] 방출 전류 15 부여</v>
+      </c>
+      <c r="H100" t="str">
         <v>./images/ego/13.webp</v>
       </c>
     </row>
-    <row r="101">
+    <row r="101" xml:space="preserve">
       <c r="A101">
         <v>12</v>
       </c>
@@ -30299,7 +31234,12 @@
       <c r="F101" t="str">
         <v>나태 x1, 탐식 x3</v>
       </c>
-      <c r="G101" t="str">
+      <c r="G101" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 진동 폭발
+코인 1: [적중시] 진동 6 부여
+코인 1: [적중시] 마비 4 부여</v>
+      </c>
+      <c r="H101" t="str">
         <v>./images/ego/12.webp</v>
       </c>
     </row>
@@ -30323,6 +31263,9 @@
         <v>나태 x1, 탐식 x4</v>
       </c>
       <c r="G102" t="str">
+        <v>코인 1: [적중시] 피해량의 60%만큼 자신의 체력 회복</v>
+      </c>
+      <c r="H102" t="str">
         <v>./images/ego/11.webp</v>
       </c>
     </row>
@@ -30346,10 +31289,13 @@
         <v>색욕 x3, 우울 x1</v>
       </c>
       <c r="G103" t="str">
+        <v>코인 1: [적중시] 화상, 출혈, 진동, 파열, 침잠 중 무작위 1개 효과 10 부여</v>
+      </c>
+      <c r="H103" t="str">
         <v>./images/ego/10.webp</v>
       </c>
     </row>
-    <row r="104">
+    <row r="104" xml:space="preserve">
       <c r="A104">
         <v>9</v>
       </c>
@@ -30368,11 +31314,21 @@
       <c r="F104" t="str">
         <v>색욕 x1, 탐식 x3, 오만 x1</v>
       </c>
-      <c r="G104" t="str">
+      <c r="G104" t="str" xml:space="preserve">
+        <v xml:space="preserve">스킬 사용 시 필요한 탐식 E.G.O 자원 1 감소
+[공격 시작 전] (최대 공명 수)가 4 이상이면 공격 가중치 +1
+(최대 공명 수)가 6 이상이면, 추가로 공격 가중치 +1
+[공격 시작 전] 모든 공격 대상과 자신의 화상 위력의 합 1당, 피해량 +5% (최대 100%)
+코인 1: [적중시] 화상 3 부여
+코인 1: [적중시] 방어 레벨 감소 5 부여
+코인 1: [적중시] 대상의 화상 2를 방어 레벨 감소 1로 전환 (최대 5. 이 효과로 대상의 화상 위력이 1 미만이 되지 않음)
+코인 1: - 자신의 30을 초과하는 화상을 대상의 화상이 부족한 만큼 대신 전환 가능</v>
+      </c>
+      <c r="H104" t="str">
         <v>./images/ego/9.webp</v>
       </c>
     </row>
-    <row r="105">
+    <row r="105" xml:space="preserve">
       <c r="A105">
         <v>8</v>
       </c>
@@ -30391,11 +31347,16 @@
       <c r="F105" t="str">
         <v>분노 x1, 색욕 x3, 질투 x2</v>
       </c>
-      <c r="G105" t="str">
+      <c r="G105" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 마비 3 부여
+코인 1: [공격 종료시] 자신의 충전 횟수 7 증가
+코인 1: [앞면 공격 종료 시] 다음 턴에 무작위 아군 2명에게 질투 위력 증가 1, 신속 1 부여, 자신의 충전 횟수 3 증가</v>
+      </c>
+      <c r="H105" t="str">
         <v>./images/ego/8.webp</v>
       </c>
     </row>
-    <row r="106">
+    <row r="106" xml:space="preserve">
       <c r="A106">
         <v>7</v>
       </c>
@@ -30414,11 +31375,16 @@
       <c r="F106" t="str">
         <v>색욕 x2, 우울 x4, 질투 x3</v>
       </c>
-      <c r="G106" t="str">
+      <c r="G106" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [공격 종료시] 아군 전체 정신력 15 회복
+코인 1: [공격 종료시] 아군 전체 최대 체력의 15%만큼 체력 회복
+코인 1: [앞면 공격 종료 시] 아군 전체 정신력 10 회복</v>
+      </c>
+      <c r="H106" t="str">
         <v>./images/ego/7.webp</v>
       </c>
     </row>
-    <row r="107">
+    <row r="107" xml:space="preserve">
       <c r="A107">
         <v>6</v>
       </c>
@@ -30437,7 +31403,14 @@
       <c r="F107" t="str">
         <v>질투 x6</v>
       </c>
-      <c r="G107" t="str">
+      <c r="G107" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 관통 취약 3 부여
+코인 1: [적중시] 질투 취약 1 부여
+코인 1: [앞면 적중시] 저주 3 부여
+코인 1: [앞면 적중시] 못 3 부여
+코인 1: [적중시] 대상에게 저주가 있으면 피해량 +50%</v>
+      </c>
+      <c r="H107" t="str">
         <v>./images/ego/6.webp</v>
       </c>
     </row>
@@ -30461,10 +31434,13 @@
         <v>탐식 x2, 오만 x4</v>
       </c>
       <c r="G108" t="str">
+        <v>코인 1: [공격 종료시] 정신력이 가장 낮은 아군 4명의 정신력 12 회복</v>
+      </c>
+      <c r="H108" t="str">
         <v>./images/ego/5.webp</v>
       </c>
     </row>
-    <row r="109">
+    <row r="109" xml:space="preserve">
       <c r="A109">
         <v>4</v>
       </c>
@@ -30483,11 +31459,18 @@
       <c r="F109" t="str">
         <v>색욕 x5</v>
       </c>
-      <c r="G109" t="str">
+      <c r="G109" t="str" xml:space="preserve">
+        <v xml:space="preserve">메인 타겟의 화상과 출혈의 합 4당 최종 위력 +1 (최대 3)
+[공격 시작 전] 보유한 색욕 E.G.O 자원 6당 편성 순서 순으로 다음 턴에 색욕 위력 증가 1 부여 (최대 5명)
+[공격 시작 전] 보유한 색욕 E.G.O 자원 1개당 피해량 +6% (최대 120%)
+코인 1: [적중시] 화상 횟수 3 증가
+코인 1: [적중시] 출혈 횟수 3 증가</v>
+      </c>
+      <c r="H109" t="str">
         <v>./images/ego/4.webp</v>
       </c>
     </row>
-    <row r="110">
+    <row r="110" xml:space="preserve">
       <c r="A110">
         <v>3</v>
       </c>
@@ -30506,11 +31489,15 @@
       <c r="F110" t="str">
         <v>분노 x1, 우울 x2, 질투 x2</v>
       </c>
-      <c r="G110" t="str">
+      <c r="G110" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 충전 횟수 10을 얻음
+코인 1: [공격 종료시] 질투 공명 수에 비례하여 모든 아군에게 충전 횟수 부여</v>
+      </c>
+      <c r="H110" t="str">
         <v>./images/ego/3.webp</v>
       </c>
     </row>
-    <row r="111">
+    <row r="111" xml:space="preserve">
       <c r="A111">
         <v>2</v>
       </c>
@@ -30529,11 +31516,17 @@
       <c r="F111" t="str">
         <v>색욕 x1, 우울 x4, 오만 x2</v>
       </c>
-      <c r="G111" t="str">
+      <c r="G111" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 진동 폭발
+코인 1: [적중시] 대상에게 정신력 25 피해
+코인 1: 대상이 흐트러짐, 사기 저하, 패닉 상태라면 피해량의 30%만큼 추가 피해
+코인 1: [적중시] 침잠 2 부여</v>
+      </c>
+      <c r="H111" t="str">
         <v>./images/ego/2.webp</v>
       </c>
     </row>
-    <row r="112">
+    <row r="112" xml:space="preserve">
       <c r="A112">
         <v>1</v>
       </c>
@@ -30552,11 +31545,15 @@
       <c r="F112" t="str">
         <v>색욕 x2, 오만 x2</v>
       </c>
-      <c r="G112" t="str">
+      <c r="G112" t="str" xml:space="preserve">
+        <v xml:space="preserve">코인 1: [적중시] 출혈 8 부여
+코인 1: [적중시] 피해량의 50%만큼 체력 회복</v>
+      </c>
+      <c r="H112" t="str">
         <v>./images/ego/1.webp</v>
       </c>
     </row>
-    <row r="113">
+    <row r="113" xml:space="preserve">
       <c r="A113" t="str">
         <v>128</v>
       </c>
@@ -30575,11 +31572,21 @@
       <c r="F113" t="str">
         <v>분노 x2, 나태 x2, 우울 x1, 오만 x1</v>
       </c>
-      <c r="G113" t="str">
+      <c r="G113" t="str" xml:space="preserve">
+        <v xml:space="preserve">자신의 호흡 위력과 메인 타겟의 진동 위력의 합 6당, 합 위력 +1 (최대 4)
+[공격 시작 전] (4 + 최대 공명 수)만큼 호흡 얻음 (최대 8)
+[공격 시작 전] 자신의 호흡 횟수 4 증가
+[공격 종료시] 공격 대상 중 무작위 적에게 (1 + 최대 공명 수)만큼 감각 균열을 1씩 나누어 부여 (최대 5)
+코인 1: [적중시] 진동 4 부여
+코인 2: [적중시] 진동 횟수 3 증가
+코인 3: [적중시] 공격 레벨 감소 2 부여
+코인 3: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소</v>
+      </c>
+      <c r="H113" t="str">
         <v>./images/ego/128.webp</v>
       </c>
     </row>
-    <row r="114">
+    <row r="114" xml:space="preserve">
       <c r="A114" t="str">
         <v>129</v>
       </c>
@@ -30598,11 +31605,18 @@
       <c r="F114" t="str">
         <v>색욕 x2, 오만 x1, 질투 x2</v>
       </c>
-      <c r="G114" t="str">
+      <c r="G114" t="str" xml:space="preserve">
+        <v xml:space="preserve">[사용시] 자신의 충전 위력만큼 합 위력 증가 (최대 3)
+[공격 시작 전] 자신의 충전 횟수 5 증가
+[공격 시작 전] 자신의 충전 횟수를 최대 10까지 소모하고, 자신과 자신을 제외한 아군 최대 (1 + 소모한 충전 횟수/2)명에게 충전 역장 5 부여 (최대 7명, 소수점 버림)
+코인 1: [적중시] 자신의 충전 횟수 2 증가
+코인 2: [적중시] 광전 2 부여</v>
+      </c>
+      <c r="H114" t="str">
         <v>./images/ego/129.webp</v>
       </c>
     </row>
-    <row r="115">
+    <row r="115" xml:space="preserve">
       <c r="A115" t="str">
         <v>130</v>
       </c>
@@ -30621,11 +31635,22 @@
       <c r="F115" t="str">
         <v>우울 x2, 오만 x4, 질투 x2</v>
       </c>
-      <c r="G115" t="str">
+      <c r="G115" t="str" xml:space="preserve">
+        <v xml:space="preserve">[합 불가능]
+전투에서 처음 사용 시 정신력 소모량이 5 감소하고, 필요한 E.G.O 자원이 우울 2, 오만 2, 질투 2 감소
+잿빛 탄환이 1 이상이면, '부셰'로 발동됨
+이 스킬은 적에게 적중하지 않고, 수비 스킬을 발동시키지 않으며, 외부 효과로 재사용이 불가능함
+[공격 종료시] 잿빛 탄환 5 얻음
+[공격 종료시] 호흡 위력 5 얻음
+[공격 종료시] 호흡 횟수 3 얻음
+[공격 종료시] 충전 횟수 5 얻음
+[공격 종료시] 검은 날개 4 얻음</v>
+      </c>
+      <c r="H115" t="str">
         <v>./images/ego/130.webp</v>
       </c>
     </row>
-    <row r="116">
+    <row r="116" xml:space="preserve">
       <c r="A116" t="str">
         <v>131</v>
       </c>
@@ -30644,14 +31669,38 @@
       <c r="F116" t="str">
         <v>나태 x2, 우울 x2, 오만 x4, 질투 x4</v>
       </c>
-      <c r="G116" t="str">
+      <c r="G116" t="str" xml:space="preserve">
+        <v xml:space="preserve">스킬 시전 중 공격 대상 사망 시, 체력이 가장 낮은 공격 대상을 우선 지정 (집중 전투의 경우, 부위로 판정)
+(자신의 호흡 위력 + 충전 횟수) 4당 합 위력 +1 (최대 10)
+자신의 잿빛 탄환 1당 합 위력 +2
+[공격 시작 전] 자신의 호흡 횟수 3, 충전 횟수 5 증가
+[공격 시작 전] 정신력을 (5-보유한 잿빛 탄환) × 3 만큼 소모하여, 잿빛 탄환을 최대치로 얻음
+[공격 종료시] 검은 날개 2 얻음
+코인 1: 파괴 불가 코인
+코인 1: 이 코인은 메인 타겟에게만 적중함
+코인 1: 잿빛 탄환 1 소모
+코인 1: 크리티컬 피해량 +20%
+코인 1: 처음 사용한 코인이면,
+코인 1: - 피해량 +(자신의 충전 횟수 × 5)% (최대 100%)
+코인 1: - 크리티컬 피해량 +(자신의 호흡 위력 × 횟수)% (최대 100%)
+코인 1: - 해당 코인에 한해 대상의 관통 속성 내성을 취약으로 변경함
+코인 1: [적중시] 관통 취약 1 부여 (스킬당 1회)
+코인 1: [적중시] 침잠 1 부여
+코인 1: [크리티컬 적중 시] 마지막 코인 위력 +1
+코인 1: [이 코인 공격 종료 시] 잿빛 탄환이 1 이상이면 이 코인 재사용 (스킬당 4회)
+코인 2: 파괴 불가 코인
+코인 2: 크리티컬 피해량 +50%
+코인 2: [코인 시작 시] 공격 대상이 1명이면, 피해량 +100% (집중 전투의 경우, 본체로 판정)
+코인 2: [코인 시작 시] 자신의 충전 횟수 4당 코인 위력 +1 (최대 5)
+코인 2: [적중시] 침잠 횟수 3 증가</v>
+      </c>
+      <c r="H116" t="str">
         <v>./images/ego/131.webp</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G116"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H116"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add keyword hint to the EGO quiz
Collects the awakening skill's keyword badges (e.g. 출혈 (부여),
호흡 (강화)) from limbusdeck.com alongside the effect text, stores them
in the EGOData 키워드 column, and shows them as a paid hint and on the
result screen. EGOs without badges show 없음.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CharacterTable.xlsx
+++ b/CharacterTable.xlsx
@@ -28089,7 +28089,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H116"/>
+  <dimension ref="A1:I116"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -28111,9 +28111,12 @@
         <v>자원</v>
       </c>
       <c r="G1" t="str">
+        <v>키워드</v>
+      </c>
+      <c r="H1" t="str">
         <v>효과</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>아이콘</v>
       </c>
     </row>
@@ -28136,7 +28139,10 @@
       <c r="F2" t="str">
         <v>질투 x5</v>
       </c>
-      <c r="G2" t="str" xml:space="preserve">
+      <c r="G2" t="str">
+        <v>출혈 (부여)</v>
+      </c>
+      <c r="H2" t="str" xml:space="preserve">
         <v xml:space="preserve">[합 승리 후 공격 종료 시] 현재 체력 비율이 가장 낮은 아군 (2 + 질투 공명 수 / 2)명의 체력을 각자의 최대 체력 6%만큼 회복하고 정신력 5 회복 (최대 4명)
 [합 패배] (질투 공명 수 × 5)만큼 보호막 얻음 (최대 30)
 [합 패배] 메인 타겟에게 가하는 피해량 +200%
@@ -28144,7 +28150,7 @@
 코인 1: [합 승리 후 적중시] 다음 턴에 위력 감소 1 부여 (대상 별 턴당 1회)
 코인 1: [적중시] 출혈 4 부여</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>./images/ego/127.png</v>
       </c>
     </row>
@@ -28167,7 +28173,10 @@
       <c r="F3" t="str">
         <v>나태 x1, 우울 x4, 오만 x2</v>
       </c>
-      <c r="G3" t="str" xml:space="preserve">
+      <c r="G3" t="str">
+        <v>침잠 (부여), 진동 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H3" t="str" xml:space="preserve">
         <v xml:space="preserve">광역 난사
 이 스킬의 효과로 무작위 나비 부여시 앞면이 나올 확률로 죽은나비를 부여. 부여하지 않은 경우, 산나비를 부여. (나비 1당 개별 판정)
 메인 타겟의 침잠과 모든 나비의 합 4당, 합 위력 +1 (최대 4)
@@ -28199,7 +28208,7 @@
 코인 5: [적중시] 대상의 모든 나비만큼 우울 피해
 코인 5: [적중시] 이 코인 최종 피해량의 (이 코인에서 소모한 산나비·죽은나비 × 2)%만큼 우울 피해</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>./images/ego/126.webp</v>
       </c>
     </row>
@@ -28222,7 +28231,10 @@
       <c r="F4" t="str">
         <v>분노 x1, 오만 x4, 질투 x1</v>
       </c>
-      <c r="G4" t="str" xml:space="preserve">
+      <c r="G4" t="str">
+        <v>출혈 (부여), 호흡 (강화)</v>
+      </c>
+      <c r="H4" t="str" xml:space="preserve">
         <v xml:space="preserve">전투에서 처음 사용 시 정신력 소모량 15 감소
 - 검계 우두머리 뫼르소면, 필요한 E.G.O 자원이 분노 1, 오만 1, 질투 1 감소
 자신의 호흡 4당, 합 위력 +1, 피해량 +6% (각각 최대 8, 30%)
@@ -28235,7 +28247,7 @@
 코인 1: [적중시] 출혈 4 부여
 코인 2: [적중시] 출혈 횟수 2 증가</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>./images/ego/125.webp</v>
       </c>
     </row>
@@ -28258,7 +28270,10 @@
       <c r="F5" t="str">
         <v>분노 x2, 색욕 x3</v>
       </c>
-      <c r="G5" t="str" xml:space="preserve">
+      <c r="G5" t="str">
+        <v>화상 (부여), 출혈 (부여)</v>
+      </c>
+      <c r="H5" t="str" xml:space="preserve">
         <v xml:space="preserve">[사용시] 모든 대상의 화상과 출혈의 합 6당 합 위력 +1 (최대 2)
 [공격 종료시] 현재 체력 비율이 가장 낮은 아군 2명의 체력을 최대 체력의 10%만큼 회복하고 주홍 나방 2 부여 (최소 체력 회복량: 1)
 - (색욕 공명 수 - 1)만큼 회복 대상 수 증가 (최대 2명)
@@ -28267,7 +28282,7 @@
 코인 1: [적중시] 출혈 3 부여
 코인 1: [이 코인 공격 종료 시] 적중한 대상에게 다음 턴에 분노 취약 1, 색욕 취약 1 부여</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
         <v>./images/ego/124.webp</v>
       </c>
     </row>
@@ -28290,7 +28305,10 @@
       <c r="F6" t="str">
         <v>분노 x3, 나태 x2, 오만 x2</v>
       </c>
-      <c r="G6" t="str" xml:space="preserve">
+      <c r="G6" t="str">
+        <v>화상 (부여)</v>
+      </c>
+      <c r="H6" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 모든 공격 대상과 자신의 화상 위력의 합 10당 최종 위력 +1 (최대 2)
 [공격 종료시] 화상 10 얻음, 자신의 화상 횟수 1 증가
 [공격 종료시] 자신의 화상이 15 이상이면, 다음 턴에 분노 피해량 증가 1 얻음 (턴당 1회)
@@ -28299,7 +28317,7 @@
 코인 2: [적중시] (분노 공명 수 / 3)만큼 화상 횟수 증가 (최대 2, 소수점 버림)
 코인 2: [이 코인 공격 종료시] 자신의 화상이 15 이상이면, 모든 공격 대상에게 잔불 1 부여 (턴당 1회, 집중 전투인 경우 부위로 취급)</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>./images/ego/123.webp</v>
       </c>
     </row>
@@ -28322,7 +28340,10 @@
       <c r="F7" t="str">
         <v>분노 x3, 색욕 x2, 나태 x1, 오만 x1, 질투 x1</v>
       </c>
-      <c r="G7" t="str" xml:space="preserve">
+      <c r="G7" t="str">
+        <v>출혈 (부여), 화상 (부여)</v>
+      </c>
+      <c r="H7" t="str" xml:space="preserve">
         <v xml:space="preserve">메인 타겟의 출혈과 화상의 합 2당, 합 위력 +1 (최대 10)
 자신의 잃은 체력 비율만큼 피해량 증가 (최대 20%)
 서브 타겟에게 가하는 피해량 -50%
@@ -28338,7 +28359,7 @@
 코인 3: [적중시] 출혈 1 부여
 코인 3: [적중시] 무작위 아군 1명이 다음 턴에 리듬 1 ~ 3 얻음 (코인당 1회)</v>
       </c>
-      <c r="H7" t="str">
+      <c r="I7" t="str">
         <v>./images/ego/122.webp</v>
       </c>
     </row>
@@ -28361,7 +28382,10 @@
       <c r="F8" t="str">
         <v>분노 x4, 색욕 x4, 오만 x4</v>
       </c>
-      <c r="G8" t="str" xml:space="preserve">
+      <c r="G8" t="str">
+        <v>화상 (부여), 출혈 (부여), 호흡 (강화)</v>
+      </c>
+      <c r="H8" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 최대 공명 수만큼 호흡 얻음 (최대 7)
 [공격 시작 전] 자신의 호흡 횟수 3 증가
 [공격 종료시] 나생 [羅生] 1 얻음
@@ -28379,7 +28403,7 @@
 코인 3: [코인 시작 시] 자신의 나생 [羅生] 을 모두 소모하고, 소모한 수치 5당 피해량 +1% (최대 198%)
 코인 3: - 공격 대상이 1명이면, 이 효과가 2배로 적용됨 (집중 전투인 경우, 본체를 기준으로 판정)</v>
       </c>
-      <c r="H8" t="str">
+      <c r="I8" t="str">
         <v>./images/ego/121.webp</v>
       </c>
     </row>
@@ -28402,7 +28426,10 @@
       <c r="F9" t="str">
         <v>분노 x4, 우울 x2, 오만 x2, 질투 x4</v>
       </c>
-      <c r="G9" t="str" xml:space="preserve">
+      <c r="G9" t="str">
+        <v>침잠 (부여), 화상 (부여)</v>
+      </c>
+      <c r="H9" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 메인 대상의 화상과 침잠의 합이 10 이상이면, 코인 위력 +1
 [공격 시작 전] 최대 공명 수만큼 호흡 얻음 (최대 7)
 - 해당 공명이 완전 공명이면, (최대 공명 수) / 3만큼 추가로 호흡 횟수 증가 (최대 2, 소수점 버림)
@@ -28417,7 +28444,7 @@
 코인 4: 파괴 불가 코인
 코인 4: [파괴되지 않고 적중시] 화상 1회 발동. 화상 횟수 1 감소</v>
       </c>
-      <c r="H9" t="str">
+      <c r="I9" t="str">
         <v>./images/ego/120.webp</v>
       </c>
     </row>
@@ -28440,7 +28467,10 @@
       <c r="F10" t="str">
         <v>분노 x2, 탐식 x1, 질투 x3</v>
       </c>
-      <c r="G10" t="str" xml:space="preserve">
+      <c r="G10" t="str">
+        <v>화상 (부여), 충전 (강화)</v>
+      </c>
+      <c r="H10" t="str" xml:space="preserve">
         <v xml:space="preserve">메인 타겟의 화상 6당 코인 위력 +1 (최대 3)
 [공격 시작 전] (최대 공명 수 + 1)만큼 자신의 충전 횟수 증가 (최대 7)
 - 질투 공명이 4 이상이면, 대신 자신의 충전 횟수 7 증가
@@ -28452,7 +28482,7 @@
 코인 3: [적중시] 주민등록 마이크로 칩 2 부여
 코인 3: [적중시] 자신의 충전 횟수 1~3 증가</v>
       </c>
-      <c r="H10" t="str">
+      <c r="I10" t="str">
         <v>./images/ego/119.png</v>
       </c>
     </row>
@@ -28475,7 +28505,10 @@
       <c r="F11" t="str">
         <v>색욕 x1, 질투 x3</v>
       </c>
-      <c r="G11" t="str" xml:space="preserve">
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str" xml:space="preserve">
         <v xml:space="preserve">일방 공격 시 이 스킬의
 [파괴되지 않고 적중시] 효과가 발동하지 않음
 [합 승리시] 질투 공명 수만큼 질투 E.G.O 자원을 소모하고 소모한 자원 1당, 제일 적은 E.G.O 자원을 1씩 나누어 얻음 (최대 소모량 6)
@@ -28487,7 +28520,7 @@
 코인 1: [적중시] 저주 1 부여
 코인 1: [적중시] 못 1 부여</v>
       </c>
-      <c r="H11" t="str">
+      <c r="I11" t="str">
         <v>./images/ego/118.webp</v>
       </c>
     </row>
@@ -28510,7 +28543,10 @@
       <c r="F12" t="str">
         <v>분노 x2, 나태 x3, 오만 x2</v>
       </c>
-      <c r="G12" t="str" xml:space="preserve">
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str" xml:space="preserve">
         <v xml:space="preserve">[합 불가능]
 전투에서 처음 사용시 필요한 E.G.O 자원이 분노 1, 나태 2, 오만 1 감소
 칼집 속 사람이 1 이상이면, 눈부시지 않은 영광 - 광휘(光輝)로 발동됨
@@ -28519,7 +28555,7 @@
 [공격 종료시] 정신력 25 회복
 [공격 종료시] 다음 턴에 공격 레벨 증가 2, 피해량 증가 1 얻음</v>
       </c>
-      <c r="H12" t="str">
+      <c r="I12" t="str">
         <v>./images/ego/117.webp</v>
       </c>
     </row>
@@ -28542,7 +28578,10 @@
       <c r="F13" t="str">
         <v>나태 x1, 탐식 x5, 오만 x2</v>
       </c>
-      <c r="G13" t="str" xml:space="preserve">
+      <c r="G13" t="str">
+        <v>파열 (부여), 화상 (부여)</v>
+      </c>
+      <c r="H13" t="str" xml:space="preserve">
         <v xml:space="preserve">메인 타겟에게 화상 또는 파열이 있으면, 최종 위력 +3
 [공격 시작 전] 메인 타겟의 파열 위력과 파열 횟수의 합 1당 피해량 +1% (최대 25%)
 경화막이 있으면, 이 효과와 최댓값이 2배로 증가
@@ -28553,7 +28592,7 @@
 코인 1: [적중시] 파열 3 부여
 코인 1: [적중시] 화상 3 부여</v>
       </c>
-      <c r="H13" t="str">
+      <c r="I13" t="str">
         <v>./images/ego/116.webp</v>
       </c>
     </row>
@@ -28576,7 +28615,10 @@
       <c r="F14" t="str">
         <v>나태 x1, 우울 x2, 오만 x4</v>
       </c>
-      <c r="G14" t="str" xml:space="preserve">
+      <c r="G14" t="str">
+        <v>침잠 (부여), 호흡 (강화)</v>
+      </c>
+      <c r="H14" t="str" xml:space="preserve">
         <v xml:space="preserve">[사용시] 호흡 4 얻음
 [공격 시작 전] 호흡 위력과 호흡 횟수의 합 5당, 최종 위력 +1 (최대 3)
 [공격 시작 전] 시엔징, 상급 시엔징이 없으면, 이 스킬에서 소모한 E.G.O 자원과 정신력을 절반만큼 돌려받음 (소수점 버림. 이 효과는 각성 스킬 사용 시 침식되는 경우에도 적용됨)
@@ -28588,7 +28630,7 @@
 코인 2: 상급 시엔징이 있으면, 크리티컬 피해량 +(호흡 위력과 호흡 횟수의 합)% (최대 40%)
 코인 2: [적중시] 침잠 3 부여</v>
       </c>
-      <c r="H14" t="str">
+      <c r="I14" t="str">
         <v>./images/ego/115.webp</v>
       </c>
     </row>
@@ -28611,7 +28653,10 @@
       <c r="F15" t="str">
         <v>우울 x4, 오만 x2</v>
       </c>
-      <c r="G15" t="str" xml:space="preserve">
+      <c r="G15" t="str">
+        <v>침잠 (부여), 진동 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H15" t="str" xml:space="preserve">
         <v xml:space="preserve">공격 대상이 1명이면, 코인 위력 +2, 피해량 +100% (집중 전투인 경우, 본체를 기준으로 판정)
 [사용시] 메인 타겟의 침잠 4 당 합 위력 +1 (최대 2)
 [공격 시작 전] 메인 타겟의 우울 내성이 1을 초과하면, 초과하는 값 0.1 당 피해량 +5% (최대 20%)
@@ -28627,7 +28672,7 @@
 코인 3: 공격 대상이 1명이면, 대신 3명에게 부여
 코인 3: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소</v>
       </c>
-      <c r="H15" t="str">
+      <c r="I15" t="str">
         <v>./images/ego/114.webp</v>
       </c>
     </row>
@@ -28650,7 +28695,10 @@
       <c r="F16" t="str">
         <v>분노 x2, 색욕 x2, 나태 x6, 질투 x1</v>
       </c>
-      <c r="G16" t="str" xml:space="preserve">
+      <c r="G16" t="str">
+        <v>진동 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H16" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 메인 타겟의 (진동 위력 + 진동 횟수)가 30 이상이면 가중치 +1
 - 100 이상이면, 대신 가중치 +3
 [공격 시작 전] 최대 공명 수 2 당, 공격하는 모든 대상에게 진동 1 부여 (최대 3)
@@ -28667,7 +28715,7 @@
 코인 4: [적중시] 이 코인의 효과로 인한 피해량 증가량이 50% 이상이면, 진동 폭발 1회.
 코인 4: [적중시] 이 코인의 효과로 인한 피해량 증가량이 100% 이상이면, 진동 폭발 2회. 진동 횟수 2 감소</v>
       </c>
-      <c r="H16" t="str">
+      <c r="I16" t="str">
         <v>./images/ego/103.webp</v>
       </c>
     </row>
@@ -28690,7 +28738,10 @@
       <c r="F17" t="str">
         <v>분노 x2, 우울 x2, 오만 x2, 질투 x6</v>
       </c>
-      <c r="G17" t="str" xml:space="preserve">
+      <c r="G17" t="str">
+        <v>파열 (부여), 충전 (강화)</v>
+      </c>
+      <c r="H17" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 자신을 제외한 무작위 아군 1 + (질투 공명 수 / 2)명에게 마법소녀의 영창 1 부여 (최대 4명)
 - 자신에게 마법소녀 등장!이 있으면, 대신하여 무작위 아군 1 + (질투 공명 수 / 2)명에게 마법소녀의 영창 2 부여 (최대 4명)
 [공격 시작 전] (충전 - 1)만큼 공격 가중치 증가 (최대 5)
@@ -28704,7 +28755,7 @@
 코인 2: [적중시] 파열을 (충전 - 1)만큼 부여 (최대 4)
 코인 2: - 자신에게 마법소녀 등장!이 있으면, 파열 횟수 1 증가</v>
       </c>
-      <c r="H17" t="str">
+      <c r="I17" t="str">
         <v>./images/ego/102.webp</v>
       </c>
     </row>
@@ -28727,14 +28778,17 @@
       <c r="F18" t="str">
         <v>탐식 x5, 우울 x1, 질투 x1</v>
       </c>
-      <c r="G18" t="str" xml:space="preserve">
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [합 불가능]
 코인 1: 대상 수비 스킬 무시
 코인 1: 이 스킬은 적에게 적중하지 않음
 코인 1: [공격 종료시] 매화첨 [埋花櫼] 얻음이 스킬의 최종 위력만큼 자신이 고정 피해를 받음
 코인 1: - 이 피해로 흐트러지거나 체력이 1 미만으로 감소하지 않음</v>
       </c>
-      <c r="H18" t="str">
+      <c r="I18" t="str">
         <v>./images/ego/101.webp</v>
       </c>
     </row>
@@ -28757,7 +28811,10 @@
       <c r="F19" t="str">
         <v>색욕 x2, 탐식 x6, 오만 x2</v>
       </c>
-      <c r="G19" t="str" xml:space="preserve">
+      <c r="G19" t="str">
+        <v>파열 (부여)</v>
+      </c>
+      <c r="H19" t="str" xml:space="preserve">
         <v xml:space="preserve">자신의 매화침 [埋花針] 6 당 코인 위력 +1 (최대 3)
 [전투 시작시] 불허 [不許] 얻음
 [공격 시작 전] 탐식 공명 수만큼 매화침 [埋花針] 얻음 (최대 5)
@@ -28770,7 +28827,7 @@
 코인 2: [적중시] 자신의 현재 체력이 최대 체력의 30% 미만이거나, 매화침 [埋花針] 수치가 20이면 이 코인 재사용 (스킬 당 1회)
 코인 2: [재사용 적중시] 자신의 모든 체력을 소모하여 이 코인의 피해량 +20% (턴 당 1회)</v>
       </c>
-      <c r="H19" t="str">
+      <c r="I19" t="str">
         <v>./images/ego/100.webp</v>
       </c>
     </row>
@@ -28793,13 +28850,16 @@
       <c r="F20" t="str">
         <v>나태 x2, 오만 x2</v>
       </c>
-      <c r="G20" t="str" xml:space="preserve">
+      <c r="G20" t="str">
+        <v>침잠 (부여), 파열 (부여)</v>
+      </c>
+      <c r="H20" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 종료시] 자신과 메인 타겟의 부정적인 효과 수의 합만큼 지네 독 부여 (최대 10)
 코인 1: [적중시] 침잠 2 부여
 코인 2: [적중시] 파열 2 부여
 코인 2: [적중시] 탐식 혹은 우울 공명이 4 이상이면, 해당 공명 수만큼 지네 독을 부여 (최대 5)</v>
       </c>
-      <c r="H20" t="str">
+      <c r="I20" t="str">
         <v>./images/ego/99.webp</v>
       </c>
     </row>
@@ -28822,13 +28882,16 @@
       <c r="F21" t="str">
         <v>색욕 x1, 탐식 x5, 우울 x2, 오만 x1</v>
       </c>
-      <c r="G21" t="str" xml:space="preserve">
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 얽혀버린 저주 부적을 4 + (탐식 공명 수)만큼 부여함 (최대 10)
 코인 2: 얽혀버린 저주 부적 당 피해량 +5% (최대 50%)
 코인 2: [적중시] 파열을 (대상의 얽혀버린 저주 부적 / 2)만큼 부여 (최대 4, 소수점 버림)
 코인 2: [적중시] 파열 횟수를 (대상의 얽혀버린 저주 부적 / 4)만큼 부여 (최대 2, 소수점 버림)</v>
       </c>
-      <c r="H21" t="str">
+      <c r="I21" t="str">
         <v>./images/ego/98.webp</v>
       </c>
     </row>
@@ -28851,14 +28914,17 @@
       <c r="F22" t="str">
         <v>분노 x7, 오만 x3</v>
       </c>
-      <c r="G22" t="str" xml:space="preserve">
+      <c r="G22" t="str">
+        <v>화상 (부여)</v>
+      </c>
+      <c r="H22" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] (최대 공명 수 / 2)만큼 공격 가중치 증가 (최대 3, 소수점 버림)
 [공격 종료시] 현재 체력 비율이 가장 낮은 아군 (1 + 최대 공명 수)명의 체력을 최대 체력의 20%만큼 회복 (최대 3명)
 [공격 종료시] 3턴 동안 턴 종료 시 정신력 10 감소
 코인 1: [적중시] 화상 8 부여
 코인 1: [적중시] 메인 타겟이면, 다음 턴에 달궈진 새장 (1 + (분노 공명 수 / 3))만큼 부여 (최대 3, 소수점 버림)</v>
       </c>
-      <c r="H22" t="str">
+      <c r="I22" t="str">
         <v>./images/ego/97.webp</v>
       </c>
     </row>
@@ -28881,12 +28947,15 @@
       <c r="F23" t="str">
         <v>나태 x1, 우울 x1, 오만 x5</v>
       </c>
-      <c r="G23" t="str" xml:space="preserve">
+      <c r="G23" t="str">
+        <v>호흡 (강화)</v>
+      </c>
+      <c r="H23" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 모든 아군에게 호흡 위력을 (최대 공명 수)만큼 부여 (최대 부여량 : 6)
 - 오만 공명 3 이상이면, 부여 대상의 호흡 횟수 1 증가, 부여 대상에게 다음 턴에 가쁜 날숨 1 부여
 코인 1: [적중시] 자신의 호흡 횟수 1 증가크리티컬 피해량 +(호흡 위력과 호흡 횟수의 합)% (최대 40%)</v>
       </c>
-      <c r="H23" t="str">
+      <c r="I23" t="str">
         <v>./images/ego/96.webp</v>
       </c>
     </row>
@@ -28909,7 +28978,10 @@
       <c r="F24" t="str">
         <v>분노 x1, 색욕 x1, 오만 x5</v>
       </c>
-      <c r="G24" t="str" xml:space="preserve">
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 최대 공명 수만큼 호흡 얻음 (최대 6)
 - 호흡이 15 이상이면, 대신 최종 위력 + (최대 공명 수) (최대 6)
 [공격 시작 전] (최대 공명 수/2)만큼 호흡 횟수 증가 (최대 3)
@@ -28918,7 +28990,7 @@
 코인 2: 크리티컬 피해량 +(호흡 위력과 호흡 횟수의 합)% (최대 40%)
 코인 2: [적중시] 깊은 들숨 4 얻음 (턴 당 1회)</v>
       </c>
-      <c r="H24" t="str">
+      <c r="I24" t="str">
         <v>./images/ego/95.webp</v>
       </c>
     </row>
@@ -28941,7 +29013,10 @@
       <c r="F25" t="str">
         <v>분노 x2, 색욕 x2, 오만 x4</v>
       </c>
-      <c r="G25" t="str" xml:space="preserve">
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str" xml:space="preserve">
         <v xml:space="preserve">대상의 화상 수치 3 당 피해량 +3% (최대 30%)
 [공격 시작 전] 마탄이 0이면, 마탄 1 얻음
 - 마탄 수치에 따라 발사할 탄환이 정해짐
@@ -28957,7 +29032,7 @@
 코인 1: [적중시] 마탄만큼 화상 부여
 코인 1: [적중시] 마탄만큼 흑염 부여 (턴 당 대상 1명마다 최대 1회 부여)</v>
       </c>
-      <c r="H25" t="str">
+      <c r="I25" t="str">
         <v>./images/ego/94.webp</v>
       </c>
     </row>
@@ -28980,7 +29055,10 @@
       <c r="F26" t="str">
         <v>나태 x2, 탐식 x2, 우울 x2, 오만 x2</v>
       </c>
-      <c r="G26" t="str" xml:space="preserve">
+      <c r="G26" t="str">
+        <v>진동 (부여), 침잠 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H26" t="str" xml:space="preserve">
         <v xml:space="preserve">대상의 정신력이 0 미만이면, 0 미만의 정신력 1 당 피해량 +1% (최대 45%)
 [공격 종료시] 자신의 체력이 최대치면, 턴 종료 시 정신력을 15 회복하고 다음 턴에 공격 위력 증가 1 얻음
 코인 1: [적중시] 진동 5 부여
@@ -28989,7 +29067,7 @@
 코인 2: [적중시] 침잠 4 부여
 코인 2: [적중시] 대상이 흐트러짐, 사기 저하, 패닉 상태면 다음 턴에 공격 위력 감소 1, 가장 높은 공명 속성의 취약을 1 부여</v>
       </c>
-      <c r="H26" t="str">
+      <c r="I26" t="str">
         <v>./images/ego/93.webp</v>
       </c>
     </row>
@@ -29012,7 +29090,10 @@
       <c r="F27" t="str">
         <v>나태 x4, 탐식 x1, 오만 x2</v>
       </c>
-      <c r="G27" t="str" xml:space="preserve">
+      <c r="G27" t="str">
+        <v>진동 (부여), 침잠 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H27" t="str" xml:space="preserve">
         <v xml:space="preserve">대상의 정신력이 0 미만이면, 0 미만의 정신력 1 당 피해량 +1% (최대 45%)
 [공격 시작 전] (최대 공명 수 + 5)만큼 자신의 진동 횟수 증가 (최대 10)
 [공격 종료시] 공격 대상 중 흐트러짐, 사기 저하, 패닉 상태인 적이 있으면, 정신력 10 회복
@@ -29021,7 +29102,7 @@
 코인 1: [적중시] 대상이 흐트러짐, 사기 저하, 패닉 상태가 아니면, 진동 폭발 2회. 대상의 진동 횟수 2 감소
 코인 2: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소</v>
       </c>
-      <c r="H27" t="str">
+      <c r="I27" t="str">
         <v>./images/ego/92.webp</v>
       </c>
     </row>
@@ -29044,7 +29125,10 @@
       <c r="F28" t="str">
         <v>나태 x2, 우울 x1, 오만 x2, 질투 x2</v>
       </c>
-      <c r="G28" t="str" xml:space="preserve">
+      <c r="G28" t="str">
+        <v>진동 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H28" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] (4 + 최대 공명 수)만큼 자신의 진동 횟수 증가 (최대 8, 턴 당 최대 20)
 - 해당 공명이 나태 공명인 경우, 자신의 진동을 진동 - 태엽감기로 진폭 변환
 코인 1: [적중시] 진동 횟수 1 증가
@@ -29054,7 +29138,7 @@
 코인 2: - 진동 폭발 시 이번 턴에 나태 취약 1 부여
 코인 2: - 최대 공명이 나태 공명 3 이상이면, 다음 턴에도 나태 취약 1 부여</v>
       </c>
-      <c r="H28" t="str">
+      <c r="I28" t="str">
         <v>./images/ego/91.webp</v>
       </c>
     </row>
@@ -29077,7 +29161,10 @@
       <c r="F29" t="str">
         <v>분노 x2, 오만 x6</v>
       </c>
-      <c r="G29" t="str" xml:space="preserve">
+      <c r="G29" t="str">
+        <v>출혈 (부여), 호흡 (강화)</v>
+      </c>
+      <c r="H29" t="str" xml:space="preserve">
         <v xml:space="preserve">체력이 가장 낮은 대상 우선 공격 (아군 우선 지정)
 [공격 시작 전] (최대 공명 수 + 1)만큼 찢어진 추억을 얻음 (최대 7)
 - 해당 공명이 오만 공명이면, 효과를 대신하여 (최대 공명 수 × 2)만큼 찢어진 추억을 얻음 (최대 7)
@@ -29093,7 +29180,7 @@
 코인 2: 찢어진 추억당 크리티컬 피해량 +9% (최대 63%)
 코인 2: [크리티컬 적중 시] 출혈 3 부여</v>
       </c>
-      <c r="H29" t="str">
+      <c r="I29" t="str">
         <v>./images/ego/90.webp</v>
       </c>
     </row>
@@ -29116,7 +29203,10 @@
       <c r="F30" t="str">
         <v>색욕 x5, 탐식 x3, 오만 x2, 질투 x2</v>
       </c>
-      <c r="G30" t="str" xml:space="preserve">
+      <c r="G30" t="str">
+        <v>출혈 (부여)</v>
+      </c>
+      <c r="H30" t="str" xml:space="preserve">
         <v xml:space="preserve">이 스킬을 사용하는 동안은 체력이 1 미만으로 되지 않음.
 대상의 출혈 10 당 코인 위력 +1 (최대 2)
 자신의 누적 소모 혈찬이 100 당, 합 위력 +1 (최대 5)
@@ -29132,7 +29222,7 @@
 코인 4: 공용 누적 소모 혈찬 300 이상이면, 1 당 피해량 +0.1% (최대 50%)
 코인 4: [합 승리 후 적중] 최대 색욕 완전 공명 수에 비례해서 목마른 장미 부여 (최대 4)</v>
       </c>
-      <c r="H30" t="str">
+      <c r="I30" t="str">
         <v>./images/ego/89.webp</v>
       </c>
     </row>
@@ -29155,7 +29245,10 @@
       <c r="F31" t="str">
         <v>색욕 x4, 오만 x3, 질투 x4</v>
       </c>
-      <c r="G31" t="str" xml:space="preserve">
+      <c r="G31" t="str">
+        <v>출혈 (부여)</v>
+      </c>
+      <c r="H31" t="str" xml:space="preserve">
         <v xml:space="preserve">대상의 출혈 6 당 코인 위력 +1 (최대 2)
 [공격 종료시] 3턴 동안 턴 종료 시 정신력 10 감소
 코인 1: [적중시] 출혈 2 부여
@@ -29169,7 +29262,7 @@
 코인 4: [합 승리 후 적중] 대상의 출혈 1 + (최대 공명 수 / 2)회 발동 (최대 3회. 발동한 횟수만큼 출혈 횟수 감소)
 코인 4: [적 처치시] 적의 남은 체력을 초과하여 피해를 준 경우, 초과한 피해량을 고정 피해로 적 전체에 나눠서 가함. (최소 1)</v>
       </c>
-      <c r="H31" t="str">
+      <c r="I31" t="str">
         <v>./images/ego/88.webp</v>
       </c>
     </row>
@@ -29192,7 +29285,10 @@
       <c r="F32" t="str">
         <v>색욕 x2, 오만 x1, 질투 x4</v>
       </c>
-      <c r="G32" t="str" xml:space="preserve">
+      <c r="G32" t="str">
+        <v>출혈 (부여)</v>
+      </c>
+      <c r="H32" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 종료시] 자신과 현재 체력 비율이 가장 낮은 아군 2명의 체력을 자신의 최대 체력의 15%만큼 회복
 - 회복받는 대상이 보유한 부정적인 효과 종류 1개당 최대 체력의 2.5%만큼 회복량이 증가 (최대 10%)
 - 이 스킬을 포함하여 질투 공명이 4 이상이면, 회복 대상 수 +1
@@ -29200,7 +29296,7 @@
 코인 2: [적중시] 저주 3 부여
 코인 2: [앞면 적중시] 못 3 부여</v>
       </c>
-      <c r="H32" t="str">
+      <c r="I32" t="str">
         <v>./images/ego/87.webp</v>
       </c>
     </row>
@@ -29223,7 +29319,10 @@
       <c r="F33" t="str">
         <v>색욕 x2, 오만 x2, 질투 x2</v>
       </c>
-      <c r="G33" t="str" xml:space="preserve">
+      <c r="G33" t="str">
+        <v>출혈 (부여)</v>
+      </c>
+      <c r="H33" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 이 스킬을 포함하여 공명 수 3 당 공격 가중치 +1 (최대 2)
 [공격 종료시] 대상에게 저주가 있다면 즉시 해당 효과를 2번 발동시키고 저주 2 감소
 코인 1: [앞면 적중시] 출혈 2 부여
@@ -29233,7 +29332,7 @@
 코인 2: [적중시] 대상의 저주가 4 이상이면, 합 위력 감소 1 부여 (턴 당 1회)
 코인 2: [앞면 적중시] 다음 턴에 속박 2 부여 (턴 당 1회)</v>
       </c>
-      <c r="H33" t="str">
+      <c r="I33" t="str">
         <v>./images/ego/86.webp</v>
       </c>
     </row>
@@ -29256,7 +29355,10 @@
       <c r="F34" t="str">
         <v>색욕 x1, 탐식 x4, 오만 x1</v>
       </c>
-      <c r="G34" t="str" xml:space="preserve">
+      <c r="G34" t="str">
+        <v>파열 (부여)</v>
+      </c>
+      <c r="H34" t="str" xml:space="preserve">
         <v xml:space="preserve">대상과 자신의 속도의 합이 6 이상이면, 코인 위력 +1
 대상의 파열 7 당 코인 위력 +1 (최대 2)
 [공격 시작 전] 다음 턴에 신속 2 얻음
@@ -29266,7 +29368,7 @@
 코인 4: [적중시] 자신의 속도만큼 출혈을 무작위로 공격 대상에게 나누어 부여 (최대 7)
 코인 4: [적중시] 자신의 속도만큼 파열을 무작위로 공격 대상에게 나누어 부여 (최대 7)</v>
       </c>
-      <c r="H34" t="str">
+      <c r="I34" t="str">
         <v>./images/ego/85.webp</v>
       </c>
     </row>
@@ -29289,7 +29391,10 @@
       <c r="F35" t="str">
         <v>색욕 x1, 탐식 x3, 질투 x2</v>
       </c>
-      <c r="G35" t="str" xml:space="preserve">
+      <c r="G35" t="str">
+        <v>파열 (부여)</v>
+      </c>
+      <c r="H35" t="str" xml:space="preserve">
         <v xml:space="preserve">자신과 대상의 속도의 합이 6 이상이면, 코인 위력 +1
 대상의 파열 7 당 코인 위력 +1 (최대 2)
 [공격 시작 전] 다음 턴에 신속 2 얻음
@@ -29299,7 +29404,7 @@
 코인 2: [적중시] 파열 2 부여
 코인 3: [적중시] 파열 2 부여</v>
       </c>
-      <c r="H35" t="str">
+      <c r="I35" t="str">
         <v>./images/ego/84.webp</v>
       </c>
     </row>
@@ -29322,7 +29427,10 @@
       <c r="F36" t="str">
         <v>색욕 x2, 나태 x1, 우울 x3</v>
       </c>
-      <c r="G36" t="str" xml:space="preserve">
+      <c r="G36" t="str">
+        <v>침잠 (부여)</v>
+      </c>
+      <c r="H36" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 최대 공명이 4 이상이면, 공격 가중치 +1
 - 해당 공명이 우울 공명이면, 공격 가중치 +1
 [공격 종료시] 현재 체력 비율이 가장 낮은 아군 2명이 최대 체력의 (10 + (메인 공격 대상의 침잠과 침잠 횟수의 합) / 3)%만큼 체력 회복 (최대 20% 회복)
@@ -29332,7 +29440,7 @@
 코인 1: [적중시] 우울 공명 4 이상이면, 우울 취약 1 부여
 코인 1: [적중시] 초청받지 않은 자 2 부여</v>
       </c>
-      <c r="H36" t="str">
+      <c r="I36" t="str">
         <v>./images/ego/83.webp</v>
       </c>
     </row>
@@ -29355,7 +29463,10 @@
       <c r="F37" t="str">
         <v>색욕 x1, 나태 x2, 우울 x2, 질투 x2</v>
       </c>
-      <c r="G37" t="str" xml:space="preserve">
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str" xml:space="preserve">
         <v xml:space="preserve">이 스킬의 코인을 굴릴 때, 공격 대상 중에 하나를 무작위로 선택해 공격
 - 첫 코인은 반드시 메인 공격 대상에게 적중함
 - 모든 적중시 효과, 해당 코인의 피해는 위 효과에서 선택된 공격 대상에게만 적용됨
@@ -29368,7 +29479,7 @@
 코인 3: [적중시] 정신력 2 ~ 6 감소
 코인 3: [적중시] 자신의 정신력이 0 이상이면, 이 코인 재사용 (스킬 당 최대 5회)</v>
       </c>
-      <c r="H37" t="str">
+      <c r="I37" t="str">
         <v>./images/ego/82.webp</v>
       </c>
     </row>
@@ -29391,7 +29502,10 @@
       <c r="F38" t="str">
         <v>분노 x1, 우울 x3, 오만 x1, 질투 x4</v>
       </c>
-      <c r="G38" t="str" xml:space="preserve">
+      <c r="G38" t="str">
+        <v>충전 (강화)</v>
+      </c>
+      <c r="H38" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] (최대 공명 수 - 2)만큼 공격 가중치 증가 (최대 2)
 [공격 시작 전] 보유한 충전 횟수가 10 미만일 때, 최대 체력의 10%만큼 체력을 소모하여 충전 횟수를 10 얻음 (이 피해로 체력이 0이 되지 않음, 소수점 버림)
 [공격 시작 전] 충전 횟수를 최대 40 소모하여 소모한 충전 횟수당 피해량 +1% (최대 30%)
@@ -29399,7 +29513,7 @@
 코인 1: [적중시] 충전만큼 다음 턴에 신속 1, 부하 1 얻음 (한 스킬당 최대 3)
 코인 1: [적 처치시] 충전 횟수 2 증가</v>
       </c>
-      <c r="H38" t="str">
+      <c r="I38" t="str">
         <v>./images/ego/81.webp</v>
       </c>
     </row>
@@ -29422,7 +29536,10 @@
       <c r="F39" t="str">
         <v>분노 x1, 오만 x3, 질투 x2</v>
       </c>
-      <c r="G39" t="str" xml:space="preserve">
+      <c r="G39" t="str">
+        <v>출혈 (부여), 침잠 (부여), 호흡 (강화)</v>
+      </c>
+      <c r="H39" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] (최대 공명 수 + 1)만큼 찢어진 추억을 얻음 (최대 7)
 - 해당 공명이 완전 공명이면 찢어진 추억을 (최대 공명 수 + 2)만큼 얻음
 [공격 시작 전] 찢어진 추억 당 호흡 1 얻음 (최대 7)
@@ -29433,7 +29550,7 @@
 코인 2: [크리티컬 적중 시] 침잠 3 부여
 코인 2: [크리티컬 처치 시] 자신에게 탄환 효과가 있다면, 탄환 1 얻음 (전투 당 3회)</v>
       </c>
-      <c r="H39" t="str">
+      <c r="I39" t="str">
         <v>./images/ego/80.webp</v>
       </c>
     </row>
@@ -29456,14 +29573,17 @@
       <c r="F40" t="str">
         <v>분노 x3, 색욕 x4, 오만 x4, 질투 x3</v>
       </c>
-      <c r="G40" t="str" xml:space="preserve">
+      <c r="G40" t="str">
+        <v>출혈 (부여)</v>
+      </c>
+      <c r="H40" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 최대 공명 수만큼 공격 가중치 증가 (최대 6)
 [공격 시작 전] 이번 턴과 다음 턴에 (최대 공명 수 + 1)만큼 경멸의 시선 얻음 (최대 7)
 [공격 종료시] 이 스킬을 포함하여 색욕 공명을 했다면, 자신이 보유한 기본 공격 스킬과 동일한 속성의 E.G.O 자원 +1
 [공격 종료시] 2턴 동안 턴 종료 시 자신의 정신력 10 감소
 코인 1: [공격 종료시] 출혈 15를 공격 대상에게 균등하게 나눠서 부여</v>
       </c>
-      <c r="H40" t="str">
+      <c r="I40" t="str">
         <v>./images/ego/79.webp</v>
       </c>
     </row>
@@ -29486,7 +29606,10 @@
       <c r="F41" t="str">
         <v>분노 x1, 색욕 x1, 나태 x4, 오만 x4</v>
       </c>
-      <c r="G41" t="str" xml:space="preserve">
+      <c r="G41" t="str">
+        <v>진동 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H41" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] (오만 또는 나태 공명 중 가장 높은 공명 수 - 2)만큼 공격 가중치 증가 (최대 2)
 진동 폭발 시 흐트러짐 손상 100% 증가
 [공격 종료시] 3턴 동안 턴 종료 시 정신력 8 감소
@@ -29494,7 +29617,7 @@
 코인 1: [적중시] 진동 - 균열로 진폭 변환
 코인 1: [적중시] 진동 폭발</v>
       </c>
-      <c r="H41" t="str">
+      <c r="I41" t="str">
         <v>./images/ego/78.webp</v>
       </c>
     </row>
@@ -29517,7 +29640,10 @@
       <c r="F42" t="str">
         <v>색욕 x2, 우울 x4, 오만 x2, 질투 x3</v>
       </c>
-      <c r="G42" t="str" xml:space="preserve">
+      <c r="G42" t="str">
+        <v>침잠 (부여), 진동 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H42" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 종료시] 3턴 동안 턴 종료 시 정신력 10 감소
 [공격 종료시] 다음 턴에 속박 20, 묶인 왕의 앞으로 1, 공격 위력 증가 2 얻음
 코인 1: [적중시] 다음 턴에 속박 1 부여
@@ -29525,7 +29651,7 @@
 코인 1: [적중시] 진동 4 부여
 코인 1: [적중시] 진동 폭발</v>
       </c>
-      <c r="H42" t="str">
+      <c r="I42" t="str">
         <v>./images/ego/77.webp</v>
       </c>
     </row>
@@ -29548,7 +29674,10 @@
       <c r="F43" t="str">
         <v>분노 x1, 질투 x4</v>
       </c>
-      <c r="G43" t="str" xml:space="preserve">
+      <c r="G43" t="str">
+        <v>파열 (부여), 충전 (강화)</v>
+      </c>
+      <c r="H43" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 자신의 충전 횟수 12 증가
 [공격 종료시] 자신을 제외하고 충전 횟수가 가장 낮은 아군 1명의 충전 횟수 8 증가
 - (최대 질투 공명 수 - 2)만큼 부여 대상 수 증가 (최대 5)
@@ -29556,7 +29685,7 @@
 - 최대 질투 공명 수가 6 이상이면, 자신과 부여 대상에게 질투 피해량 증가 1 부여
 코인 1: [적중시] 파열 3 부여</v>
       </c>
-      <c r="H43" t="str">
+      <c r="I43" t="str">
         <v>./images/ego/76.webp</v>
       </c>
     </row>
@@ -29579,13 +29708,16 @@
       <c r="F44" t="str">
         <v>오만 x2, 질투 x4</v>
       </c>
-      <c r="G44" t="str" xml:space="preserve">
+      <c r="G44" t="str">
+        <v>충전 (강화)</v>
+      </c>
+      <c r="H44" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] (질투 공명 수 - 2)만큼 공격 가중치 증가 (최대 3)
 [공격 시작 전] (질투 공명 수 - 3) × 10%만큼 피해량이 증가 (최대 30%)
 [공격 시작 전] 자신의 충전 횟수가 20 이상이면, 충전 횟수를 20 소모하여 피해량 +40%
 코인 1: [적 처치 시] 자신의 충전 횟수 2 증가</v>
       </c>
-      <c r="H44" t="str">
+      <c r="I44" t="str">
         <v>./images/ego/75.webp</v>
       </c>
     </row>
@@ -29608,12 +29740,15 @@
       <c r="F45" t="str">
         <v>색욕 x2, 우울 x4</v>
       </c>
-      <c r="G45" t="str" xml:space="preserve">
+      <c r="G45" t="str">
+        <v>침잠 (부여)</v>
+      </c>
+      <c r="H45" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 종료시] 자신과 자신을 제외한 정신력이 가장 낮은 아군 2명의 정신력 15 회복
 - 대상이 사망하지 않았다면, 대상의 침잠 횟수를 3 소모하고, 대상의 침잠 위력만큼 회복 대상의 정신력 추가 회복 (최대 회복량 : 20)
 - 대상이 사망했다면, 무작위 적 3명에게 침잠 3, 저주 1 부여 (집중 전투인 경우, 무작위 부위에 부여)</v>
       </c>
-      <c r="H45" t="str">
+      <c r="I45" t="str">
         <v>./images/ego/74.webp</v>
       </c>
     </row>
@@ -29636,11 +29771,14 @@
       <c r="F46" t="str">
         <v>나태 x3, 우울 x3</v>
       </c>
-      <c r="G46" t="str" xml:space="preserve">
+      <c r="G46" t="str">
+        <v/>
+      </c>
+      <c r="H46" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 종료시] 침잠 6 + (우울 공명 수 × 1.5)을 무작위로 공격 대상에게 나눠서 부여
 코인 1: [적중시] 대상에게 침잠이 6 이상이면 다음 턴에 속박 2 부여</v>
       </c>
-      <c r="H46" t="str">
+      <c r="I46" t="str">
         <v>./images/ego/73.webp</v>
       </c>
     </row>
@@ -29663,7 +29801,10 @@
       <c r="F47" t="str">
         <v>색욕 x2, 나태 x4, 우울 x2, 오만 x3</v>
       </c>
-      <c r="G47" t="str" xml:space="preserve">
+      <c r="G47" t="str">
+        <v>진동 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H47" t="str" xml:space="preserve">
         <v xml:space="preserve">대상의 속도가 자신보다 느릴 때, 피해량 +(대상과의 속도 차이 × 5)% (최대 50%)
 [공격 시작 전] 최대 공명 수가 3 이상일 경우, (최대 공명 수 × 2)만큼 진동 위력 부여 (최대 10)
 - 최대 공명이 나태 완전 공명일 경우, 부여한 진동 위력 값만큼 진동 횟수 부여 (최대 10)
@@ -29676,7 +29817,7 @@
 코인 4: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소
 코인 4: [적중시] 다음 턴에 대상의 속도 최댓값 절반으로 감소</v>
       </c>
-      <c r="H47" t="str">
+      <c r="I47" t="str">
         <v>./images/ego/66.webp</v>
       </c>
     </row>
@@ -29699,13 +29840,16 @@
       <c r="F48" t="str">
         <v>색욕 x1, 나태 x2, 우울 x3</v>
       </c>
-      <c r="G48" t="str" xml:space="preserve">
+      <c r="G48" t="str">
+        <v/>
+      </c>
+      <c r="H48" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] (최대 공명 수 - 2)만큼 공격 가중치 증가 (최대 2)
 코인 1: [공격 종료시] 자신과 현재 체력이 가장 적은 아군 1 + (최대 공명 수 - 2)명에게 자신의 최대 체력 20%만큼 보호막을 부여하고 울음 방울 2 부여 (자신 제외 최대 부여 대상 수 : 3)
 코인 1: - 대상에게 이미 울음 방울이 있으면, 울음 방울 수치를 2로 변경
 코인 1: - 최대 우울 완전 공명 수가 4 이상이면, 이 스킬의 울음 방울 수치가 3로 부여, 적용됨</v>
       </c>
-      <c r="H48" t="str">
+      <c r="I48" t="str">
         <v>./images/ego/65.webp</v>
       </c>
     </row>
@@ -29728,7 +29872,10 @@
       <c r="F49" t="str">
         <v>분노 x1, 색욕 x3, 오만 x3, 질투 x3</v>
       </c>
-      <c r="G49" t="str" xml:space="preserve">
+      <c r="G49" t="str">
+        <v/>
+      </c>
+      <c r="H49" t="str" xml:space="preserve">
         <v xml:space="preserve">대상의 출혈 2당 코인 위력 +1 (최대 13)
 [전투 시작시] 이 스킬의 메인 타겟은 이번 턴 동안 출혈 횟수가 감소하지 않음.
 [공격 종료시] 3턴 동안 턴 종료 시 정신력 10 감소.
@@ -29739,7 +29886,7 @@
 코인 1: [적 처치 시] 이 스킬의 피해 또는 코인 효과로 적의 남은 체력을 초과하여 피해를 준 경우, 초과한 피해량을 고정 피해로 적 전체에 나눠서 가함.
 코인 1: (집중 전투인 경우, 본체의 체력을 기준으로 계산)</v>
       </c>
-      <c r="H49" t="str">
+      <c r="I49" t="str">
         <v>./images/ego/64.webp</v>
       </c>
     </row>
@@ -29762,14 +29909,17 @@
       <c r="F50" t="str">
         <v>나태 x3, 우울 x3, 오만 x2</v>
       </c>
-      <c r="G50" t="str" xml:space="preserve">
+      <c r="G50" t="str">
+        <v>진동 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H50" t="str" xml:space="preserve">
         <v xml:space="preserve">대상에게 진동이 있으면, 피해량 +(5 + 대상의 진동 위력과 진동 횟수의 합 / 2)% (최대 30%)
 - 최대 공명 수가 4 이상이면, 대신 피해량 +(7.5 + 대상의 진동 위력과 진동 횟수의 합 / 1.5)% (최대 40%)
 코인 1: [적중시] 진동 3, 진동 횟수 3 부여
 코인 1: [적중시] 진동 - 반향으로 진폭 변환
 코인 1: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소</v>
       </c>
-      <c r="H50" t="str">
+      <c r="I50" t="str">
         <v>./images/ego/63.webp</v>
       </c>
     </row>
@@ -29792,7 +29942,10 @@
       <c r="F51" t="str">
         <v>색욕 x1, 탐식 x3, 오만 x2</v>
       </c>
-      <c r="G51" t="str" xml:space="preserve">
+      <c r="G51" t="str">
+        <v/>
+      </c>
+      <c r="H51" t="str" xml:space="preserve">
         <v xml:space="preserve">이 스킬의 효과로 자신의 체력을 초과하여 회복한 경우, 초과한 회복량만큼 체력 비율이 가장 낮은 아군 1명의 체력을 대신 회복
 코인 1: [적중시] 자신의 체력을 최대 체력의 20% 만큼 회복
 코인 2: [앞면 적중시] 정신력 1 ~ 2 감소
@@ -29801,7 +29954,7 @@
 코인 2: [적중시] 탐식 취약 1 부여
 코인 2: [적중시] 출혈 1 ~ 4 부여</v>
       </c>
-      <c r="H51" t="str">
+      <c r="I51" t="str">
         <v>./images/ego/62.webp</v>
       </c>
     </row>
@@ -29824,7 +29977,10 @@
       <c r="F52" t="str">
         <v>분노 x2, 색욕 x2, 나태 x2, 탐식 x2, 우울 x2, 오만 x2, 질투 x2</v>
       </c>
-      <c r="G52" t="str" xml:space="preserve">
+      <c r="G52" t="str">
+        <v/>
+      </c>
+      <c r="H52" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] (가장 높은 공명 수 - 2)만큼 공격 가중치 증가 (최대 3)
 [사용시] 아군 4 + (가장 높은 공명 수)명에게 해당 공명 속성의 피해량 증가와 위력 증가를 1 부여
 - 해당 공명이 4 이상이면, 해당 속성 피해량 증가를 1 추가 부여
@@ -29833,7 +29989,7 @@
 코인 1: [공격 종료 시] 체력 비율이 가장 낮은 아군 4명의 체력을 최대 체력의 22%만큼 회복
 코인 1: - (가장 높은 공명 수 - 2)만큼 회복 대상 증가 (최대 3)</v>
       </c>
-      <c r="H52" t="str">
+      <c r="I52" t="str">
         <v>./images/ego/61.webp</v>
       </c>
     </row>
@@ -29856,12 +30012,15 @@
       <c r="F53" t="str">
         <v>분노 x2, 나태 x2, 오만 x1</v>
       </c>
-      <c r="G53" t="str" xml:space="preserve">
+      <c r="G53" t="str">
+        <v>출혈 (부여), 진동 (부여)</v>
+      </c>
+      <c r="H53" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 출혈 횟수 4 증가
 코인 1: [적중시] 진동 5 부여
 코인 1: [앞면 적중시] 마비 2 부여</v>
       </c>
-      <c r="H53" t="str">
+      <c r="I53" t="str">
         <v>./images/ego/60.webp</v>
       </c>
     </row>
@@ -29884,11 +30043,14 @@
       <c r="F54" t="str">
         <v>나태 x4, 탐식 x2, 우울 x2, 오만 x2</v>
       </c>
-      <c r="G54" t="str" xml:space="preserve">
+      <c r="G54" t="str">
+        <v/>
+      </c>
+      <c r="H54" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 이번 턴, 다음 턴 동안 모든 아군에게 나태 위력 증가 1, 나태 피해량 증가 2, 보호 3 부여
 코인 1: [앞면 적중시] 자신의 정신력 15 회복</v>
       </c>
-      <c r="H54" t="str">
+      <c r="I54" t="str">
         <v>./images/ego/59.webp</v>
       </c>
     </row>
@@ -29911,13 +30073,16 @@
       <c r="F55" t="str">
         <v>나태 x3, 탐식 x3</v>
       </c>
-      <c r="G55" t="str" xml:space="preserve">
+      <c r="G55" t="str">
+        <v/>
+      </c>
+      <c r="H55" t="str" xml:space="preserve">
         <v xml:space="preserve">가장 뒤에 있는 적 공격 (일반 전투 한정)
 [공격 시작 전] 충전 횟수를 소모하고 소모한 만큼 피해량이 증가함 (최대 75%)
 코인 1: [적중시] 충전 횟수를 소모한 경우, 차원 균열 5 부여.
 코인 1: [적중시] 피해량의 (대상의 파열x10)%만큼 오만 추가 피해를 주고, 파열 횟수 5 소모 (최대 100%)</v>
       </c>
-      <c r="H55" t="str">
+      <c r="I55" t="str">
         <v>./images/ego/58.webp</v>
       </c>
     </row>
@@ -29940,14 +30105,17 @@
       <c r="F56" t="str">
         <v>분노 x5, 나태 x1, 탐식 x1</v>
       </c>
-      <c r="G56" t="str" xml:space="preserve">
+      <c r="G56" t="str">
+        <v>화상 (부여)</v>
+      </c>
+      <c r="H56" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 모든 공격 대상의 화상의 합
 - 6당, 최종 위력 +1 (최대 4)
 - 1당, 피해량 +1% (최대 30%)
 코인 1: [적중시] 화상 4 부여
 코인 1: [앞면 적중시] 화상 6 부여</v>
       </c>
-      <c r="H56" t="str">
+      <c r="I56" t="str">
         <v>./images/ego/57.webp</v>
       </c>
     </row>
@@ -29970,12 +30138,15 @@
       <c r="F57" t="str">
         <v>나태 x4, 우울 x1</v>
       </c>
-      <c r="G57" t="str" xml:space="preserve">
+      <c r="G57" t="str">
+        <v/>
+      </c>
+      <c r="H57" t="str" xml:space="preserve">
         <v xml:space="preserve">가장 뒤에 있는 대상 공격 (일반 전투 한정)
 코인 1: [적중시] 나태 취약 2 부여
 코인 1: [앞면 적중시] 마비 3 부여</v>
       </c>
-      <c r="H57" t="str">
+      <c r="I57" t="str">
         <v>./images/ego/56.webp</v>
       </c>
     </row>
@@ -29998,12 +30169,15 @@
       <c r="F58" t="str">
         <v>분노 x1, 나태 x3</v>
       </c>
-      <c r="G58" t="str" xml:space="preserve">
+      <c r="G58" t="str">
+        <v/>
+      </c>
+      <c r="H58" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 공격 위력 감소 2 부여
 코인 1: [적중시] 모든 아군에게 다음 턴에 신속 3 부여
 코인 1: [적중시] 다음 턴에 속박 2 부여</v>
       </c>
-      <c r="H58" t="str">
+      <c r="I58" t="str">
         <v>./images/ego/55.webp</v>
       </c>
     </row>
@@ -30026,14 +30200,17 @@
       <c r="F59" t="str">
         <v>분노 x2, 색욕 x5, 질투 x1</v>
       </c>
-      <c r="G59" t="str" xml:space="preserve">
+      <c r="G59" t="str">
+        <v>화상 (부여)</v>
+      </c>
+      <c r="H59" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] (색욕 공명 수)가 4 이상이면, 공격 가중치 +1
 [공격 시작 전] (최대 색욕 완전 공명 수)가 4 이상이면, 추가로 공격 가중치 +1
 코인 1: [적중시] 대상에게 화상이 없으면 화상 4 부여
 코인 1: [적중시] 화상 4 부여
 코인 1: [뒷면 적중시] 대상의 화상이 10 이상이면 다음 턴에 공격 위력 감소 1, 수비 위력 감소 1 부여</v>
       </c>
-      <c r="H59" t="str">
+      <c r="I59" t="str">
         <v>./images/ego/54.webp</v>
       </c>
     </row>
@@ -30056,12 +30233,15 @@
       <c r="F60" t="str">
         <v>색욕 x1, 탐식 x4, 오만 x2</v>
       </c>
-      <c r="G60" t="str" xml:space="preserve">
+      <c r="G60" t="str">
+        <v>파열 (부여)</v>
+      </c>
+      <c r="H60" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 자신의 체력이 50% 미만이면, 공격 가중치 +2
 코인 1: [적중시] 파열 3 부여
 코인 1: [적중시] 현재 체력 비율이 가장 낮은 아군 2명의 체력을 최대 체력의 15%만큼 회복</v>
       </c>
-      <c r="H60" t="str">
+      <c r="I60" t="str">
         <v>./images/ego/53.webp</v>
       </c>
     </row>
@@ -30084,7 +30264,10 @@
       <c r="F61" t="str">
         <v>분노 x3, 색욕 x2, 탐식 x1</v>
       </c>
-      <c r="G61" t="str" xml:space="preserve">
+      <c r="G61" t="str">
+        <v>화상 (부여)</v>
+      </c>
+      <c r="H61" t="str" xml:space="preserve">
         <v xml:space="preserve">[피아식별불가]
 현재 체력이 가장 낮은 대상 공격
 스킬 사용 시 필요한 탐식 E.G.O 자원이 0으로 변경됨
@@ -30099,7 +30282,7 @@
 코인 1: - 다음 턴에 E.G.O 자원 획득량 + 1, 신속 2 부여
 코인 1: [뒷면 적중시] 화상 7 부여</v>
       </c>
-      <c r="H61" t="str">
+      <c r="I61" t="str">
         <v>./images/ego/52.webp</v>
       </c>
     </row>
@@ -30122,12 +30305,15 @@
       <c r="F62" t="str">
         <v>분노 x3, 색욕 x2</v>
       </c>
-      <c r="G62" t="str" xml:space="preserve">
+      <c r="G62" t="str">
+        <v/>
+      </c>
+      <c r="H62" t="str" xml:space="preserve">
         <v xml:space="preserve">대상의 체력이 25%미만일 때 피해량 +40%
 코인 1: [적 처치 시] 다음 턴에 공격 위력 증가 1 얻음
 코인 1: [적 처치 시] 아군 전체가 각자 최대 체력의 15%만큼 체력 회복</v>
       </c>
-      <c r="H62" t="str">
+      <c r="I62" t="str">
         <v>./images/ego/51.webp</v>
       </c>
     </row>
@@ -30150,12 +30336,15 @@
       <c r="F63" t="str">
         <v>분노 x1, 탐식 x3</v>
       </c>
-      <c r="G63" t="str" xml:space="preserve">
+      <c r="G63" t="str">
+        <v>파열 (부여)</v>
+      </c>
+      <c r="H63" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [앞면 적중시] 파열 12 부여
 코인 1: [앞면 적중시] 정신력 10 감소. 다음 턴에 공격 위력 증가 1을 얻음
 코인 1: [뒷면 적중시] 정신력 10 회복. 다음 턴에 보호 1을 얻음</v>
       </c>
-      <c r="H63" t="str">
+      <c r="I63" t="str">
         <v>./images/ego/50.webp</v>
       </c>
     </row>
@@ -30178,13 +30367,16 @@
       <c r="F64" t="str">
         <v>우울 x2, 오만 x2, 질투 x2</v>
       </c>
-      <c r="G64" t="str" xml:space="preserve">
+      <c r="G64" t="str">
+        <v>호흡 (강화), 충전 (강화)</v>
+      </c>
+      <c r="H64" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 호흡 4 얻음
 [공격 종료시] 이 스킬이 적중한 대상 중 사망한 캐릭터 수만큼 호흡 2를 얻음
 코인 1: [적중시] 충전 횟수 2 증가
 코인 1: [크리티컬 적중 시] 자신의 충전 횟수 2 증가</v>
       </c>
-      <c r="H64" t="str">
+      <c r="I64" t="str">
         <v>./images/ego/49.webp</v>
       </c>
     </row>
@@ -30207,7 +30399,10 @@
       <c r="F65" t="str">
         <v>탐식 x2, 오만 x2, 질투 x2</v>
       </c>
-      <c r="G65" t="str" xml:space="preserve">
+      <c r="G65" t="str">
+        <v>침잠 (부여)</v>
+      </c>
+      <c r="H65" t="str" xml:space="preserve">
         <v xml:space="preserve">대상의 현재 체력이 최대 체력의 25% 미만이면, 피해량 +40%
 [공격 시작 전] 최대 공명수가 4 이상이면, 공격 가중치 +1
 [공격 종료시] 다음 턴에 자신을 포함한 무작위 아군 2+ (최대 공명 수)명에게 E.G.O 자원 획득량 + 1 부여 (최대 7명)
@@ -30216,7 +30411,7 @@
 코인 1: [적중시] 침잠 6 부여
 코인 1: [적 처치 시] 현재 보유 중인 E.G.O 자원 중 무작위 속성 1개의 E.G.O 자원을 3개 얻음. 모든 아군의 정신력 3 회복</v>
       </c>
-      <c r="H65" t="str">
+      <c r="I65" t="str">
         <v>./images/ego/48.webp</v>
       </c>
     </row>
@@ -30239,12 +30434,15 @@
       <c r="F66" t="str">
         <v>분노 x2, 색욕 x2, 질투 x3</v>
       </c>
-      <c r="G66" t="str" xml:space="preserve">
+      <c r="G66" t="str">
+        <v/>
+      </c>
+      <c r="H66" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 다음 턴에 속박 3 부여
 코인 1: [적중시] 대상에게 속박이 3 이상 있을 때 다음 턴에 더하기 코인 약화 1 부여
 코인 1: [적중시] 대상의 속도가 자신보다 느릴 때 다음 턴에 참격 취약 2 부여</v>
       </c>
-      <c r="H66" t="str">
+      <c r="I66" t="str">
         <v>./images/ego/47.webp</v>
       </c>
     </row>
@@ -30267,12 +30465,15 @@
       <c r="F67" t="str">
         <v>색욕 x2, 탐식 x2, 질투 x1</v>
       </c>
-      <c r="G67" t="str" xml:space="preserve">
+      <c r="G67" t="str">
+        <v/>
+      </c>
+      <c r="H67" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 다음 턴에 속박 3 부여
 코인 1: [적중시] 대상에게 속박이 3 이상 있을 때 다음 턴에 더하기 코인 약화 1 부여
 코인 1: [적중시] 대상의 속도가 자신보다 느릴 때 다음 턴에 참격 취약 2 부여</v>
       </c>
-      <c r="H67" t="str">
+      <c r="I67" t="str">
         <v>./images/ego/46.webp</v>
       </c>
     </row>
@@ -30295,14 +30496,17 @@
       <c r="F68" t="str">
         <v>분노 x4, 오만 x2</v>
       </c>
-      <c r="G68" t="str" xml:space="preserve">
+      <c r="G68" t="str">
+        <v>화상 (부여)</v>
+      </c>
+      <c r="H68" t="str" xml:space="preserve">
         <v xml:space="preserve">대상에게 화상이 있으면 스킬 위력 +2
 [공격 시작 전] 모든 공격 대상의 화상 위력의 합 1당 5%만큼 피해량 증가 (최대 100%)
 [적 처치 시] 다음 턴에 공격 위력 증가 2 얻음
 코인 1: [적중시] 이 코인 최종 피해량의 (대상의 화상 위력 × 2)%만큼 분노 피해 (최대 20%)
 코인 1: [적중시] 화상 4 부여</v>
       </c>
-      <c r="H68" t="str">
+      <c r="I68" t="str">
         <v>./images/ego/45.webp</v>
       </c>
     </row>
@@ -30325,12 +30529,15 @@
       <c r="F69" t="str">
         <v>분노 x2, 색욕 x2</v>
       </c>
-      <c r="G69" t="str" xml:space="preserve">
+      <c r="G69" t="str">
+        <v>화상 (부여)</v>
+      </c>
+      <c r="H69" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 화상 6 부여
 코인 1: [적중시] 다음 턴에 취약 1 부여
 코인 1: [앞면 적중시] 다음 턴에 취약 1 부여</v>
       </c>
-      <c r="H69" t="str">
+      <c r="I69" t="str">
         <v>./images/ego/44.webp</v>
       </c>
     </row>
@@ -30353,12 +30560,15 @@
       <c r="F70" t="str">
         <v>나태 x4, 오만 x3</v>
       </c>
-      <c r="G70" t="str" xml:space="preserve">
+      <c r="G70" t="str">
+        <v/>
+      </c>
+      <c r="H70" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 다음 턴에 나태 취약 1 부여
 코인 1: [공격 종료시] 자신을 제외하고 현재 체력 비율이 가장 낮은 아군 2명의 체력을 자신의 최대 체력의 30%만큼 회복
 코인 1: [앞면 공격 종료 시] 대상이 흐트러지거나 사망한 경우, 체력을 회복시킨 캐릭터들에게 자신의 최대 체력의 15%만큼 보호막 부여</v>
       </c>
-      <c r="H70" t="str">
+      <c r="I70" t="str">
         <v>./images/ego/43.webp</v>
       </c>
     </row>
@@ -30381,13 +30591,16 @@
       <c r="F71" t="str">
         <v>나태 x2, 우울 x2, 오만 x2</v>
       </c>
-      <c r="G71" t="str" xml:space="preserve">
+      <c r="G71" t="str">
+        <v>진동 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H71" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 메인 공격 대상의 체력이 최대 체력의 50% 이상이면, 공격 가중치 +1, 최대 체력의 75% 이상이면, 추가로 공격 가중치 +1
 코인 1: [적중시] 진동 3, 진동 횟수 7 부여
 코인 1: [앞면 적중시] 다음 턴에 속박 2 부여
 코인 1: [적중시] 진동 폭발</v>
       </c>
-      <c r="H71" t="str">
+      <c r="I71" t="str">
         <v>./images/ego/42.webp</v>
       </c>
     </row>
@@ -30410,13 +30623,16 @@
       <c r="F72" t="str">
         <v>우울 x5, 질투 x3</v>
       </c>
-      <c r="G72" t="str" xml:space="preserve">
+      <c r="G72" t="str">
+        <v>침잠 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H72" t="str" xml:space="preserve">
         <v xml:space="preserve">대상의 체력이 50%이상이면, 피해량 +30%
 코인 1: [적중시] 진동 폭발
 코인 1: [적중시] 침잠 5 부여
 코인 1: [적중시] 침잠 횟수 5 증가</v>
       </c>
-      <c r="H72" t="str">
+      <c r="I72" t="str">
         <v>./images/ego/41.webp</v>
       </c>
     </row>
@@ -30439,14 +30655,17 @@
       <c r="F73" t="str">
         <v>분노 x3, 오만 x2, 질투 x1</v>
       </c>
-      <c r="G73" t="str" xml:space="preserve">
+      <c r="G73" t="str">
+        <v>화상 (부여)</v>
+      </c>
+      <c r="H73" t="str" xml:space="preserve">
         <v xml:space="preserve">최대 공명 수 1당, 피해량 +5% (최대 30%)
 [공격 종료시] 다음 턴에 분노 위력 증가 1, 분노 피해량 증가 1 얻음
 코인 1: 파괴 불가 코인
 코인 1: [파괴되지 않고 적중시] 화상 6 부여
 코인 1: [적중시] 다음 턴에 분노 취약 3 부여</v>
       </c>
-      <c r="H73" t="str">
+      <c r="I73" t="str">
         <v>./images/ego/40.webp</v>
       </c>
     </row>
@@ -30469,13 +30688,16 @@
       <c r="F74" t="str">
         <v>우울 x1, 오만 x3</v>
       </c>
-      <c r="G74" t="str" xml:space="preserve">
+      <c r="G74" t="str">
+        <v>출혈 (부여)</v>
+      </c>
+      <c r="H74" t="str" xml:space="preserve">
         <v xml:space="preserve">대상의 체력이 50%이상이면, 피해량 +30%
 코인 1: [적중시] 출혈 4 부여
 코인 1: [적중시] 다음 턴에 정신력 회복 효율 +2
 코인 1: [적중시] 다음 턴에 정신력 감소 효율 -2</v>
       </c>
-      <c r="H74" t="str">
+      <c r="I74" t="str">
         <v>./images/ego/39.webp</v>
       </c>
     </row>
@@ -30498,12 +30720,15 @@
       <c r="F75" t="str">
         <v>색욕 x2, 나태 x1, 오만 x3, 질투 x2</v>
       </c>
-      <c r="G75" t="str" xml:space="preserve">
+      <c r="G75" t="str">
+        <v>진동 (소모)</v>
+      </c>
+      <c r="H75" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 진동 폭발
 코인 1: [공격 종료시] 현재 정신력이 가장 낮은 아군 4명에게 가장 높은 공명 속성의 피해량 증가를 1 부여
 코인 1: [공격 종료시] 현재 정신력이 가장 낮은 아군 4명의 정신력 20 회복</v>
       </c>
-      <c r="H75" t="str">
+      <c r="I75" t="str">
         <v>./images/ego/38.webp</v>
       </c>
     </row>
@@ -30526,13 +30751,16 @@
       <c r="F76" t="str">
         <v>나태 x2, 탐식 x2, 우울 x1</v>
       </c>
-      <c r="G76" t="str" xml:space="preserve">
+      <c r="G76" t="str">
+        <v>침잠 (부여), 호흡 (강화), 진동 (소모)</v>
+      </c>
+      <c r="H76" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 호흡 횟수 7 증가
 코인 1: [적중시] 침잠 6 부여
 코인 1: [적중시] 다음 턴에 속박 3 부여
 코인 1: [크리티컬 적중 시] 진동 폭발. 침잠 횟수 3 증가</v>
       </c>
-      <c r="H76" t="str">
+      <c r="I76" t="str">
         <v>./images/ego/37.webp</v>
       </c>
     </row>
@@ -30555,12 +30783,15 @@
       <c r="F77" t="str">
         <v>색욕 x2, 탐식 x3, 우울 x1, 오만 x4</v>
       </c>
-      <c r="G77" t="str" xml:space="preserve">
+      <c r="G77" t="str">
+        <v>파열 (부여), 출혈 (부여)</v>
+      </c>
+      <c r="H77" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 파열 2 부여
 코인 1: [앞면 적중시] 출혈 2 부여
 코인 1: [적중시] 탐식 취약 2 부여</v>
       </c>
-      <c r="H77" t="str">
+      <c r="I77" t="str">
         <v>./images/ego/36.webp</v>
       </c>
     </row>
@@ -30583,12 +30814,15 @@
       <c r="F78" t="str">
         <v>색욕 x2, 나태 x2, 오만 x2</v>
       </c>
-      <c r="G78" t="str" xml:space="preserve">
+      <c r="G78" t="str">
+        <v/>
+      </c>
+      <c r="H78" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 종료시] 정신력 18 회복
 [공격 종료시] 본인 제외 무작위 아군 2명에게 공격 위력 증가 1 부여
 코인 1: [적중시] 색욕 취약 2 부여</v>
       </c>
-      <c r="H78" t="str">
+      <c r="I78" t="str">
         <v>./images/ego/35.webp</v>
       </c>
     </row>
@@ -30611,12 +30845,15 @@
       <c r="F79" t="str">
         <v>나태 x2, 오만 x2</v>
       </c>
-      <c r="G79" t="str" xml:space="preserve">
+      <c r="G79" t="str">
+        <v>파열 (부여)</v>
+      </c>
+      <c r="H79" t="str" xml:space="preserve">
         <v xml:space="preserve">대상의 체력이 50%미만일 때 피해량+30%
 코인 1: [적중시] 파열 4 부여
 코인 1: [적 처치 시] 무작위 아군 1명에게 피해량 증가 1 부여</v>
       </c>
-      <c r="H79" t="str">
+      <c r="I79" t="str">
         <v>./images/ego/34.webp</v>
       </c>
     </row>
@@ -30639,13 +30876,16 @@
       <c r="F80" t="str">
         <v>분노 x3, 오만 x2</v>
       </c>
-      <c r="G80" t="str" xml:space="preserve">
+      <c r="G80" t="str">
+        <v>진동 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H80" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 자신에게 부여된 해제 가능한 부정적인 효과 중 무작위 2개 제거
 코인 1: [적중시] 진동 횟수 3 증가, (분노 완전 공명의 수)/3만큼 추가 증가
 코인 1: [적중시] 진동 폭발
 코인 1: 진동 폭발 시 대상에게 흐트러짐 구간이 없는 경우, 최종 흐트러짐 손상의 (12 + 3×(분노 완전 공명 수))%만큼 분노 피해를 줌</v>
       </c>
-      <c r="H80" t="str">
+      <c r="I80" t="str">
         <v>./images/ego/33.webp</v>
       </c>
     </row>
@@ -30668,14 +30908,17 @@
       <c r="F81" t="str">
         <v>분노 x2, 색욕 x1, 나태 x2</v>
       </c>
-      <c r="G81" t="str" xml:space="preserve">
+      <c r="G81" t="str">
+        <v>화상 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H81" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 종료시] 다음 턴에 신속 2, 분노 위력 증가 1, 타격 위력 증가 1 얻음
 코인 1: [적중시] 화상 10 부여
 코인 1: [적중시] 대상의 화상 수치만큼 진동 부여
 코인 1: [적중시] 무작위 적 5명에게 화상 3 부여
 코인 1: [적중시] 진동 폭발. 진동 폭발 시 진동 횟수 2 감소, 진동 폭발로 대상이 흐트러진 경우 무작위 적 5명의 화상 횟수 3 증가</v>
       </c>
-      <c r="H81" t="str">
+      <c r="I81" t="str">
         <v>./images/ego/32.webp</v>
       </c>
     </row>
@@ -30698,12 +30941,15 @@
       <c r="F82" t="str">
         <v>나태 x2, 오만 x1, 질투 x2</v>
       </c>
-      <c r="G82" t="str" xml:space="preserve">
+      <c r="G82" t="str">
+        <v/>
+      </c>
+      <c r="H82" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 종료시] 보호 3 얻음
 [공격 종료시] 다음 턴에 시술 1 얻음
 코인 1: [앞면 적중시] 마비 3 부여</v>
       </c>
-      <c r="H82" t="str">
+      <c r="I82" t="str">
         <v>./images/ego/31.webp</v>
       </c>
     </row>
@@ -30726,11 +30972,14 @@
       <c r="F83" t="str">
         <v>나태 x4, 우울 x1, 오만 x2</v>
       </c>
-      <c r="G83" t="str" xml:space="preserve">
+      <c r="G83" t="str">
+        <v>진동 (소모)</v>
+      </c>
+      <c r="H83" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 종료시] 자신을 제외하고 현재 체력이 가장 낮은 아군 2명 최대 체력의 30%만큼 체력을 회복, 다음 턴에 보호 2 부여
 코인 1: [적중시] 진동 폭발</v>
       </c>
-      <c r="H83" t="str">
+      <c r="I83" t="str">
         <v>./images/ego/30.webp</v>
       </c>
     </row>
@@ -30753,14 +31002,17 @@
       <c r="F84" t="str">
         <v>나태 x1, 우울 x1, 질투 x2</v>
       </c>
-      <c r="G84" t="str" xml:space="preserve">
+      <c r="G84" t="str">
+        <v/>
+      </c>
+      <c r="H84" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 다음 턴에 속박 5 부여
 코인 1: [적중시] 다음 턴에 속박 3 얻음
 코인 1: [적중시] 다음 턴에 공격 위력 감소 4 부여
 코인 1: [적중시] 다음 턴에 공격 위력 감소 3 얻음
 코인 1: [적중시] 다음 턴에 보호 2 얻음</v>
       </c>
-      <c r="H84" t="str">
+      <c r="I84" t="str">
         <v>./images/ego/29.webp</v>
       </c>
     </row>
@@ -30783,13 +31035,16 @@
       <c r="F85" t="str">
         <v>분노 x2, 우울 x3, 오만 x3, 질투 x3</v>
       </c>
-      <c r="G85" t="str" xml:space="preserve">
+      <c r="G85" t="str">
+        <v>충전 (강화)</v>
+      </c>
+      <c r="H85" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 종료시] 정신력이 가장 낮은 아군 4명의 정신력 25 회복
 코인 1: [적중시] 자신의 충전 횟수 6 증가
 코인 1: [적중시] 무작위 아군 1명에게 호흡 횟수 2 부여
 코인 1: [공격 종료시] 정신력이 가장 높은 아군 4명에게 관통 위력 증가 2, 피해량 증가 2 부여</v>
       </c>
-      <c r="H85" t="str">
+      <c r="I85" t="str">
         <v>./images/ego/28.webp</v>
       </c>
     </row>
@@ -30812,12 +31067,15 @@
       <c r="F86" t="str">
         <v>분노 x2, 색욕 x2, 나태 x1</v>
       </c>
-      <c r="G86" t="str" xml:space="preserve">
+      <c r="G86" t="str">
+        <v>화상 (부여)</v>
+      </c>
+      <c r="H86" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 종료시] 다음 턴에 모든 아군에게 분노 피해량 증가 1 부여
 코인 1: [적중시] 화상 4 부여
 코인 1: [적중시] 대상에게 정신력 15 피해</v>
       </c>
-      <c r="H86" t="str">
+      <c r="I86" t="str">
         <v>./images/ego/27.webp</v>
       </c>
     </row>
@@ -30840,13 +31098,16 @@
       <c r="F87" t="str">
         <v>분노 x1, 색욕 x4</v>
       </c>
-      <c r="G87" t="str" xml:space="preserve">
+      <c r="G87" t="str">
+        <v/>
+      </c>
+      <c r="H87" t="str" xml:space="preserve">
         <v xml:space="preserve">가장 뒤에 있는 대상 공격 (일반 전투 한정)
 코인 1: [적중시] 공격 레벨 감소 10 부여
 코인 1: [적중시] 마비 3 부여
 코인 1: [적중시] 다음 턴에 속박 3 부여</v>
       </c>
-      <c r="H87" t="str">
+      <c r="I87" t="str">
         <v>./images/ego/26.webp</v>
       </c>
     </row>
@@ -30869,13 +31130,16 @@
       <c r="F88" t="str">
         <v>분노 x4, 색욕 x2, 질투 x1</v>
       </c>
-      <c r="G88" t="str" xml:space="preserve">
+      <c r="G88" t="str">
+        <v>화상 (부여)</v>
+      </c>
+      <c r="H88" t="str" xml:space="preserve">
         <v xml:space="preserve">가장 뒤에 있는 대상 공격 (일반 전투 한정)
 코인 1: [앞면 적중시] 피해량의 40%만큼 흐트러짐 손상 입힘
 코인 1: [적중시] 분노 공명 수만큼 화상 부여
 코인 1: [앞면 공격 종료 시] 무작위 적 3명에게 화상 5 부여</v>
       </c>
-      <c r="H88" t="str">
+      <c r="I88" t="str">
         <v>./images/ego/25.webp</v>
       </c>
     </row>
@@ -30898,13 +31162,16 @@
       <c r="F89" t="str">
         <v>분노 x2, 우울 x2</v>
       </c>
-      <c r="G89" t="str" xml:space="preserve">
+      <c r="G89" t="str">
+        <v>진동 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H89" t="str" xml:space="preserve">
         <v xml:space="preserve">가장 뒤에 있는 대상 공격 (일반 전투 한정)
 코인 1: [적중시] 다음 턴에 속박 6 부여
 코인 1: [적중시] 진동 3 부여
 코인 1: [적중시] 진동 폭발</v>
       </c>
-      <c r="H89" t="str">
+      <c r="I89" t="str">
         <v>./images/ego/24.webp</v>
       </c>
     </row>
@@ -30927,14 +31194,17 @@
       <c r="F90" t="str">
         <v>탐식 x6, 우울 x1</v>
       </c>
-      <c r="G90" t="str" xml:space="preserve">
+      <c r="G90" t="str">
+        <v/>
+      </c>
+      <c r="H90" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 자신의 체력이 최대 체력의 50% 미만이면, 공격 가중치 +1
 최대 체력의 25% 미만이면, 추가로 공격 가중치 +1
 코인 1: [적중시] (탐식 공명 수/2)만큼 파열 부여
 코인 1: [적중시] 다음 턴에 탐식 취약 2 부여
 코인 1: [적중시] 다음 턴에 속박 2 부여</v>
       </c>
-      <c r="H90" t="str">
+      <c r="I90" t="str">
         <v>./images/ego/23.webp</v>
       </c>
     </row>
@@ -30957,12 +31227,15 @@
       <c r="F91" t="str">
         <v>탐식 x3, 우울 x2, 질투 x2</v>
       </c>
-      <c r="G91" t="str" xml:space="preserve">
+      <c r="G91" t="str">
+        <v/>
+      </c>
+      <c r="H91" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [앞면 공격 종료 시] 체력 비율이 가장 낮은 아군 2명의 체력 15 회복
 코인 1: [뒷면 공격 종료 시] 정신력이 가장 낮은 아군 2명의 정신력 15 회복
 코인 1: [크리티컬 공격 종료 시] 체력 비율이 가장 낮은 아군 1명의 체력 8 회복, 정신력이 가장 낮은 아군 1명의 정신력 8 회복</v>
       </c>
-      <c r="H91" t="str">
+      <c r="I91" t="str">
         <v>./images/ego/22.webp</v>
       </c>
     </row>
@@ -30985,12 +31258,15 @@
       <c r="F92" t="str">
         <v>탐식 x3, 오만 x3</v>
       </c>
-      <c r="G92" t="str" xml:space="preserve">
+      <c r="G92" t="str">
+        <v>충전 (강화)</v>
+      </c>
+      <c r="H92" t="str" xml:space="preserve">
         <v xml:space="preserve">가장 뒤에 있는 적 공격 (일반 전투 한정)
 [공격 시작 전] 충전 횟수 5 증가. 다음 턴에 신속 2를 얻음
 코인 1: [적중시] 취약 1, 차원 균열 4 부여</v>
       </c>
-      <c r="H92" t="str">
+      <c r="I92" t="str">
         <v>./images/ego/21.webp</v>
       </c>
     </row>
@@ -31013,11 +31289,14 @@
       <c r="F93" t="str">
         <v>색욕 x4, 질투 x2</v>
       </c>
-      <c r="G93" t="str" xml:space="preserve">
+      <c r="G93" t="str">
+        <v/>
+      </c>
+      <c r="H93" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 수비 위력 감소 2 부여
 코인 1: [적중시] 방어 레벨 감소 5 부여</v>
       </c>
-      <c r="H93" t="str">
+      <c r="I93" t="str">
         <v>./images/ego/20.webp</v>
       </c>
     </row>
@@ -31040,12 +31319,15 @@
       <c r="F94" t="str">
         <v>색욕 x1, 우울 x5</v>
       </c>
-      <c r="G94" t="str" xml:space="preserve">
+      <c r="G94" t="str">
+        <v>침잠 (부여)</v>
+      </c>
+      <c r="H94" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 종료시] 정신력 15 회복
 코인 1: [적중시] 침잠 5 부여
 코인 1: [공격 종료시] 다음 턴에 모든 아군의 정신력 감소 효율 -2, E.G.O 사용시 정신력 감소량 -2</v>
       </c>
-      <c r="H94" t="str">
+      <c r="I94" t="str">
         <v>./images/ego/19.webp</v>
       </c>
     </row>
@@ -31068,11 +31350,14 @@
       <c r="F95" t="str">
         <v>탐식 x3, 질투 x2</v>
       </c>
-      <c r="G95" t="str" xml:space="preserve">
+      <c r="G95" t="str">
+        <v/>
+      </c>
+      <c r="H95" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 다음 턴에 화상, 출혈, 진동, 파열, 침잠 중 무작위 1개 효과의 위력을 (2 + (최대 탐식 완전 공명의 수))회 부여 (최대 7)
 코인 1: [적 처치 시] 무작위 아군 2명에게 다음 턴에 호흡 횟수 2, 충전 횟수 2, 신속 2, 공격 레벨 증가 2, 방어 레벨 증가 2 중 무작위 1개 효과를 부여</v>
       </c>
-      <c r="H95" t="str">
+      <c r="I95" t="str">
         <v>./images/ego/18.webp</v>
       </c>
     </row>
@@ -31095,12 +31380,15 @@
       <c r="F96" t="str">
         <v>분노 x2, 색욕 x2, 나태 x2, 우울 x2</v>
       </c>
-      <c r="G96" t="str" xml:space="preserve">
+      <c r="G96" t="str">
+        <v/>
+      </c>
+      <c r="H96" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 자신의 정신력이 15 이상이면 공격 가중치 +2
 코인 1: [적중시] 다음 턴에 공격 위력 감소 2 부여
 코인 1: [공격 종료 시] 자신을 제외하고 정신력이 가장 낮은 아군 4명의 정신력 25 회복</v>
       </c>
-      <c r="H96" t="str">
+      <c r="I96" t="str">
         <v>./images/ego/17.webp</v>
       </c>
     </row>
@@ -31123,12 +31411,15 @@
       <c r="F97" t="str">
         <v>우울 x3, 질투 x2</v>
       </c>
-      <c r="G97" t="str" xml:space="preserve">
+      <c r="G97" t="str">
+        <v>충전 (강화)</v>
+      </c>
+      <c r="H97" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 자신의 잃은 체력의 10%당 충전 횟수 1 증가 (최대 7)
 다음 턴에 신속 2를 얻음
 코인 1: [적중시] 마비 3, 우울 취약 1 부여</v>
       </c>
-      <c r="H97" t="str">
+      <c r="I97" t="str">
         <v>./images/ego/16.webp</v>
       </c>
     </row>
@@ -31151,12 +31442,15 @@
       <c r="F98" t="str">
         <v>분노 x3, 색욕 x2, 질투 x3</v>
       </c>
-      <c r="G98" t="str" xml:space="preserve">
+      <c r="G98" t="str">
+        <v>충전 (강화)</v>
+      </c>
+      <c r="H98" t="str" xml:space="preserve">
         <v xml:space="preserve">[사용시] 질투 공명 수만큼 자신의 충전 횟수 증가
 충전 횟수 5를 소모할 때마다 스킬 위력 +3 (최대 12)
 코인 1: [뒷면 적중시] 자신의 충전 횟수 5 증가</v>
       </c>
-      <c r="H98" t="str">
+      <c r="I98" t="str">
         <v>./images/ego/15.webp</v>
       </c>
     </row>
@@ -31179,12 +31473,15 @@
       <c r="F99" t="str">
         <v>색욕 x2, 질투 x2</v>
       </c>
-      <c r="G99" t="str" xml:space="preserve">
+      <c r="G99" t="str">
+        <v/>
+      </c>
+      <c r="H99" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 다음 턴에 공격 위력 증가 1 얻음
 코인 1: [적중시] 다음 턴에 신속 3 얻음
 코인 1: [적 처치 시] 다음 턴에 공격 위력 증가 2 얻음</v>
       </c>
-      <c r="H99" t="str">
+      <c r="I99" t="str">
         <v>./images/ego/14.webp</v>
       </c>
     </row>
@@ -31207,11 +31504,14 @@
       <c r="F100" t="str">
         <v>우울 x3, 질투 x3</v>
       </c>
-      <c r="G100" t="str" xml:space="preserve">
+      <c r="G100" t="str">
+        <v>충전 (강화)</v>
+      </c>
+      <c r="H100" t="str" xml:space="preserve">
         <v xml:space="preserve">[공격 시작 전] 자신의 충전 횟수 10 증가
 코인 1: [적중시] 방출 전류 15 부여</v>
       </c>
-      <c r="H100" t="str">
+      <c r="I100" t="str">
         <v>./images/ego/13.webp</v>
       </c>
     </row>
@@ -31234,12 +31534,15 @@
       <c r="F101" t="str">
         <v>나태 x1, 탐식 x3</v>
       </c>
-      <c r="G101" t="str" xml:space="preserve">
+      <c r="G101" t="str">
+        <v>진동 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H101" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 진동 폭발
 코인 1: [적중시] 진동 6 부여
 코인 1: [적중시] 마비 4 부여</v>
       </c>
-      <c r="H101" t="str">
+      <c r="I101" t="str">
         <v>./images/ego/12.webp</v>
       </c>
     </row>
@@ -31263,9 +31566,12 @@
         <v>나태 x1, 탐식 x4</v>
       </c>
       <c r="G102" t="str">
+        <v/>
+      </c>
+      <c r="H102" t="str">
         <v>코인 1: [적중시] 피해량의 60%만큼 자신의 체력 회복</v>
       </c>
-      <c r="H102" t="str">
+      <c r="I102" t="str">
         <v>./images/ego/11.webp</v>
       </c>
     </row>
@@ -31289,9 +31595,12 @@
         <v>색욕 x3, 우울 x1</v>
       </c>
       <c r="G103" t="str">
+        <v/>
+      </c>
+      <c r="H103" t="str">
         <v>코인 1: [적중시] 화상, 출혈, 진동, 파열, 침잠 중 무작위 1개 효과 10 부여</v>
       </c>
-      <c r="H103" t="str">
+      <c r="I103" t="str">
         <v>./images/ego/10.webp</v>
       </c>
     </row>
@@ -31314,7 +31623,10 @@
       <c r="F104" t="str">
         <v>색욕 x1, 탐식 x3, 오만 x1</v>
       </c>
-      <c r="G104" t="str" xml:space="preserve">
+      <c r="G104" t="str">
+        <v>화상 (부여)</v>
+      </c>
+      <c r="H104" t="str" xml:space="preserve">
         <v xml:space="preserve">스킬 사용 시 필요한 탐식 E.G.O 자원 1 감소
 [공격 시작 전] (최대 공명 수)가 4 이상이면 공격 가중치 +1
 (최대 공명 수)가 6 이상이면, 추가로 공격 가중치 +1
@@ -31324,7 +31636,7 @@
 코인 1: [적중시] 대상의 화상 2를 방어 레벨 감소 1로 전환 (최대 5. 이 효과로 대상의 화상 위력이 1 미만이 되지 않음)
 코인 1: - 자신의 30을 초과하는 화상을 대상의 화상이 부족한 만큼 대신 전환 가능</v>
       </c>
-      <c r="H104" t="str">
+      <c r="I104" t="str">
         <v>./images/ego/9.webp</v>
       </c>
     </row>
@@ -31347,12 +31659,15 @@
       <c r="F105" t="str">
         <v>분노 x1, 색욕 x3, 질투 x2</v>
       </c>
-      <c r="G105" t="str" xml:space="preserve">
+      <c r="G105" t="str">
+        <v>충전 (강화)</v>
+      </c>
+      <c r="H105" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 마비 3 부여
 코인 1: [공격 종료시] 자신의 충전 횟수 7 증가
 코인 1: [앞면 공격 종료 시] 다음 턴에 무작위 아군 2명에게 질투 위력 증가 1, 신속 1 부여, 자신의 충전 횟수 3 증가</v>
       </c>
-      <c r="H105" t="str">
+      <c r="I105" t="str">
         <v>./images/ego/8.webp</v>
       </c>
     </row>
@@ -31375,12 +31690,15 @@
       <c r="F106" t="str">
         <v>색욕 x2, 우울 x4, 질투 x3</v>
       </c>
-      <c r="G106" t="str" xml:space="preserve">
+      <c r="G106" t="str">
+        <v/>
+      </c>
+      <c r="H106" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [공격 종료시] 아군 전체 정신력 15 회복
 코인 1: [공격 종료시] 아군 전체 최대 체력의 15%만큼 체력 회복
 코인 1: [앞면 공격 종료 시] 아군 전체 정신력 10 회복</v>
       </c>
-      <c r="H106" t="str">
+      <c r="I106" t="str">
         <v>./images/ego/7.webp</v>
       </c>
     </row>
@@ -31403,14 +31721,17 @@
       <c r="F107" t="str">
         <v>질투 x6</v>
       </c>
-      <c r="G107" t="str" xml:space="preserve">
+      <c r="G107" t="str">
+        <v/>
+      </c>
+      <c r="H107" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 관통 취약 3 부여
 코인 1: [적중시] 질투 취약 1 부여
 코인 1: [앞면 적중시] 저주 3 부여
 코인 1: [앞면 적중시] 못 3 부여
 코인 1: [적중시] 대상에게 저주가 있으면 피해량 +50%</v>
       </c>
-      <c r="H107" t="str">
+      <c r="I107" t="str">
         <v>./images/ego/6.webp</v>
       </c>
     </row>
@@ -31434,9 +31755,12 @@
         <v>탐식 x2, 오만 x4</v>
       </c>
       <c r="G108" t="str">
+        <v/>
+      </c>
+      <c r="H108" t="str">
         <v>코인 1: [공격 종료시] 정신력이 가장 낮은 아군 4명의 정신력 12 회복</v>
       </c>
-      <c r="H108" t="str">
+      <c r="I108" t="str">
         <v>./images/ego/5.webp</v>
       </c>
     </row>
@@ -31459,14 +31783,17 @@
       <c r="F109" t="str">
         <v>색욕 x5</v>
       </c>
-      <c r="G109" t="str" xml:space="preserve">
+      <c r="G109" t="str">
+        <v>화상 (부여)</v>
+      </c>
+      <c r="H109" t="str" xml:space="preserve">
         <v xml:space="preserve">메인 타겟의 화상과 출혈의 합 4당 최종 위력 +1 (최대 3)
 [공격 시작 전] 보유한 색욕 E.G.O 자원 6당 편성 순서 순으로 다음 턴에 색욕 위력 증가 1 부여 (최대 5명)
 [공격 시작 전] 보유한 색욕 E.G.O 자원 1개당 피해량 +6% (최대 120%)
 코인 1: [적중시] 화상 횟수 3 증가
 코인 1: [적중시] 출혈 횟수 3 증가</v>
       </c>
-      <c r="H109" t="str">
+      <c r="I109" t="str">
         <v>./images/ego/4.webp</v>
       </c>
     </row>
@@ -31489,11 +31816,14 @@
       <c r="F110" t="str">
         <v>분노 x1, 우울 x2, 질투 x2</v>
       </c>
-      <c r="G110" t="str" xml:space="preserve">
+      <c r="G110" t="str">
+        <v>충전 (강화)</v>
+      </c>
+      <c r="H110" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 충전 횟수 10을 얻음
 코인 1: [공격 종료시] 질투 공명 수에 비례하여 모든 아군에게 충전 횟수 부여</v>
       </c>
-      <c r="H110" t="str">
+      <c r="I110" t="str">
         <v>./images/ego/3.webp</v>
       </c>
     </row>
@@ -31516,13 +31846,16 @@
       <c r="F111" t="str">
         <v>색욕 x1, 우울 x4, 오만 x2</v>
       </c>
-      <c r="G111" t="str" xml:space="preserve">
+      <c r="G111" t="str">
+        <v>침잠 (부여), 진동 (소모)</v>
+      </c>
+      <c r="H111" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 진동 폭발
 코인 1: [적중시] 대상에게 정신력 25 피해
 코인 1: 대상이 흐트러짐, 사기 저하, 패닉 상태라면 피해량의 30%만큼 추가 피해
 코인 1: [적중시] 침잠 2 부여</v>
       </c>
-      <c r="H111" t="str">
+      <c r="I111" t="str">
         <v>./images/ego/2.webp</v>
       </c>
     </row>
@@ -31545,11 +31878,14 @@
       <c r="F112" t="str">
         <v>색욕 x2, 오만 x2</v>
       </c>
-      <c r="G112" t="str" xml:space="preserve">
+      <c r="G112" t="str">
+        <v>출혈 (부여)</v>
+      </c>
+      <c r="H112" t="str" xml:space="preserve">
         <v xml:space="preserve">코인 1: [적중시] 출혈 8 부여
 코인 1: [적중시] 피해량의 50%만큼 체력 회복</v>
       </c>
-      <c r="H112" t="str">
+      <c r="I112" t="str">
         <v>./images/ego/1.webp</v>
       </c>
     </row>
@@ -31572,7 +31908,10 @@
       <c r="F113" t="str">
         <v>분노 x2, 나태 x2, 우울 x1, 오만 x1</v>
       </c>
-      <c r="G113" t="str" xml:space="preserve">
+      <c r="G113" t="str">
+        <v>진동 (부여), 호흡 (강화), 진동 (소모)</v>
+      </c>
+      <c r="H113" t="str" xml:space="preserve">
         <v xml:space="preserve">자신의 호흡 위력과 메인 타겟의 진동 위력의 합 6당, 합 위력 +1 (최대 4)
 [공격 시작 전] (4 + 최대 공명 수)만큼 호흡 얻음 (최대 8)
 [공격 시작 전] 자신의 호흡 횟수 4 증가
@@ -31582,7 +31921,7 @@
 코인 3: [적중시] 공격 레벨 감소 2 부여
 코인 3: [적중시] 진동 폭발. 대상의 진동 횟수 1 감소</v>
       </c>
-      <c r="H113" t="str">
+      <c r="I113" t="str">
         <v>./images/ego/128.webp</v>
       </c>
     </row>
@@ -31605,14 +31944,17 @@
       <c r="F114" t="str">
         <v>색욕 x2, 오만 x1, 질투 x2</v>
       </c>
-      <c r="G114" t="str" xml:space="preserve">
+      <c r="G114" t="str">
+        <v>충전 (강화)</v>
+      </c>
+      <c r="H114" t="str" xml:space="preserve">
         <v xml:space="preserve">[사용시] 자신의 충전 위력만큼 합 위력 증가 (최대 3)
 [공격 시작 전] 자신의 충전 횟수 5 증가
 [공격 시작 전] 자신의 충전 횟수를 최대 10까지 소모하고, 자신과 자신을 제외한 아군 최대 (1 + 소모한 충전 횟수/2)명에게 충전 역장 5 부여 (최대 7명, 소수점 버림)
 코인 1: [적중시] 자신의 충전 횟수 2 증가
 코인 2: [적중시] 광전 2 부여</v>
       </c>
-      <c r="H114" t="str">
+      <c r="I114" t="str">
         <v>./images/ego/129.webp</v>
       </c>
     </row>
@@ -31635,7 +31977,10 @@
       <c r="F115" t="str">
         <v>우울 x2, 오만 x4, 질투 x2</v>
       </c>
-      <c r="G115" t="str" xml:space="preserve">
+      <c r="G115" t="str">
+        <v>호흡 (강화), 충전 (강화)</v>
+      </c>
+      <c r="H115" t="str" xml:space="preserve">
         <v xml:space="preserve">[합 불가능]
 전투에서 처음 사용 시 정신력 소모량이 5 감소하고, 필요한 E.G.O 자원이 우울 2, 오만 2, 질투 2 감소
 잿빛 탄환이 1 이상이면, '부셰'로 발동됨
@@ -31646,7 +31991,7 @@
 [공격 종료시] 충전 횟수 5 얻음
 [공격 종료시] 검은 날개 4 얻음</v>
       </c>
-      <c r="H115" t="str">
+      <c r="I115" t="str">
         <v>./images/ego/130.webp</v>
       </c>
     </row>
@@ -31669,7 +32014,10 @@
       <c r="F116" t="str">
         <v>나태 x2, 우울 x2, 오만 x4, 질투 x4</v>
       </c>
-      <c r="G116" t="str" xml:space="preserve">
+      <c r="G116" t="str">
+        <v>침잠 (부여), 호흡 (강화)</v>
+      </c>
+      <c r="H116" t="str" xml:space="preserve">
         <v xml:space="preserve">스킬 시전 중 공격 대상 사망 시, 체력이 가장 낮은 공격 대상을 우선 지정 (집중 전투의 경우, 부위로 판정)
 (자신의 호흡 위력 + 충전 횟수) 4당 합 위력 +1 (최대 10)
 자신의 잿빛 탄환 1당 합 위력 +2
@@ -31694,13 +32042,13 @@
 코인 2: [코인 시작 시] 자신의 충전 횟수 4당 코인 위력 +1 (최대 5)
 코인 2: [적중시] 침잠 횟수 3 증가</v>
       </c>
-      <c r="H116" t="str">
+      <c r="I116" t="str">
         <v>./images/ego/131.webp</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H116"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I116"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>